<commit_message>
Consistency check: crested gecko heat settled and marked fixed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CONSISTENCY_CHECK.xlsx
+++ b/CONSISTENCY_CHECK.xlsx
@@ -773,7 +773,7 @@
         <v/>
       </c>
       <c r="G7" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -5210,9 +5210,9 @@
           <t>content/CAREPACKAGE Guides/source/crested-gecko-src</t>
         </is>
       </c>
-      <c r="D43" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D43" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E43" s="13" t="inlineStr">
@@ -5232,12 +5232,12 @@
       </c>
       <c r="H43" s="13" t="inlineStr">
         <is>
-          <t>Book fix: logged in FIX_PACKAGES.md; make the change in the package source at the next edition, after the site side is settled.</t>
+          <t>Fixed 2026-10-05 (owner ruling); nothing left to do.</t>
         </is>
       </c>
       <c r="I43" s="13" t="inlineStr">
         <is>
-          <t>Waiting on owner's heat call. Logged in FIX_PACKAGES.md.</t>
+          <t>Fixed and pushed to main 2026-10-05: the package was right; the site was corrected to match the vet sources.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Consistency sweep: fix all 19 safety rows
Source-checked each conflict, then brought the stray pages in line:
garter snake cohabitation, tegu eggs cooked, gargoyle stuck shed to a
vet, corydoras ich heat capped at 78F with reduced doses, ich heat-alone
rows for 82F fish, cockatiel bar spacing, hamster floor space, flying
squirrel D3, rat heat risk at 80F, jumping spider prey size, hermit crab
humidity, raised bowls out for large breeds, no off-leash hounds.
Workbook rows marked fixed with notes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CONSISTENCY_CHECK.xlsx
+++ b/CONSISTENCY_CHECK.xlsx
@@ -820,7 +820,7 @@
         <v>8</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E9" s="4">
         <f>C9-D9</f>
@@ -831,7 +831,7 @@
         <v/>
       </c>
       <c r="G9" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -1179,7 +1179,7 @@
         <v/>
       </c>
       <c r="G21" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -1342,7 +1342,7 @@
         <v>9</v>
       </c>
       <c r="D27" s="5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E27" s="4">
         <f>C27-D27</f>
@@ -1353,7 +1353,7 @@
         <v/>
       </c>
       <c r="G27" s="5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28">
@@ -1951,7 +1951,7 @@
         <v>9</v>
       </c>
       <c r="D48" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E48" s="4">
         <f>C48-D48</f>
@@ -1962,7 +1962,7 @@
         <v/>
       </c>
       <c r="G48" s="5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="49">
@@ -2154,7 +2154,7 @@
         <v>9</v>
       </c>
       <c r="D55" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E55" s="4">
         <f>C55-D55</f>
@@ -2165,7 +2165,7 @@
         <v/>
       </c>
       <c r="G55" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56">
@@ -2183,7 +2183,7 @@
         <v>10</v>
       </c>
       <c r="D56" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E56" s="4">
         <f>C56-D56</f>
@@ -2194,7 +2194,7 @@
         <v/>
       </c>
       <c r="G56" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="57">
@@ -2212,7 +2212,7 @@
         <v>9</v>
       </c>
       <c r="D57" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E57" s="4">
         <f>C57-D57</f>
@@ -2223,7 +2223,7 @@
         <v/>
       </c>
       <c r="G57" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58">
@@ -2513,7 +2513,7 @@
         <v/>
       </c>
       <c r="G67" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="68">
@@ -2647,7 +2647,7 @@
         <v>8</v>
       </c>
       <c r="D72" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E72" s="4">
         <f>C72-D72</f>
@@ -2658,7 +2658,7 @@
         <v/>
       </c>
       <c r="G72" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="73">
@@ -2763,7 +2763,7 @@
         <v>7</v>
       </c>
       <c r="D76" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E76" s="4">
         <f>C76-D76</f>
@@ -2774,7 +2774,7 @@
         <v/>
       </c>
       <c r="G76" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="77">
@@ -2850,7 +2850,7 @@
         <v>8</v>
       </c>
       <c r="D79" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E79" s="4">
         <f>C79-D79</f>
@@ -2861,7 +2861,7 @@
         <v/>
       </c>
       <c r="G79" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="80">
@@ -2919,7 +2919,7 @@
         <v/>
       </c>
       <c r="G81" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="82">
@@ -3517,7 +3517,7 @@
         <v>1</v>
       </c>
       <c r="D102" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E102" s="4">
         <f>C102-D102</f>
@@ -3528,7 +3528,7 @@
         <v/>
       </c>
       <c r="G102" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="103">
@@ -3546,7 +3546,7 @@
         <v>3</v>
       </c>
       <c r="D103" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E103" s="4">
         <f>C103-D103</f>
@@ -3557,7 +3557,7 @@
         <v/>
       </c>
       <c r="G103" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="104">
@@ -3849,6 +3849,7 @@
         <v/>
       </c>
     </row>
+    <row r="114"/>
     <row r="115">
       <c r="A115" s="9" t="inlineStr">
         <is>
@@ -5684,9 +5685,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D57" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D57" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E57" s="13" t="inlineStr">
@@ -5709,7 +5710,11 @@
           <t>Safety: fix this first. Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I57" s="13" t="inlineStr"/>
+      <c r="I57" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: hub now soaks early shed, vet for a tight band or dark toe.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="23" t="inlineStr">
@@ -9830,9 +9835,9 @@
           <t>content/guides/argentine-tegu-tank-setup-guide.mdx</t>
         </is>
       </c>
-      <c r="D191" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D191" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E191" s="13" t="inlineStr">
@@ -9855,7 +9860,11 @@
           <t>Safety: fix this first. Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I191" s="13" t="inlineStr"/>
+      <c r="I191" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: raw eggs changed to cooked eggs (raw white blocks biotin).</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="30" t="inlineStr">
@@ -11730,9 +11739,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D251" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D251" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E251" s="13" t="inlineStr">
@@ -11755,7 +11764,11 @@
           <t>Safety: fix this first. Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I251" s="13" t="inlineStr"/>
+      <c r="I251" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: ReptiFiles confirms common, checkered, wandering, coast garters are not cohabited; pair line removed from hub.</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" s="19" t="inlineStr">
@@ -11843,9 +11856,9 @@
           <t>content/guides/garter-snake-enrichment-guide.mdx</t>
         </is>
       </c>
-      <c r="D254" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D254" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E254" s="13" t="inlineStr">
@@ -11868,7 +11881,11 @@
           <t>Safety: fix this first. Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I254" s="13" t="inlineStr"/>
+      <c r="I254" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: FAQ now says it depends on species and names the four kept alone (ReptiFiles).</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" s="19" t="inlineStr">
@@ -12010,9 +12027,9 @@
           <t>content/guides/garter-snake-tank-setup-guide.mdx</t>
         </is>
       </c>
-      <c r="D259" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D259" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E259" s="13" t="inlineStr">
@@ -12035,7 +12052,11 @@
           <t>Safety: fix this first. Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I259" s="13" t="inlineStr"/>
+      <c r="I259" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: mated-pair 55-gallon lines replaced with one snake per enclosure (ReptiFiles).</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" s="19" t="inlineStr">
@@ -18759,9 +18780,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D75" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D75" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E75" s="13" t="inlineStr">
@@ -18784,7 +18805,11 @@
           <t>Safety: fix this first. Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I75" s="13" t="inlineStr"/>
+      <c r="I75" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: hub now warms only to 78F with reduced-dose medication.</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="32" t="inlineStr">
@@ -18953,9 +18978,9 @@
           <t>content/guides/corydoras-catfish-health-issues-guide.mdx</t>
         </is>
       </c>
-      <c r="D81" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D81" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E81" s="13" t="inlineStr">
@@ -18978,7 +19003,11 @@
           <t>Safety: fix this first. Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I81" s="13" t="inlineStr"/>
+      <c r="I81" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: both lines now warm only to 78F, the top of the setup range.</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="32" t="inlineStr">
@@ -19050,9 +19079,9 @@
           <t>content/guides/aquarium-ich-treatment-guide.mdx</t>
         </is>
       </c>
-      <c r="D84" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D84" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E84" s="13" t="inlineStr">
@@ -19075,7 +19104,11 @@
           <t>Safety: fix this first. Fix it in the shared cross-species guide; one edit there clears the same conflict for every animal it covers. Source check the figure first.</t>
         </is>
       </c>
-      <c r="I84" s="13" t="inlineStr"/>
+      <c r="I84" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: FAQ and takeaway now give catfish, plecos and loaches a reduced dose, often half.</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="32" t="inlineStr">
@@ -21252,9 +21285,9 @@
           <t>content/guides/aquarium-ich-treatment-guide.mdx</t>
         </is>
       </c>
-      <c r="D158" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D158" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E158" s="13" t="inlineStr">
@@ -21277,7 +21310,11 @@
           <t>Safety: fix this first. Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I158" s="13" t="inlineStr"/>
+      <c r="I158" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: betta, angelfish and livebearer rows changed to No: ich stops reproducing at 86F (aquariumscience.org), above their 82F ceiling.</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="23" t="inlineStr">
@@ -21669,9 +21706,9 @@
           <t>content/guides/budgie-vs-cockatiel-guide.mdx</t>
         </is>
       </c>
-      <c r="D12" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E12" s="13" t="inlineStr">
@@ -21694,7 +21731,11 @@
           <t>Safety: fix this first. Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I12" s="13" t="inlineStr"/>
+      <c r="I12" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: comparison now says spacing stays half an inch or smaller for both.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="16" t="inlineStr">
@@ -21943,9 +21984,9 @@
           <t>content/guides/budgie-vs-cockatiel-guide.mdx</t>
         </is>
       </c>
-      <c r="D22" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D22" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E22" s="13" t="inlineStr">
@@ -21968,7 +22009,11 @@
           <t>Safety: fix this first. Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I22" s="13" t="inlineStr"/>
+      <c r="I22" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: same fix as the budgie row.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="18" t="inlineStr">
@@ -25110,9 +25155,9 @@
           <t>content/guides/chinchilla-vs-hamster-guide.mdx</t>
         </is>
       </c>
-      <c r="D24" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D24" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E24" s="13" t="inlineStr">
@@ -25135,7 +25180,11 @@
           <t>Safety: fix this first. Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I24" s="13" t="inlineStr"/>
+      <c r="I24" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: comparison now about 600 sq in dwarf, 700+ Syrian.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="17" t="inlineStr">
@@ -27081,9 +27130,9 @@
           <t>content/guides/flying-squirrel-cost-guide.mdx</t>
         </is>
       </c>
-      <c r="D85" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D85" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E85" s="13" t="inlineStr">
@@ -27106,7 +27155,11 @@
           <t>Safety: fix this first. Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I85" s="13" t="inlineStr"/>
+      <c r="I85" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: calcium stays required; D3 multivitamin is a vet-set dose. Table row kept (combo pack includes the plain calcium).</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="30" t="inlineStr">
@@ -28569,9 +28622,9 @@
           <t>content/guides/rat-tank-setup-guide.mdx</t>
         </is>
       </c>
-      <c r="D133" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D133" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E133" s="13" t="inlineStr">
@@ -28594,7 +28647,11 @@
           <t>Safety: fix this first. Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I133" s="13" t="inlineStr"/>
+      <c r="I133" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: 86F changed to 80F in both lines and the hub (Lafeber, rescues: risk above 80F).</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="12" t="inlineStr">
@@ -29370,9 +29427,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D13" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E13" s="13" t="inlineStr">
@@ -29395,7 +29452,11 @@
           <t>Safety: fix this first. Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I13" s="13" t="inlineStr"/>
+      <c r="I13" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: hub FAQ now says no bigger than the abdomen.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="17" t="inlineStr">
@@ -29704,9 +29765,9 @@
           <t>content/guides/uromastyx-tokay-africangrey-jumpingspider-overview.mdx</t>
         </is>
       </c>
-      <c r="D23" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D23" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E23" s="13" t="inlineStr">
@@ -29729,7 +29790,11 @@
           <t>Safety: fix this first. Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I23" s="13" t="inlineStr"/>
+      <c r="I23" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: overview now says no bigger than the abdomen.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="18" t="inlineStr">
@@ -30440,9 +30505,9 @@
           <t>content/guides/four-unusual-pets-overview.mdx</t>
         </is>
       </c>
-      <c r="D47" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D47" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E47" s="13" t="inlineStr">
@@ -30465,7 +30530,11 @@
           <t>Safety: fix this first. Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I47" s="13" t="inlineStr"/>
+      <c r="I47" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: overview now 75 to 85% to match the setup guide (sources span 70 to 85%).</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="21" t="inlineStr">
@@ -34837,9 +34906,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D16" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D16" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E16" s="13" t="inlineStr">
@@ -34862,7 +34931,11 @@
           <t>Safety: fix this first. Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I16" s="13" t="inlineStr"/>
+      <c r="I16" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: raised bowl replaced with slow-feeder bowl in costs, diet, checklist and FAQ (Glickman 2000, JAVMA).</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="21" t="inlineStr">
@@ -35003,9 +35076,9 @@
           <t>content/guides/why-your-dog-needs-daily-exercise.mdx</t>
         </is>
       </c>
-      <c r="D22" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D22" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E22" s="13" t="inlineStr">
@@ -35028,7 +35101,11 @@
           <t>Safety: fix this first. Fix it in the shared cross-species guide; one edit there clears the same conflict for every animal it covers. Source check the figure first.</t>
         </is>
       </c>
-      <c r="I22" s="13" t="inlineStr"/>
+      <c r="I22" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: hound activities now long-line tracking and sprinting in a fenced area.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="25" t="inlineStr">

</xml_diff>

<commit_message>
Safety sweep: apply Fable review corrections
Revert the flying squirrel cost guide and the large-breed cost row (cost
data is off limits), and the betta and angelfish ich rows. Keep cooked
tegu eggs and rewrite that feeding paragraph in original wording. Fix
the garter pair line left behind, cory ich heat for sterbai, ich dosing
for scaleless fish, jumping spider prey to the sourced ratio, hermit
crab humidity wording, and soften the raised-bowl lines. Workbook notes
corrected; two cost rows reopened.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CONSISTENCY_CHECK.xlsx
+++ b/CONSISTENCY_CHECK.xlsx
@@ -2647,7 +2647,7 @@
         <v>8</v>
       </c>
       <c r="D72" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E72" s="4">
         <f>C72-D72</f>
@@ -2658,7 +2658,7 @@
         <v/>
       </c>
       <c r="G72" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73">
@@ -3517,7 +3517,7 @@
         <v>1</v>
       </c>
       <c r="D102" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E102" s="4">
         <f>C102-D102</f>
@@ -3528,7 +3528,7 @@
         <v/>
       </c>
       <c r="G102" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="103">
@@ -5712,7 +5712,7 @@
       </c>
       <c r="I57" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: hub now soaks early shed, vet for a tight band or dark toe.</t>
+          <t>2026-10-05: hub now soaks early shed, vet for a tight band or dark toe. Matches the health guide and its listed Reptile Direct source.</t>
         </is>
       </c>
     </row>
@@ -9862,7 +9862,7 @@
       </c>
       <c r="I191" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: raw eggs changed to cooked eggs (raw white blocks biotin).</t>
+          <t>2026-10-05: owner chose cooked eggs (ReptiFiles: raw white blocks biotin; the page's LafeberVet sheet allows raw). Feeding paragraph also rewritten in original wording; it tracked the LafeberVet PDF too closely.</t>
         </is>
       </c>
     </row>
@@ -11766,7 +11766,7 @@
       </c>
       <c r="I251" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: ReptiFiles confirms common, checkered, wandering, coast garters are not cohabited; pair line removed from hub.</t>
+          <t>2026-10-05: ReptiFiles (on the enrichment page) and Bio Dude (on the tank page) say common, checkered, wandering and coast garters are not cohabited; pair line removed from hub. PetMD and Reptiles Magazine on the tank page still endorse pairs.</t>
         </is>
       </c>
     </row>
@@ -11883,7 +11883,7 @@
       </c>
       <c r="I254" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: FAQ now says it depends on species and names the four kept alone (ReptiFiles).</t>
+          <t>2026-10-05: FAQ now says it depends on species and names the four kept alone (ReptiFiles, listed on the page).</t>
         </is>
       </c>
     </row>
@@ -12054,7 +12054,7 @@
       </c>
       <c r="I259" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: mated-pair 55-gallon lines replaced with one snake per enclosure (ReptiFiles).</t>
+          <t>2026-10-05: pair lines at 45, 63 and 65 replaced with one snake per enclosure (Bio Dude, listed). PetMD and Reptiles Magazine on this page still endorse pairs; left for the owner.</t>
         </is>
       </c>
     </row>
@@ -18807,7 +18807,7 @@
       </c>
       <c r="I75" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: hub now warms only to 78F with reduced-dose medication.</t>
+          <t>2026-10-05: hub now warms to the top of the species range, 78F for most cories and 82F for a sterbai, with a reduced dose. The half or quarter dose on the health guide is not in its listed sources (Aquarium Co-Op says no half strength); not fixed here.</t>
         </is>
       </c>
     </row>
@@ -19005,7 +19005,7 @@
       </c>
       <c r="I81" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: both lines now warm only to 78F, the top of the setup range.</t>
+          <t>2026-10-05: both lines now warm to the top of the species range, 78F for most, 82F for a sterbai, matching the setup guide.</t>
         </is>
       </c>
     </row>
@@ -19106,7 +19106,7 @@
       </c>
       <c r="I84" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: FAQ and takeaway now give catfish, plecos and loaches a reduced dose, often half.</t>
+          <t>2026-10-05: FAQ and takeaway now say to use the label dose for scaleless fish, half for formalin (UF IFAS, listed). Aquarium Co-Op (listed) says no half strength for Ich-X.</t>
         </is>
       </c>
     </row>
@@ -21312,7 +21312,7 @@
       </c>
       <c r="I158" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: betta, angelfish and livebearer rows changed to No: ich stops reproducing at 86F (aquariumscience.org), above their 82F ceiling.</t>
+          <t>2026-10-05: guppy, molly, swordtail row changed to No, since 82F is under the 86F line (VCA, listed). Betta and angelfish rows left as Yes by owner choice. Line 72 rewritten; it was a near copy of VCA.</t>
         </is>
       </c>
     </row>
@@ -21733,7 +21733,7 @@
       </c>
       <c r="I12" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: comparison now says spacing stays half an inch or smaller for both.</t>
+          <t>2026-10-05: comparison now says half an inch or smaller for both (Merck, PetMD on the setup guide). The comparison page's own LafeberVet source allows 0.5 to 0.75 in for cockatiels.</t>
         </is>
       </c>
     </row>
@@ -25182,7 +25182,7 @@
       </c>
       <c r="I24" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: comparison now about 600 sq in dwarf, 700+ Syrian.</t>
+          <t>2026-10-05: comparison now about 600 sq in dwarf, 700+ Syrian, matching the setup guide. Published minimums run 700 to 900 sq in Syrian (PDSA, PetMD).</t>
         </is>
       </c>
     </row>
@@ -27130,9 +27130,9 @@
           <t>content/guides/flying-squirrel-cost-guide.mdx</t>
         </is>
       </c>
-      <c r="D85" s="14" t="inlineStr">
-        <is>
-          <t>✓ Fixed</t>
+      <c r="D85" s="15" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="E85" s="13" t="inlineStr">
@@ -27157,7 +27157,7 @@
       </c>
       <c r="I85" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: calcium stays required; D3 multivitamin is a vet-set dose. Table row kept (combo pack includes the plain calcium).</t>
+          <t>2026-10-05: cost guides are off limits (owner). Note only: the cost guide calls the calcium and multivitamin combo not optional, while the feeding guide makes the D3 multivitamin a vet-set dose (Squirrel Refuge). Needs owner OK to change.</t>
         </is>
       </c>
     </row>
@@ -28649,7 +28649,7 @@
       </c>
       <c r="I133" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: 86F changed to 80F in both lines and the hub (Lafeber, rescues: risk above 80F).</t>
+          <t>2026-10-05: 86F changed to 80F in both lines and the hub. VCA (listed on the rat page): keep at or below 80F.</t>
         </is>
       </c>
     </row>
@@ -29454,7 +29454,7 @@
       </c>
       <c r="I13" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: hub FAQ now says no bigger than the abdomen.</t>
+          <t>2026-10-05: settled on the sourced ratio instead: half the spider's body length, three quarters at most (Bugs in Cyberspace, listed). Hub FAQ and feeding guide changed; the abdomen rule had no source.</t>
         </is>
       </c>
     </row>
@@ -29792,7 +29792,7 @@
       </c>
       <c r="I23" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: overview now says no bigger than the abdomen.</t>
+          <t>2026-10-05: overview left as it was (half to three quarters, sourced); the feeding guide and hub now match it.</t>
         </is>
       </c>
     </row>
@@ -30532,7 +30532,7 @@
       </c>
       <c r="I47" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: overview now 75 to 85% to match the setup guide (sources span 70 to 85%).</t>
+          <t>2026-10-05: overview now says high 70s to low 80s percent, which fits both its own Tree of Life source (70 to 80%) and the setup guide (75 to 85%).</t>
         </is>
       </c>
     </row>
@@ -34906,9 +34906,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D16" s="14" t="inlineStr">
-        <is>
-          <t>✓ Fixed</t>
+      <c r="D16" s="15" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="E16" s="13" t="inlineStr">
@@ -34933,7 +34933,7 @@
       </c>
       <c r="I16" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: raised bowl replaced with slow-feeder bowl in costs, diet, checklist and FAQ (Glickman 2000, JAVMA).</t>
+          <t>2026-10-05: diet line, checklist and FAQ fixed to match the bloat guide (Glickman 2000 found more bloat with raised bowls, Pipan 2012 found no link; no study shows they help). Still open: cost row L194 lists a raised food bowl; cost data off limits, needs owner OK.</t>
         </is>
       </c>
     </row>
@@ -35103,7 +35103,7 @@
       </c>
       <c r="I22" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: hound activities now long-line tracking and sprinting in a fenced area.</t>
+          <t>2026-10-05: hound activities now long-line tracking and sprinting in a fenced area (National Beagle Club: on leash at all times).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Consistency sweep: fish factual rows
Molly ich treatment, angelfish overview tank size, discus tankmates,
koi pump turnover, neon temperature in the stocking guide, swordtail
tank size. Cost lines and the koi temperature row left as notes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CONSISTENCY_CHECK.xlsx
+++ b/CONSISTENCY_CHECK.xlsx
@@ -1806,7 +1806,7 @@
         <v>7</v>
       </c>
       <c r="D43" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E43" s="4">
         <f>C43-D43</f>
@@ -1817,7 +1817,7 @@
         <v/>
       </c>
       <c r="G43" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44">
@@ -1875,7 +1875,7 @@
         <v/>
       </c>
       <c r="G45" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46">
@@ -1893,7 +1893,7 @@
         <v>9</v>
       </c>
       <c r="D46" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E46" s="4">
         <f>C46-D46</f>
@@ -1904,7 +1904,7 @@
         <v/>
       </c>
       <c r="G46" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47">
@@ -1951,7 +1951,7 @@
         <v>9</v>
       </c>
       <c r="D48" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E48" s="4">
         <f>C48-D48</f>
@@ -1962,7 +1962,7 @@
         <v/>
       </c>
       <c r="G48" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="49">
@@ -2020,7 +2020,7 @@
         <v/>
       </c>
       <c r="G50" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51">
@@ -2038,7 +2038,7 @@
         <v>8</v>
       </c>
       <c r="D51" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E51" s="4">
         <f>C51-D51</f>
@@ -2049,7 +2049,7 @@
         <v/>
       </c>
       <c r="G51" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52">
@@ -2067,7 +2067,7 @@
         <v>9</v>
       </c>
       <c r="D52" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E52" s="4">
         <f>C52-D52</f>
@@ -2078,7 +2078,7 @@
         <v/>
       </c>
       <c r="G52" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53">
@@ -2165,7 +2165,7 @@
         <v/>
       </c>
       <c r="G55" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="56">
@@ -17196,9 +17196,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D23" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D23" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E23" s="13" t="inlineStr">
@@ -17221,7 +17221,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I23" s="13" t="inlineStr"/>
+      <c r="I23" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: hub emergency line now warms to about 82F, then salt or an ich medication, matching the ich guide.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="19" t="inlineStr">
@@ -17390,9 +17394,9 @@
           <t>content/guides/molly-health-issues-guide.mdx</t>
         </is>
       </c>
-      <c r="D29" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D29" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E29" s="13" t="inlineStr">
@@ -17415,7 +17419,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I29" s="13" t="inlineStr"/>
+      <c r="I29" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: both lines now lead with a slow warm-up to about 82F, then salt or malachite green or formalin; copper kept as a last pick because its dose needs an alkalinity test (ich guide). Listed Aquarium Co-Op livebearer page names Ich-X.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="19" t="inlineStr">
@@ -17981,9 +17989,9 @@
           <t>content/guides/ackie-milksnake-mhc-angelfish-overview.mdx</t>
         </is>
       </c>
-      <c r="D50" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D50" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E50" s="13" t="inlineStr">
@@ -18006,7 +18014,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I50" s="13" t="inlineStr"/>
+      <c r="I50" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: overview now says 29 gallon tall for one adult, 55 for four to six, matching the setup guide. Note: Aquarium Co-Op (listed on both pages) allows up to four adults in a 29 gallon community tank; the old overview line was a near copy of it. Owner may want the setup guide reviewed.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="23" t="inlineStr">
@@ -18193,7 +18205,11 @@
           <t>Copy the cost guide's figure into the hub line, exactly as the cost guide prints it.</t>
         </is>
       </c>
-      <c r="I55" s="13" t="inlineStr"/>
+      <c r="I55" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: cost figures are off limits (owner). Note only: hub route line says $155 to $265, cost guide says roughly $150 to $310. Needs owner OK.</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="26" t="inlineStr">
@@ -18400,9 +18416,9 @@
           <t>content/guides/discus-handling-guide.mdx</t>
         </is>
       </c>
-      <c r="D63" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D63" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E63" s="13" t="inlineStr">
@@ -18425,7 +18441,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I63" s="13" t="inlineStr"/>
+      <c r="I63" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: discus handling guide and hub now say a bristlenose is a compromise past its 80F comfort, and only for a discus tank held at the cool end. aqua-fish (listed) names bristlenose as a discus tankmate.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="26" t="inlineStr">
@@ -18852,7 +18872,11 @@
           <t>Copy the cost guide's figure into the hub line, exactly as the cost guide prints it.</t>
         </is>
       </c>
-      <c r="I76" s="13" t="inlineStr"/>
+      <c r="I76" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: cost figures are off limits (owner). Note only: hub route line says $150 to $215, cost guide says roughly $140 to $250. Needs owner OK.</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="32" t="inlineStr">
@@ -19126,9 +19150,9 @@
           <t>content/guides/discus-handling-guide.mdx</t>
         </is>
       </c>
-      <c r="D85" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D85" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E85" s="13" t="inlineStr">
@@ -19151,7 +19175,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I85" s="13" t="inlineStr"/>
+      <c r="I85" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: discus handling guide and hub now say sterbai fits only a tank held near 82F, the top of its range.</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="33" t="inlineStr">
@@ -19631,9 +19659,9 @@
           <t>content/guides/aquarium-ich-treatment-guide.mdx</t>
         </is>
       </c>
-      <c r="D104" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D104" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E104" s="13" t="inlineStr">
@@ -19656,7 +19684,11 @@
           <t>Fix it in the shared cross-species guide; one edit there clears the same conflict for every animal it covers. Source check the figure first.</t>
         </is>
       </c>
-      <c r="I104" s="13" t="inlineStr"/>
+      <c r="I104" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: cleared by the safety row fix (Fish row 158): guppy, molly, swordtail row now says No.</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="36" t="inlineStr">
@@ -19775,9 +19807,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D108" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D108" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E108" s="13" t="inlineStr">
@@ -19800,7 +19832,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I108" s="13" t="inlineStr"/>
+      <c r="I108" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: hub buy list now says once or twice an hour, matching the setup guide and KoiPondCalculator (listed): one to two turnovers an hour for koi.</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="12" t="inlineStr">
@@ -19913,7 +19949,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I111" s="13" t="inlineStr"/>
+      <c r="I111" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: left open for the owner. The feeding guide is the sourced side: Hikari (listed) feeds 2 to 4 times daily at 68 to 86F. The setup guide line 76 "59 to 77F outer limits" is not in its PetMD source (PetMD only gives 64 to 75F best). Fixing it means changing the setup guide and the ich table koi row.</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="12" t="inlineStr">
@@ -20313,9 +20353,9 @@
           <t>content/guides/aquarium-stocking-and-tankmates-guide.mdx</t>
         </is>
       </c>
-      <c r="D126" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D126" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E126" s="13" t="inlineStr">
@@ -20338,7 +20378,11 @@
           <t>Fix it in the shared cross-species guide; one edit there clears the same conflict for every animal it covers. Source check the figure first.</t>
         </is>
       </c>
-      <c r="I126" s="13" t="inlineStr"/>
+      <c r="I126" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: stocking guide now says neons do best at 78F or below and top out around 81F, matching the neon setup guide. Cardinal tetra setup guide lines 49 and 69 still give neons a 77F ceiling.</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="17" t="inlineStr">
@@ -20439,7 +20483,11 @@
           <t>Copy the cost guide's figure into the hub line, exactly as the cost guide prints it.</t>
         </is>
       </c>
-      <c r="I129" s="13" t="inlineStr"/>
+      <c r="I129" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: cost figures are off limits (owner). Note only: hub route line says $575 to $670, cost guide says $470 to $685. Needs owner OK.</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="19" t="inlineStr">
@@ -21172,9 +21220,9 @@
           <t>content/guides/swordtail-tank-setup-guide.mdx</t>
         </is>
       </c>
-      <c r="D155" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D155" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E155" s="13" t="inlineStr">
@@ -21197,7 +21245,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I155" s="13" t="inlineStr"/>
+      <c r="I155" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: line 65 now says 30 gallons or more, long rather than tall, so it no longer contradicts the 29 to 30 gallon target. Dropped the 48 by 12 inch footprint (SeriouslyFish, listed), which a 29 gallon does not meet; Aquarium Source (listed) gives 30 gallons for a group.</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="23" t="inlineStr">

</xml_diff>

<commit_message>
Fish sweep: apply Fable review corrections
Swordtail FAQs to 30 gallons, stocking guide credit, angelfish 29 gallon
wording across pages, koi temperature bands, and platy and swordtail ich
treatment matched to the ich guide with links. No numbers changed in
cost or setup guides.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CONSISTENCY_CHECK.xlsx
+++ b/CONSISTENCY_CHECK.xlsx
@@ -2038,7 +2038,7 @@
         <v>8</v>
       </c>
       <c r="D51" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E51" s="4">
         <f>C51-D51</f>
@@ -2049,7 +2049,7 @@
         <v/>
       </c>
       <c r="G51" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="52">
@@ -17421,7 +17421,7 @@
       </c>
       <c r="I29" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: both lines now lead with a slow warm-up to about 82F, then salt or malachite green or formalin; copper kept as a last pick because its dose needs an alkalinity test (ich guide). Listed Aquarium Co-Op livebearer page names Ich-X.</t>
+          <t>2026-10-05: FAQ and body now lead with a slow warm-up to about 82F, then salt or malachite green or formalin; copper last because its dose needs an alkalinity test. Backed by the ich guide (UF IFAS), now linked from the body. The page's own listed sources do not give this protocol.</t>
         </is>
       </c>
     </row>
@@ -18016,7 +18016,7 @@
       </c>
       <c r="I50" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: overview now says 29 gallon tall for one adult, 55 for four to six, matching the setup guide. Note: Aquarium Co-Op (listed on both pages) allows up to four adults in a 29 gallon community tank; the old overview line was a near copy of it. Owner may want the setup guide reviewed.</t>
+          <t>2026-10-05: overview, setup guide (FAQ and body), stocking table and hub now say a 29 gallon tall is the smallest worth starting with, 55 for four to six. "One adult" dropped: no source says it (Aquarium Co-Op allows up to four adults in a 29, angelfishtypes says a pair, SeriouslyFish about 53 gal). Numbers unchanged.</t>
         </is>
       </c>
     </row>
@@ -19924,9 +19924,9 @@
           <t>content/guides/koi-feeding-guide.mdx</t>
         </is>
       </c>
-      <c r="D111" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D111" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E111" s="13" t="inlineStr">
@@ -19951,7 +19951,7 @@
       </c>
       <c r="I111" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: left open for the owner. The feeding guide is the sourced side: Hikari (listed) feeds 2 to 4 times daily at 68 to 86F. The setup guide line 76 "59 to 77F outer limits" is not in its PetMD source (PetMD only gives 64 to 75F best). Fixing it means changing the setup guide and the ich table koi row.</t>
+          <t>2026-10-05: setup guide and hub now call 59 to 77F the band where koi grow best (Koi Organisation International, VIN), not outer limits; feeding guide "optimal growth range" now "the warm band", matching Hikari (listed). Ich table koi row reworded. Numbers unchanged.</t>
         </is>
       </c>
     </row>
@@ -20380,7 +20380,7 @@
       </c>
       <c r="I126" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: stocking guide now says neons do best at 78F or below and top out around 81F, matching the neon setup guide. Cardinal tetra setup guide lines 49 and 69 still give neons a 77F ceiling.</t>
+          <t>2026-10-05: stocking guide now says neons do best at 78F or below and top out around 81F (neon setup guide and its sources), and credits "the tetra pages". Cardinal tetra guide lines 49, 69 and hub row 294 give 77F as the neon comfort ceiling; left as is, since they describe comfort, not the limit.</t>
         </is>
       </c>
     </row>
@@ -21247,7 +21247,7 @@
       </c>
       <c r="I155" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: line 65 now says 30 gallons or more, long rather than tall, so it no longer contradicts the 29 to 30 gallon target. Dropped the 48 by 12 inch footprint (SeriouslyFish, listed), which a 29 gallon does not meet; Aquarium Source (listed) gives 30 gallons for a group.</t>
+          <t>2026-10-05: body and both FAQs (page and hub) now say 30 gallons or more for a group, length over height (Aquarium Source, listed). The 48 by 12 inch footprint (SeriouslyFish, listed) was dropped because the 29 to 30 gallon target does not meet it.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fish sweep: Fable recheck follow-ups
Koi feeding FAQ warm band, cardinal FAQ neon comfort wording, angelfish
29 gallon wording on the cost and setup guides, koi cost guide pump
turnover. No prices changed. Workbook notes corrected.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CONSISTENCY_CHECK.xlsx
+++ b/CONSISTENCY_CHECK.xlsx
@@ -3849,7 +3849,6 @@
         <v/>
       </c>
     </row>
-    <row r="114"/>
     <row r="115">
       <c r="A115" s="9" t="inlineStr">
         <is>
@@ -18016,7 +18015,7 @@
       </c>
       <c r="I50" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: overview, setup guide (FAQ and body), stocking table and hub now say a 29 gallon tall is the smallest worth starting with, 55 for four to six. "One adult" dropped: no source says it (Aquarium Co-Op allows up to four adults in a 29, angelfishtypes says a pair, SeriouslyFish about 53 gal). Numbers unchanged.</t>
+          <t>2026-10-05: overview, setup guide (FAQ and body), stocking table and hub now say a 29 gallon tall is the smallest worth starting with, 55 for four to six. "One adult" dropped: no source says it (Aquarium Co-Op allows up to four adults in a 29, angelfishtypes says a pair, SeriouslyFish about 53 gal). Numbers unchanged. Angelfish cost guide (lines 50, 74, 79, 88) and setup guide line 82 reworded from "single fish" to the same wording; prices unchanged.</t>
         </is>
       </c>
     </row>
@@ -19834,7 +19833,7 @@
       </c>
       <c r="I108" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: hub buy list now says once or twice an hour, matching the setup guide and KoiPondCalculator (listed): one to two turnovers an hour for koi.</t>
+          <t>2026-10-05: hub buy list now says once or twice an hour, matching the setup guide and KoiPondCalculator (listed): one to two turnovers an hour for koi. Koi cost guide line 79 pump wording matched too (factual figure, not a price).</t>
         </is>
       </c>
     </row>
@@ -19951,7 +19950,7 @@
       </c>
       <c r="I111" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: setup guide and hub now call 59 to 77F the band where koi grow best (Koi Organisation International, VIN), not outer limits; feeding guide "optimal growth range" now "the warm band", matching Hikari (listed). Ich table koi row reworded. Numbers unchanged.</t>
+          <t>2026-10-05: setup guide and hub now call 59 to 77F the band where koi grow best, not outer limits (Koi Organisation International: 15 to 25C is the optimal koi range; not listed on the setup guide, whose PetMD source gives only 64 to 75F). Feeding guide body and FAQ now say "the warm band", matching Hikari (listed). Ich table koi row reworded.</t>
         </is>
       </c>
     </row>
@@ -20380,7 +20379,7 @@
       </c>
       <c r="I126" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: stocking guide now says neons do best at 78F or below and top out around 81F (neon setup guide and its sources), and credits "the tetra pages". Cardinal tetra guide lines 49, 69 and hub row 294 give 77F as the neon comfort ceiling; left as is, since they describe comfort, not the limit.</t>
+          <t>2026-10-05: stocking guide now says neons do best at 78F or below and top out around 81F (neon setup guide and its sources), and credits "the tetra pages". Cardinal tetra FAQ line 49 reworded to the 77F neon tetra is comfortable with, matching its body line 69 and hub row 294.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fish sweep: last recheck items
Cardinal hub neon wording, angelfish cost guide sentence, koi setup
turnover line rewritten (too close to its source). No prices changed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CONSISTENCY_CHECK.xlsx
+++ b/CONSISTENCY_CHECK.xlsx
@@ -19833,7 +19833,7 @@
       </c>
       <c r="I108" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: hub buy list now says once or twice an hour, matching the setup guide and KoiPondCalculator (listed): one to two turnovers an hour for koi. Koi cost guide line 79 pump wording matched too (factual figure, not a price).</t>
+          <t>2026-10-05: hub buy list now says once or twice an hour, matching the setup guide and KoiPondCalculator (listed): one to two turnovers an hour for koi. Koi cost guide line 79 pump wording matched too (factual figure, not a price). Setup guide line 96 reworded; it tracked KoiPondCalculator too closely.</t>
         </is>
       </c>
     </row>
@@ -20379,7 +20379,7 @@
       </c>
       <c r="I126" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: stocking guide now says neons do best at 78F or below and top out around 81F (neon setup guide and its sources), and credits "the tetra pages". Cardinal tetra FAQ line 49 reworded to the 77F neon tetra is comfortable with, matching its body line 69 and hub row 294.</t>
+          <t>2026-10-05: stocking guide now says neons do best at 78F or below and top out around 81F (neon setup guide and its sources), and credits "the tetra pages". Cardinal tetra FAQ line 49 and hub row 294 reworded to the 77F neon tetra is comfortable with, matching body line 69.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Consistency sweep: amphibian factual rows
White's tree frog glove FAQ, tiger salamander ban count to twelve on the
hub and cost guide, overview toad toxin line, koi pump example reworded.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CONSISTENCY_CHECK.xlsx
+++ b/CONSISTENCY_CHECK.xlsx
@@ -1632,7 +1632,7 @@
         <v>8</v>
       </c>
       <c r="D37" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E37" s="4">
         <f>C37-D37</f>
@@ -1643,7 +1643,7 @@
         <v/>
       </c>
       <c r="G37" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
@@ -1719,7 +1719,7 @@
         <v>10</v>
       </c>
       <c r="D40" s="5" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E40" s="4">
         <f>C40-D40</f>
@@ -1730,7 +1730,7 @@
         <v/>
       </c>
       <c r="G40" s="5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="41">
@@ -3849,6 +3849,7 @@
         <v/>
       </c>
     </row>
+    <row r="114"/>
     <row r="115">
       <c r="A115" s="9" t="inlineStr">
         <is>
@@ -15597,9 +15598,9 @@
           <t>content/guides/whites-tree-frog-handling-guide.mdx</t>
         </is>
       </c>
-      <c r="D18" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D18" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E18" s="13" t="inlineStr">
@@ -15622,7 +15623,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I18" s="13" t="inlineStr"/>
+      <c r="I18" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: FAQ now says vinyl gloves first, nitrile as the fallback, never latex, matching the body and hub. Merck Clinical Techniques in Amphibians (listed): moistened, powder-free vinyl, not latex.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="17" t="inlineStr">
@@ -16214,9 +16219,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D41" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D41" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E41" s="13" t="inlineStr">
@@ -16239,7 +16244,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I41" s="13" t="inlineStr"/>
+      <c r="I41" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: hub now says twelve, matching the legal guide; its table lists twelve (Wyoming, Alabama, New York, Oregon, Maryland, Delaware, Nebraska, New Jersey, California, Virginia, DC, New York City).</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="23" t="inlineStr">
@@ -16257,9 +16266,9 @@
           <t>content/guides/tiger-salamander-cost-guide.mdx</t>
         </is>
       </c>
-      <c r="D42" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D42" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E42" s="13" t="inlineStr">
@@ -16282,7 +16291,11 @@
           <t>Re-read the legal guide table and its cited statutes, then make this line match the table.</t>
         </is>
       </c>
-      <c r="I42" s="13" t="inlineStr"/>
+      <c r="I42" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: cost guide count changed to twelve (a count, not a price), matching the legal guide table.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="23" t="inlineStr">
@@ -16505,9 +16518,9 @@
           <t>content/guides/greenanole-tegu-firebelliedtoad-tigersalamander-overview.mdx</t>
         </is>
       </c>
-      <c r="D50" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D50" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E50" s="13" t="inlineStr">
@@ -16530,7 +16543,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I50" s="13" t="inlineStr"/>
+      <c r="I50" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: overview no longer calls the toad the only one with skin toxin; it now says the red belly warns of its toxin, which leaves room for the tiger salamander secretions the handling guide describes.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="23" t="inlineStr">
@@ -19833,7 +19850,7 @@
       </c>
       <c r="I108" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: hub buy list now says once or twice an hour, matching the setup guide and KoiPondCalculator (listed): one to two turnovers an hour for koi. Koi cost guide line 79 pump wording matched too (factual figure, not a price). Setup guide line 96 reworded; it tracked KoiPondCalculator too closely.</t>
+          <t>2026-10-05: hub buy list now says once or twice an hour, matching the setup guide and KoiPondCalculator (listed): one to two turnovers an hour for koi. Koi cost guide line 79 pump wording matched too (factual figure, not a price). Setup guide line 96 reworded; it tracked KoiPondCalculator too closely. Line 98 pump example also reworded in original words; figures unchanged.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Consistency sweep: bird factual rows
Cockatoo size on the hub, encyclopedia and comparison matched to VCA's
300 to 900 g; canary housing on the colony guide and zebra finch cost
guide matched to the canary pages. Zebra finch hub prices noted only.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CONSISTENCY_CHECK.xlsx
+++ b/CONSISTENCY_CHECK.xlsx
@@ -2135,16 +2135,16 @@
         <v>11</v>
       </c>
       <c r="D58" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E58" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F58" s="6" t="n">
-        <v>0.6363636363636364</v>
+        <v>0.8181818181818182</v>
       </c>
       <c r="G58" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="59">
@@ -2216,16 +2216,16 @@
         <v>9</v>
       </c>
       <c r="D61" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E61" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="F61" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G61" s="5" t="n">
         <v>2</v>
-      </c>
-      <c r="E61" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="F61" s="6" t="n">
-        <v>0.7777777777777778</v>
-      </c>
-      <c r="G61" s="5" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="62">
@@ -3616,22 +3616,22 @@
         <v>784</v>
       </c>
       <c r="D113" s="7" t="n">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="E113" s="7" t="n">
-        <v>537</v>
+        <v>541</v>
       </c>
       <c r="F113" s="8" t="n">
-        <v>0.6849489795918368</v>
+        <v>0.6900510204081632</v>
       </c>
       <c r="G113" s="7" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="9" t="inlineStr">
         <is>
-          <t>Every number on this tab is a value counted from the category tabs, recounted on each update (no formulas, so it reads the same in any viewer). Conflicts overall: 324 found, 36 fixed, 288 open (11% fixed). Last recount 2026-10-05.</t>
+          <t>Every number on this tab is a value counted from the category tabs, recounted on each update (no formulas, so it reads the same in any viewer). Conflicts overall: 324 found, 40 fixed, 284 open (12% fixed). Last recount 2026-10-05.</t>
         </is>
       </c>
     </row>
@@ -21892,9 +21892,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D24" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D24" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E24" s="13" t="inlineStr">
@@ -21917,7 +21917,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I24" s="13" t="inlineStr"/>
+      <c r="I24" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: hub Adult size row and the encyclopedia entry (same page, toggle) now say 12 to 27 inches and roughly 300 to 900 g across species, Goffin's and galahs light, Moluccans heavy. VCA Cockatoos General Information: 300 to 900 g, 12 to 27 in. Package figures (about 350 to 880 g) sit inside it.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="19" t="inlineStr">
@@ -22218,9 +22222,9 @@
           <t>content/guides/cockatiel-vs-cockatoo-guide.mdx</t>
         </is>
       </c>
-      <c r="D34" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D34" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E34" s="13" t="inlineStr">
@@ -22243,7 +22247,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I34" s="13" t="inlineStr"/>
+      <c r="I34" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: comparison now says 12 to 27 inches, roughly 300 to 900 g, and a Moluccan or umbrella approaching 900 g instead of over a kilogram. VCA (listed on the page): 300 to 900 g.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="20" t="inlineStr">
@@ -23024,9 +23032,9 @@
           <t>content/guides/bird-colony-aviary-keeping-guide.mdx</t>
         </is>
       </c>
-      <c r="D64" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D64" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E64" s="13" t="inlineStr">
@@ -23049,7 +23057,11 @@
           <t>Fix it in the shared cross-species guide; one edit there clears the same conflict for every animal it covers. Source check the figure first.</t>
         </is>
       </c>
-      <c r="I64" s="13" t="inlineStr"/>
+      <c r="I64" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: colony guide now says one cage per canary is the safest default, never two males, and a male and female pair can share a roomy flight. Lafeber canary page (listed): own cage, territorial. PetMD canary sheet (not listed): males fight, opposite-sex pairs possible. Line 91 now says males above all.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="26" t="inlineStr">
@@ -23067,9 +23079,9 @@
           <t>content/guides/zebra-finch-cost-guide.mdx</t>
         </is>
       </c>
-      <c r="D65" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D65" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E65" s="13" t="inlineStr">
@@ -23092,7 +23104,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I65" s="13" t="inlineStr"/>
+      <c r="I65" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: zebra finch cost guide now says a canary is kept solo, or as a male and female or two females, never two males. No prices touched.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="29" t="inlineStr">
@@ -23988,7 +24004,11 @@
           <t>Copy the cost guide's figure into the hub line, exactly as the cost guide prints it.</t>
         </is>
       </c>
-      <c r="I97" s="13" t="inlineStr"/>
+      <c r="I97" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: prices are never changed (owner). Note only: hub FAQ says setup $180 to $400 and cage $120 to $220; the cost guide says $225 to $465 and $175 to $300. Needs owner OK.</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="36" t="inlineStr">

</xml_diff>

<commit_message>
Consistency sweep: dog and cat factual rows, flying squirrel cost wording
Dog dental brushing, chew hardness, poodle bloat, dachshund IVDD advice,
golden shedding, dysplasia breed figures; cat wet food and kidney
disease, HCM screening ages, Maine Coon growth (fact 288), Persian PKD,
Ragdoll kidney reading. Large-breed bowl row renamed, price kept.
Flying squirrel cost guide wording only, prices unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CONSISTENCY_CHECK.xlsx
+++ b/CONSISTENCY_CHECK.xlsx
@@ -2513,16 +2513,16 @@
         <v>8</v>
       </c>
       <c r="D72" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E72" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F72" s="6" t="n">
-        <v>0.75</v>
+        <v>0.875</v>
       </c>
       <c r="G72" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="73">
@@ -2981,7 +2981,7 @@
         <v>0</v>
       </c>
       <c r="G89" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="90">
@@ -3080,16 +3080,16 @@
         <v>4</v>
       </c>
       <c r="D93" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E93" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F93" s="6" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G93" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="94">
@@ -3107,16 +3107,16 @@
         <v>2</v>
       </c>
       <c r="D94" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E94" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F94" s="6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G94" s="5" t="n">
         <v>2</v>
-      </c>
-      <c r="E94" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F94" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G94" s="5" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="95">
@@ -3143,7 +3143,7 @@
         <v>0</v>
       </c>
       <c r="G95" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="96">
@@ -3242,16 +3242,16 @@
         <v>2</v>
       </c>
       <c r="D99" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E99" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F99" s="6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G99" s="5" t="n">
         <v>2</v>
-      </c>
-      <c r="E99" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F99" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G99" s="5" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="100">
@@ -3305,7 +3305,7 @@
         <v>0</v>
       </c>
       <c r="G101" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="102">
@@ -3323,16 +3323,16 @@
         <v>1</v>
       </c>
       <c r="D102" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E102" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E102" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="F102" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G102" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="103">
@@ -3431,16 +3431,16 @@
         <v>2</v>
       </c>
       <c r="D106" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E106" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F106" s="6" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G106" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="107">
@@ -3512,16 +3512,16 @@
         <v>3</v>
       </c>
       <c r="D109" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E109" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="E109" s="4" t="n">
+      <c r="F109" s="6" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="G109" s="5" t="n">
         <v>1</v>
-      </c>
-      <c r="F109" s="6" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="G109" s="5" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="110">
@@ -3539,16 +3539,16 @@
         <v>3</v>
       </c>
       <c r="D110" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E110" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F110" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="E110" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="F110" s="6" t="n">
-        <v>0.6666666666666666</v>
-      </c>
       <c r="G110" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="111">
@@ -3616,22 +3616,22 @@
         <v>784</v>
       </c>
       <c r="D113" s="7" t="n">
-        <v>243</v>
+        <v>234</v>
       </c>
       <c r="E113" s="7" t="n">
-        <v>541</v>
+        <v>550</v>
       </c>
       <c r="F113" s="8" t="n">
-        <v>0.6900510204081632</v>
+        <v>0.701530612244898</v>
       </c>
       <c r="G113" s="7" t="n">
-        <v>40</v>
+        <v>54</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="9" t="inlineStr">
         <is>
-          <t>Every number on this tab is a value counted from the category tabs, recounted on each update (no formulas, so it reads the same in any viewer). Conflicts overall: 324 found, 40 fixed, 284 open (12% fixed). Last recount 2026-10-05.</t>
+          <t>Every number on this tab is a value counted from the category tabs, recounted on each update (no formulas, so it reads the same in any viewer). Conflicts overall: 324 found, 54 fixed, 270 open (17% fixed). Last recount 2026-10-05.</t>
         </is>
       </c>
     </row>
@@ -26996,9 +26996,9 @@
           <t>content/guides/flying-squirrel-cost-guide.mdx</t>
         </is>
       </c>
-      <c r="D85" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D85" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E85" s="13" t="inlineStr">
@@ -27023,7 +27023,7 @@
       </c>
       <c r="I85" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: cost guides are off limits (owner). Note only: the cost guide calls the calcium and multivitamin combo not optional, while the feeding guide makes the D3 multivitamin a vet-set dose (Squirrel Refuge). Needs owner OK to change.</t>
+          <t>2026-10-05: wording only, prices unchanged (owner OK). FAQ, table label and paragraph now say calcium is required and the combo pack multivitamin, which carries vitamin D3, goes in only at a vet-set dose, matching the feeding guide (Squirrel Refuge MBD page).</t>
         </is>
       </c>
     </row>
@@ -32916,9 +32916,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D3" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D3" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E3" s="13" t="inlineStr">
@@ -32941,7 +32941,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I3" s="13" t="inlineStr"/>
+      <c r="I3" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: general cat hub diet line and FAQ now say wet food raises water intake and helps urinary health, but wet versus dry did not change who developed kidney disease, matching the kidney guide. Maine Coon diet line also drops "and kidney health".</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
@@ -33493,9 +33497,9 @@
           <t>content/guides/cardiomyopathy-in-cats-and-dogs-guide.mdx</t>
         </is>
       </c>
-      <c r="D22" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D22" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E22" s="13" t="inlineStr">
@@ -33518,7 +33522,11 @@
           <t>Fix it in the shared cross-species guide; one edit there clears the same conflict for every animal it covers. Source check the figure first.</t>
         </is>
       </c>
-      <c r="I22" s="13" t="inlineStr"/>
+      <c r="I22" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: cardiomyopathy guide now says echo screening is standard for the four breeds, and for the Maine Coon starts at age 1, yearly until past 3, then at 5, matching the Maine Coon hub.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="23" t="inlineStr">
@@ -33536,9 +33544,9 @@
           <t>fact 288 (src/lib/data/facts.js)</t>
         </is>
       </c>
-      <c r="D23" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D23" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E23" s="13" t="inlineStr">
@@ -33561,7 +33569,11 @@
           <t>Correct the fun fact to match the deep dive; never renumber or remove a fact id.</t>
         </is>
       </c>
-      <c r="I23" s="13" t="inlineStr"/>
+      <c r="I23" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: fact 288 now says up to three years (CFA), matching the hub and encyclopedia. Fact id unchanged.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="23" t="inlineStr">
@@ -33637,9 +33649,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D26" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D26" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E26" s="13" t="inlineStr">
@@ -33662,7 +33674,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I26" s="13" t="inlineStr"/>
+      <c r="I26" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: Persian checklist now asks for PKD1 results for both parents, since one affected parent passes it to about half the litter.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="26" t="inlineStr">
@@ -33766,9 +33782,9 @@
           <t>content/guides/persian-cat-enrichment-guide.mdx</t>
         </is>
       </c>
-      <c r="D29" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D29" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E29" s="13" t="inlineStr">
@@ -33791,7 +33807,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I29" s="13" t="inlineStr"/>
+      <c r="I29" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: Persian enrichment FAQ and body now say PKD was once common and is now rare thanks to DNA testing, still worth asking about, matching the hub and kidney guide.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="26" t="inlineStr">
@@ -33851,9 +33871,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D32" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D32" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E32" s="13" t="inlineStr">
@@ -33876,7 +33896,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I32" s="13" t="inlineStr"/>
+      <c r="I32" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: Ragdoll hub health line and FAQ now read the 1.93 vs 21.18 percent gap as age, not missed diagnoses, matching the kidney guide.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="30" t="inlineStr">
@@ -34345,9 +34369,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D3" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D3" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E3" s="13" t="inlineStr">
@@ -34370,7 +34394,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I3" s="13" t="inlineStr"/>
+      <c r="I3" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: hub health line and FAQ now say brush daily or at least every other day, chews only as a VOHC-sealed fallback, matching the periodontal guide (Merck, greyhound brushing trial).</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
@@ -34458,9 +34486,9 @@
           <t>content/guides/the-best-dog-toys-for-big-and-small-dogs-a-2026-guide.mdx</t>
         </is>
       </c>
-      <c r="D6" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E6" s="13" t="inlineStr">
@@ -34483,7 +34511,11 @@
           <t>Fix it in the shared cross-species guide; one edit there clears the same conflict for every animal it covers. Source check the figure first.</t>
         </is>
       </c>
-      <c r="I6" s="13" t="inlineStr"/>
+      <c r="I6" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: toy guide chew row now says heavy-duty rubber that dents under a thumbnail and to skip hard nylon, matching the periodontal guide (Tufts thumbnail test).</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="16" t="inlineStr">
@@ -34601,9 +34633,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D11" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D11" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E11" s="13" t="inlineStr">
@@ -34626,7 +34658,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I11" s="13" t="inlineStr"/>
+      <c r="I11" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: medium-breed hub health line and FAQ now call the Standard Poodle a real exception near the top of bloat risk lists, matching the bloat guide.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="19" t="inlineStr">
@@ -34772,9 +34808,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D16" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D16" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E16" s="13" t="inlineStr">
@@ -34799,7 +34835,7 @@
       </c>
       <c r="I16" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: diet line, checklist and FAQ fixed to match the bloat guide (Glickman 2000 found more bloat with raised bowls, Pipan 2012 found no link; no study shows they help). Still open: cost row L194 lists a raised food bowl; cost data off limits, needs owner OK.</t>
+          <t>2026-10-05: cost row renamed Slow-feeder bowl, $20 to $35 kept (owner OK for dog and cat guides). Diet line, checklist and FAQ were fixed earlier to match the bloat guide.</t>
         </is>
       </c>
     </row>
@@ -35228,9 +35264,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D32" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D32" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E32" s="13" t="inlineStr">
@@ -35253,7 +35289,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I32" s="13" t="inlineStr"/>
+      <c r="I32" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: Dachshund hub housing line and IVDD FAQ rewritten to the IVDD guide: furniture and stair bans show no protective effect, more than an hour of exercise a day had lower odds, delay neutering, tested parents; ramps kept for a sore dog. Checklist and cost rows for ramps and gates left as is.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="32" t="inlineStr">
@@ -35849,9 +35889,9 @@
           <t>content/guides/golden-retriever-vs-german-shepherd-guide.mdx</t>
         </is>
       </c>
-      <c r="D51" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D51" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E51" s="13" t="inlineStr">
@@ -35874,7 +35914,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I51" s="13" t="inlineStr"/>
+      <c r="I51" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: comparison FAQ and table now say goldens shed year-round with seasonal blowouts on top, matching the golden hub.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="16" t="inlineStr">
@@ -35988,9 +36032,9 @@
           <t>content/guides/hip-and-elbow-dysplasia-guide.mdx</t>
         </is>
       </c>
-      <c r="D56" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D56" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E56" s="13" t="inlineStr">
@@ -36013,7 +36057,11 @@
           <t>Fix it in the shared cross-species guide; one edit there clears the same conflict for every animal it covers. Source check the figure first.</t>
         </is>
       </c>
-      <c r="I56" s="13" t="inlineStr"/>
+      <c r="I56" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: dysplasia guide line 104 rewritten: build tracks with risk, Labradors about 11 percent dysplastic in OFA data, Goldens and Rottweilers near 20 percent; line 133 drops "the two breeds where this matters most". Old line 104 also read close to its source wording.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="18" t="inlineStr">

</xml_diff>

<commit_message>
Consistency sweep: invertebrate and small mammal factual rows
Scorpion molting and handling, hermit crab tank size, hissing cockroach
broods and escapes, millipede arrivals and secretion, mantis hatch
timing, ghost shrimp housing; guinea pig wild cavies and vitamin C,
hamster sand bath, chinchilla tail and fur slip, coat, dust and heat
band, degu cage height, ferret adrenal figures and cause, ferret permit
states, gerbil citrus, mouse male housing and protein, rat vet urgency,
sugar glider Pennsylvania and cage size. Four price lines noted only.
FIX_PACKAGES gains the axolotl and White's tree frog glove notes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CONSISTENCY_CHECK.xlsx
+++ b/CONSISTENCY_CHECK.xlsx
@@ -2351,16 +2351,16 @@
         <v>10</v>
       </c>
       <c r="D66" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E66" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F66" s="6" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="G66" s="5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="67">
@@ -2387,7 +2387,7 @@
         <v>0.7272727272727273</v>
       </c>
       <c r="G67" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="68">
@@ -2432,16 +2432,16 @@
         <v>12</v>
       </c>
       <c r="D69" s="5" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E69" s="4" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F69" s="6" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="G69" s="5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="70">
@@ -2459,16 +2459,16 @@
         <v>9</v>
       </c>
       <c r="D70" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E70" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F70" s="6" t="n">
-        <v>0.7777777777777778</v>
+        <v>0.8888888888888888</v>
       </c>
       <c r="G70" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="71">
@@ -2486,16 +2486,16 @@
         <v>9</v>
       </c>
       <c r="D71" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E71" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F71" s="6" t="n">
-        <v>0.5555555555555556</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="G71" s="5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="72">
@@ -2540,16 +2540,16 @@
         <v>10</v>
       </c>
       <c r="D73" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E73" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F73" s="6" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="G73" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="74">
@@ -2594,16 +2594,16 @@
         <v>7</v>
       </c>
       <c r="D75" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E75" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F75" s="6" t="n">
-        <v>0.4285714285714285</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="G75" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="76">
@@ -2621,16 +2621,16 @@
         <v>7</v>
       </c>
       <c r="D76" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E76" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="F76" s="6" t="n">
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="G76" s="5" t="n">
         <v>2</v>
-      </c>
-      <c r="E76" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="F76" s="6" t="n">
-        <v>0.7142857142857143</v>
-      </c>
-      <c r="G76" s="5" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="77">
@@ -2648,16 +2648,16 @@
         <v>8</v>
       </c>
       <c r="D77" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E77" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F77" s="6" t="n">
-        <v>0.625</v>
+        <v>0.75</v>
       </c>
       <c r="G77" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="78">
@@ -2729,16 +2729,16 @@
         <v>12</v>
       </c>
       <c r="D80" s="5" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E80" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F80" s="6" t="n">
-        <v>0.5</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="G80" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="81">
@@ -2756,16 +2756,16 @@
         <v>8</v>
       </c>
       <c r="D81" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E81" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="F81" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="E81" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="F81" s="6" t="n">
-        <v>0.875</v>
-      </c>
       <c r="G81" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="82">
@@ -2783,16 +2783,16 @@
         <v>6</v>
       </c>
       <c r="D82" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E82" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F82" s="6" t="n">
-        <v>0.1666666666666667</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="G82" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="83">
@@ -2810,16 +2810,16 @@
         <v>9</v>
       </c>
       <c r="D83" s="5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E83" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F83" s="6" t="n">
-        <v>0.4444444444444444</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="G83" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="84">
@@ -2846,7 +2846,7 @@
         <v>0.6666666666666666</v>
       </c>
       <c r="G84" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="85">
@@ -2918,16 +2918,16 @@
         <v>7</v>
       </c>
       <c r="D87" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E87" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="E87" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="F87" s="6" t="n">
-        <v>0.4285714285714285</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="G87" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="88">
@@ -3616,22 +3616,22 @@
         <v>784</v>
       </c>
       <c r="D113" s="7" t="n">
-        <v>234</v>
+        <v>215</v>
       </c>
       <c r="E113" s="7" t="n">
-        <v>550</v>
+        <v>569</v>
       </c>
       <c r="F113" s="8" t="n">
-        <v>0.701530612244898</v>
+        <v>0.7257653061224489</v>
       </c>
       <c r="G113" s="7" t="n">
-        <v>54</v>
+        <v>80</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="9" t="inlineStr">
         <is>
-          <t>Every number on this tab is a value counted from the category tabs, recounted on each update (no formulas, so it reads the same in any viewer). Conflicts overall: 324 found, 54 fixed, 270 open (17% fixed). Last recount 2026-10-05.</t>
+          <t>Every number on this tab is a value counted from the category tabs, recounted on each update (no formulas, so it reads the same in any viewer). Conflicts overall: 324 found, 80 fixed, 244 open (25% fixed). Last recount 2026-10-05.</t>
         </is>
       </c>
     </row>
@@ -24362,9 +24362,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D3" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D3" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E3" s="13" t="inlineStr">
@@ -24387,7 +24387,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I3" s="13" t="inlineStr"/>
+      <c r="I3" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: hub route line now says a wild cavy's day.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
@@ -24432,9 +24436,9 @@
           <t>content/guides/guinea-pig-enrichment-guide.mdx</t>
         </is>
       </c>
-      <c r="D5" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E5" s="13" t="inlineStr">
@@ -24459,7 +24463,7 @@
       </c>
       <c r="I5" s="13" t="inlineStr">
         <is>
-          <t>Source check needed.</t>
+          <t>2026-10-05: enrichment guide excerpt, description, FAQ and body now say wild cavies, the guinea pig's closest relatives; no wild Cavia porcellus exists (legal guide).</t>
         </is>
       </c>
     </row>
@@ -24479,9 +24483,9 @@
           <t>content/guides/guinea-pig-feeding-guide.mdx</t>
         </is>
       </c>
-      <c r="D6" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E6" s="13" t="inlineStr">
@@ -24504,7 +24508,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I6" s="13" t="inlineStr"/>
+      <c r="I6" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: feeding guide now says about one and a half times an adult's vitamin C, 30 to 40 mg a day against 20 to 25, matching the scurvy guide.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
@@ -24727,7 +24735,7 @@
       </c>
       <c r="I13" s="13" t="inlineStr">
         <is>
-          <t>Logged in FIX_PACKAGES.md.</t>
+          <t>2026-10-05: care package, never edited from the sweep. Already listed in FIX_PACKAGES.md under Guinea pig.</t>
         </is>
       </c>
     </row>
@@ -25068,9 +25076,9 @@
           <t>content/guides/chinchilla-vs-hamster-guide.mdx</t>
         </is>
       </c>
-      <c r="D25" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D25" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E25" s="13" t="inlineStr">
@@ -25093,7 +25101,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I25" s="13" t="inlineStr"/>
+      <c r="I25" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: comparison FAQ and table now say a hamster needs a sand bath, not dust, matching the hamster setup guide.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="17" t="inlineStr">
@@ -25987,9 +25999,9 @@
           <t>content/guides/chinchilla-vs-hamster-guide.mdx</t>
         </is>
       </c>
-      <c r="D54" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D54" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E54" s="13" t="inlineStr">
@@ -26012,7 +26024,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I54" s="13" t="inlineStr"/>
+      <c r="I54" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: comparison FAQ and body no longer say the tail can deglove; never lift by the tail, a light tail-base hold can steady it, and grabbing the coat can trigger fur slip, matching the handling guide.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="21" t="inlineStr">
@@ -26030,9 +26046,9 @@
           <t>content/guides/four-unusual-pets-overview.mdx</t>
         </is>
       </c>
-      <c r="D55" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D55" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E55" s="13" t="inlineStr">
@@ -26055,7 +26071,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I55" s="13" t="inlineStr"/>
+      <c r="I55" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: overview now says up to 80 hairs per follicle and a bath of up to 15 minutes two or three times a week, matching the encyclopedia and setup guide.</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="21" t="inlineStr">
@@ -26073,9 +26093,9 @@
           <t>content/guides/small-mammal-temperature-heat-stress-guide.mdx</t>
         </is>
       </c>
-      <c r="D56" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D56" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E56" s="13" t="inlineStr">
@@ -26098,7 +26118,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I56" s="13" t="inlineStr"/>
+      <c r="I56" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: heat stress guide line 59 now says about 50 to 68F, cold tolerant, danger near 80F, matching its own table and the setup guide.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="22" t="inlineStr">
@@ -26433,9 +26457,9 @@
           <t>content/guides/degu-gerbil-overview.mdx</t>
         </is>
       </c>
-      <c r="D68" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D68" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E68" s="13" t="inlineStr">
@@ -26458,7 +26482,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I68" s="13" t="inlineStr"/>
+      <c r="I68" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: overview now says at least about 28 inches high for a pair and closer to 3 feet when possible. PetMD (on the setup guide): 28 x 18 x 28 in for two; Royal Veterinary Center (on both pages): about 90 cm high.</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="25" t="inlineStr">
@@ -26728,9 +26756,9 @@
           <t>content/guides/ferret-health-issues-guide.mdx</t>
         </is>
       </c>
-      <c r="D77" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D77" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E77" s="13" t="inlineStr">
@@ -26753,7 +26781,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I77" s="13" t="inlineStr"/>
+      <c r="I77" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: FAQ and body now present the figures as population-dependent (about 0.55 percent in Dutch studies, about a quarter of US ferrets, a repeated 70 percent estimate for 2003) instead of a range the 70 percent falls outside.</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="26" t="inlineStr">
@@ -26771,9 +26803,9 @@
           <t>content/guides/ferret-health-issues-guide.mdx</t>
         </is>
       </c>
-      <c r="D78" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D78" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E78" s="13" t="inlineStr">
@@ -26796,7 +26828,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I78" s="13" t="inlineStr"/>
+      <c r="I78" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: FAQ and body now name neutering itself as the leading suspect and say age at neutering is no longer thought to matter much, matching the adrenal guide.</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="26" t="inlineStr">
@@ -26814,9 +26850,9 @@
           <t>content/guides/ferret-legal-guide.mdx</t>
         </is>
       </c>
-      <c r="D79" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D79" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E79" s="13" t="inlineStr">
@@ -26839,7 +26875,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I79" s="13" t="inlineStr"/>
+      <c r="I79" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: lines 46 and 88 now name New Jersey and Rhode Island as the permit states, matching the table. A spaced hyphen used as a dash on line 46 removed too.</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="26" t="inlineStr">
@@ -27419,9 +27459,9 @@
           <t>content/guides/gerbil-feeding-guide.mdx</t>
         </is>
       </c>
-      <c r="D98" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D98" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E98" s="13" t="inlineStr">
@@ -27444,7 +27484,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I98" s="13" t="inlineStr"/>
+      <c r="I98" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: FAQ now rations citrus as acidic rather than listing it as toxic, matching the body.</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="32" t="inlineStr">
@@ -28042,9 +28086,9 @@
           <t>content/guides/mouse-cost-guide.mdx</t>
         </is>
       </c>
-      <c r="D119" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D119" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E119" s="13" t="inlineStr">
@@ -28067,7 +28111,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I119" s="13" t="inlineStr"/>
+      <c r="I119" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: cost guide now says females belong in groups and a lone male is the common outcome for adult males, matching the enrichment guide and hub.</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="36" t="inlineStr">
@@ -28112,9 +28160,9 @@
           <t>content/guides/mouse-feeding-guide.mdx</t>
         </is>
       </c>
-      <c r="D121" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D121" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E121" s="13" t="inlineStr">
@@ -28137,7 +28185,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I121" s="13" t="inlineStr"/>
+      <c r="I121" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: mouse feeding FAQ and hub now compare against the gerbil's 18 to 20 percent target, matching the gerbil feeding guide; hub Diet row drops the 14 to 16 figure.</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="36" t="inlineStr">
@@ -28445,9 +28497,9 @@
           <t>content/guides/rat-health-issues-guide.mdx</t>
         </is>
       </c>
-      <c r="D132" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D132" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E132" s="13" t="inlineStr">
@@ -28470,7 +28522,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I132" s="13" t="inlineStr"/>
+      <c r="I132" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: lines 94 and 66 now make labored breathing, head tilt and sudden lethargy a prompt or same-day visit, with lingering sneezing within the week, matching the FAQ and hub emergency card.</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="12" t="inlineStr">
@@ -28629,7 +28685,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I137" s="13" t="inlineStr"/>
+      <c r="I137" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: prices are never changed (owner). Note only: FAQ and hub say setup $500 to $1,200 for a pair, while the itemized table totals about $250 to $550 plus a pouch.</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="17" t="inlineStr">
@@ -28647,9 +28707,9 @@
           <t>content/guides/sugar-glider-cost-guide.mdx</t>
         </is>
       </c>
-      <c r="D138" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D138" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E138" s="13" t="inlineStr">
@@ -28672,7 +28732,11 @@
           <t>Re-read the legal guide table and its cited statutes, then make this line match the table.</t>
         </is>
       </c>
-      <c r="I138" s="13" t="inlineStr"/>
+      <c r="I138" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: cost guide FAQ now says Pennsylvania bars possession with no pet permit path, matching the legal guide.</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="17" t="inlineStr">
@@ -28841,9 +28905,9 @@
           <t>content/guides/sugar-glider-tank-setup-guide.mdx</t>
         </is>
       </c>
-      <c r="D144" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D144" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E144" s="13" t="inlineStr">
@@ -28866,7 +28930,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I144" s="13" t="inlineStr"/>
+      <c r="I144" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: the linked Critter Nation double unit is really 36 by 24 by 63 inches (retailer listings); the line now says so and that it clears the 36 x 24 x 36 minimum. Catalog covers text "24x24x48 in multi-level cage" left as is.</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="17" t="inlineStr">
@@ -29365,7 +29433,11 @@
           <t>Copy the cost guide's figure into the hub line, exactly as the cost guide prints it.</t>
         </is>
       </c>
-      <c r="I14" s="13" t="inlineStr"/>
+      <c r="I14" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: prices are never changed (owner). Note only: hub route line says setup $112 to $150; the cost guide and hub Budget row say $75 to $180.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="17" t="inlineStr">
@@ -29968,9 +30040,9 @@
           <t>content/guides/10-surprising-emperor-scorpion-facts.mdx</t>
         </is>
       </c>
-      <c r="D34" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D34" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E34" s="13" t="inlineStr">
@@ -29993,7 +30065,11 @@
           <t>Correct the fun fact to match the deep dive; never renumber or remove a fact id.</t>
         </is>
       </c>
-      <c r="I34" s="13" t="inlineStr"/>
+      <c r="I34" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: fun fact now says a young scorpion molts around five times and never again once mature, matching the health guide.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="19" t="inlineStr">
@@ -30054,9 +30130,9 @@
           <t>content/guides/invertebrate-rehousing-guide.mdx</t>
         </is>
       </c>
-      <c r="D36" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D36" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E36" s="13" t="inlineStr">
@@ -30079,7 +30155,11 @@
           <t>Fix it in the shared cross-species guide; one edit there clears the same conflict for every animal it covers. Source check the figure first.</t>
         </is>
       </c>
-      <c r="I36" s="13" t="inlineStr"/>
+      <c r="I36" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: rehousing FAQ and table now give both reasons, the sting and a fall that can injure the scorpion, and say to work low over a soft surface, matching the handling guide.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="19" t="inlineStr">
@@ -30418,9 +30498,9 @@
           <t>content/guides/four-unusual-pets-overview.mdx</t>
         </is>
       </c>
-      <c r="D48" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D48" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E48" s="13" t="inlineStr">
@@ -30443,7 +30523,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I48" s="13" t="inlineStr"/>
+      <c r="I48" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: overview now says at least 10 gallons per small or medium crab, so a pair starts at 20, matching the setup guide.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="22" t="inlineStr">
@@ -30702,9 +30786,9 @@
           <t>content/guides/10-surprising-hissing-cockroach-facts.mdx</t>
         </is>
       </c>
-      <c r="D56" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D56" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E56" s="13" t="inlineStr">
@@ -30727,7 +30811,11 @@
           <t>Correct the fun fact to match the deep dive; never renumber or remove a fact id.</t>
         </is>
       </c>
-      <c r="I56" s="13" t="inlineStr"/>
+      <c r="I56" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: fun fact now says a brood usually holds 15 to 40 nymphs and a big female can reach about 60. ADW: 15 to 40; University of Kentucky (listed on the fact page): as many as 30 to 60.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="23" t="inlineStr">
@@ -30745,9 +30833,9 @@
           <t>content/guides/10-surprising-hissing-cockroach-facts.mdx</t>
         </is>
       </c>
-      <c r="D57" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D57" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E57" s="13" t="inlineStr">
@@ -30770,7 +30858,11 @@
           <t>Correct the fun fact to match the deep dive; never renumber or remove a fact id.</t>
         </is>
       </c>
-      <c r="I57" s="13" t="inlineStr"/>
+      <c r="I57" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: fun fact now says they are not escape-proof: foot pads and hooks climb smooth glass (ADW), so a tight lid and a petroleum jelly band, matching the setup guide.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="23" t="inlineStr">
@@ -30975,9 +31067,9 @@
           <t>content/guides/giant-millipede-feeding-guide.mdx</t>
         </is>
       </c>
-      <c r="D63" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D63" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E63" s="13" t="inlineStr">
@@ -31000,7 +31092,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I63" s="13" t="inlineStr"/>
+      <c r="I63" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: feeding guide no longer calls a new arrival a wild-caught import; it says a newly shipped millipede, matching the cost guide (imports dried up, US stock captive-bred).</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="26" t="inlineStr">
@@ -31153,9 +31249,9 @@
           <t>content/guides/jacksonschameleon-canary-millipede-corydoras-overview.mdx</t>
         </is>
       </c>
-      <c r="D69" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D69" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E69" s="13" t="inlineStr">
@@ -31178,7 +31274,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I69" s="13" t="inlineStr"/>
+      <c r="I69" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: overview now says the secretion smells, can stain, and can sting eyes or sensitive skin; keep it from your face and wash hands, matching the handling guide.</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="29" t="inlineStr">
@@ -31236,7 +31336,11 @@
           <t>Copy the cost guide's figure into the hub line, exactly as the cost guide prints it.</t>
         </is>
       </c>
-      <c r="I71" s="13" t="inlineStr"/>
+      <c r="I71" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: prices are never changed (owner). Note only: hub route line says $85 to $145; the cost guide and hub Budget row say $80 to $165.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="30" t="inlineStr">
@@ -31254,9 +31358,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D72" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D72" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E72" s="13" t="inlineStr">
@@ -31279,7 +31383,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I72" s="13" t="inlineStr"/>
+      <c r="I72" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: hub ootheca row now says nymphs come all at once or in waves over several weeks, matching the ootheca guide.</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="30" t="inlineStr">
@@ -32436,9 +32544,9 @@
           <t>content/guides/cherry-shrimp-tank-setup-guide.mdx</t>
         </is>
       </c>
-      <c r="D110" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D110" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E110" s="13" t="inlineStr">
@@ -32461,7 +32569,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I110" s="13" t="inlineStr"/>
+      <c r="I110" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: setup guide now says adult ghost shrimp prey on cherry shrimp and their young, so keep them in separate tanks, matching the cost and stocking guides.</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="36" t="inlineStr">

</xml_diff>

<commit_message>
Consistency sweep: reptile factual rows
Fat-tail fasting and vet line, leaf-tail sourcing, heat by species and
dusting, mourning gecko humidity and handling, tokay dusting, skink size,
anole housing, iguana heat, savannah enclosure, tegu brumation and
obesity, uromastyx pollen and UVB zone, boa legality and humidity,
kingsnake, corn snake and garter snake legal rows, corn snake schedule,
garter size, hognose quarantine, red-foot permits and protein, slider
food refusal. Price and product lines noted only.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CONSISTENCY_CHECK.xlsx
+++ b/CONSISTENCY_CHECK.xlsx
@@ -785,16 +785,16 @@
         <v>8</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0.625</v>
+        <v>0.75</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
@@ -839,16 +839,16 @@
         <v>7</v>
       </c>
       <c r="D10" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="G10" s="5" t="n">
         <v>4</v>
-      </c>
-      <c r="E10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="F10" s="6" t="n">
-        <v>0.4285714285714285</v>
-      </c>
-      <c r="G10" s="5" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -866,16 +866,16 @@
         <v>9</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.5555555555555556</v>
+        <v>0.8888888888888888</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
@@ -893,16 +893,16 @@
         <v>8</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>0.5</v>
+        <v>0.625</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -920,16 +920,16 @@
         <v>9</v>
       </c>
       <c r="D13" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>0.7777777777777778</v>
+        <v>0.8888888888888888</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -974,16 +974,16 @@
         <v>8</v>
       </c>
       <c r="D15" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>0.625</v>
+        <v>0.75</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -1010,7 +1010,7 @@
         <v>0.5555555555555556</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -1118,7 +1118,7 @@
         <v>0.6666666666666666</v>
       </c>
       <c r="G20" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -1136,16 +1136,16 @@
         <v>8</v>
       </c>
       <c r="D21" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E21" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="F21" s="6" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G21" s="5" t="n">
         <v>3</v>
-      </c>
-      <c r="E21" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="F21" s="6" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="G21" s="5" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -1163,16 +1163,16 @@
         <v>8</v>
       </c>
       <c r="D22" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F22" s="6" t="n">
-        <v>0.5</v>
+        <v>0.625</v>
       </c>
       <c r="G22" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23">
@@ -1217,16 +1217,16 @@
         <v>9</v>
       </c>
       <c r="D24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="5" t="n">
         <v>2</v>
-      </c>
-      <c r="E24" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="F24" s="6" t="n">
-        <v>0.7777777777777778</v>
-      </c>
-      <c r="G24" s="5" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -1253,7 +1253,7 @@
         <v>0.5</v>
       </c>
       <c r="G25" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -1271,16 +1271,16 @@
         <v>8</v>
       </c>
       <c r="D26" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F26" s="6" t="n">
-        <v>0.5</v>
+        <v>0.625</v>
       </c>
       <c r="G26" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27">
@@ -1298,16 +1298,16 @@
         <v>9</v>
       </c>
       <c r="D27" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E27" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="F27" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" s="5" t="n">
         <v>6</v>
-      </c>
-      <c r="F27" s="6" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="G27" s="5" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="28">
@@ -1325,16 +1325,16 @@
         <v>11</v>
       </c>
       <c r="D28" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F28" s="6" t="n">
-        <v>0.6363636363636364</v>
+        <v>0.7272727272727273</v>
       </c>
       <c r="G28" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -1433,16 +1433,16 @@
         <v>9</v>
       </c>
       <c r="D32" s="5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F32" s="6" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.4444444444444444</v>
       </c>
       <c r="G32" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33">
@@ -1514,16 +1514,16 @@
         <v>9</v>
       </c>
       <c r="D35" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F35" s="6" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.7777777777777778</v>
       </c>
       <c r="G35" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36">
@@ -3616,22 +3616,22 @@
         <v>784</v>
       </c>
       <c r="D113" s="7" t="n">
-        <v>215</v>
+        <v>194</v>
       </c>
       <c r="E113" s="7" t="n">
-        <v>569</v>
+        <v>590</v>
       </c>
       <c r="F113" s="8" t="n">
-        <v>0.7257653061224489</v>
+        <v>0.7525510204081632</v>
       </c>
       <c r="G113" s="7" t="n">
-        <v>80</v>
+        <v>110</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="9" t="inlineStr">
         <is>
-          <t>Every number on this tab is a value counted from the category tabs, recounted on each update (no formulas, so it reads the same in any viewer). Conflicts overall: 324 found, 80 fixed, 244 open (25% fixed). Last recount 2026-10-05.</t>
+          <t>Every number on this tab is a value counted from the category tabs, recounted on each update (no formulas, so it reads the same in any viewer). Conflicts overall: 324 found, 110 fixed, 214 open (34% fixed). Last recount 2026-10-05.</t>
         </is>
       </c>
     </row>
@@ -5195,9 +5195,9 @@
           <t>content/guides/african-fat-tail-feeding-guide.mdx</t>
         </is>
       </c>
-      <c r="D49" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D49" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E49" s="13" t="inlineStr">
@@ -5220,7 +5220,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I49" s="13" t="inlineStr"/>
+      <c r="I49" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: feeding guide vet line now says stops eating outside the seasonal slowdown, matching its own fasting note.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="21" t="inlineStr">
@@ -5351,9 +5355,9 @@
           <t>content/guides/african-fat-tail-health-issues-guide.mdx</t>
         </is>
       </c>
-      <c r="D53" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D53" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E53" s="13" t="inlineStr">
@@ -5376,7 +5380,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I53" s="13" t="inlineStr"/>
+      <c r="I53" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: health guide vet line now excepts the normal fall and winter fast, matching the feeding guide.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="21" t="inlineStr">
@@ -5714,9 +5722,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D66" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D66" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E66" s="13" t="inlineStr">
@@ -5739,7 +5747,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I66" s="13" t="inlineStr"/>
+      <c r="I66" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: hub Buy captive-bred row now says most leaf-tails for sale are captive-bred, wild-caught ones still turn up, matching the cost guide.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="26" t="inlineStr">
@@ -5757,9 +5769,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D67" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D67" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E67" s="13" t="inlineStr">
@@ -5782,7 +5794,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I67" s="13" t="inlineStr"/>
+      <c r="I67" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: hub Temperature row and FAQ now set heat by species (about 75 to 82F by day, satanic leaf-tail no basking spot, Henkel's warm end near 92F), matching the setup guide table.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="26" t="inlineStr">
@@ -5827,9 +5843,9 @@
           <t>content/guides/leaf-tailed-gecko-enrichment-guide.mdx</t>
         </is>
       </c>
-      <c r="D69" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D69" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E69" s="13" t="inlineStr">
@@ -5852,7 +5868,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I69" s="13" t="inlineStr"/>
+      <c r="I69" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: enrichment FAQ and body now say the wild-caught animals that still turn up bring health problems, not that many are wild-caught.</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="26" t="inlineStr">
@@ -5924,9 +5944,9 @@
           <t>content/guides/leaf-tailed-gecko-health-issues-guide.mdx</t>
         </is>
       </c>
-      <c r="D72" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D72" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E72" s="13" t="inlineStr">
@@ -5949,7 +5969,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I72" s="13" t="inlineStr"/>
+      <c r="I72" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: health guide now says calcium at every other feeding, matching the feeding and setup guides.</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="26" t="inlineStr">
@@ -6104,7 +6128,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I77" s="13" t="inlineStr"/>
+      <c r="I77" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: prices are never changed (owner). Note only: heading says $10 to $25 a month; the annual table works out to about $18 to $33 a month.</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="30" t="inlineStr">
@@ -6230,9 +6258,9 @@
           <t>content/guides/mourning-gecko-tank-setup-guide.mdx</t>
         </is>
       </c>
-      <c r="D82" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D82" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E82" s="13" t="inlineStr">
@@ -6255,7 +6283,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I82" s="13" t="inlineStr"/>
+      <c r="I82" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: misting line now dries back toward 60 percent, the bottom of the 60 to 80 percent range on the same page.</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="30" t="inlineStr">
@@ -6300,9 +6332,9 @@
           <t>content/guides/leaftailedgecko-kingsnake-boxturtle-oscar-overview.mdx</t>
         </is>
       </c>
-      <c r="D84" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D84" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E84" s="13" t="inlineStr">
@@ -6325,7 +6357,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I84" s="13" t="inlineStr"/>
+      <c r="I84" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: overview FAQ and body now take the mourning gecko out of the handleable list and call it a watch-only pet, matching the handling guide.</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="30" t="inlineStr">
@@ -6343,9 +6379,9 @@
           <t>content/guides/tokay-gecko-handling-guide.mdx</t>
         </is>
       </c>
-      <c r="D85" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D85" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E85" s="13" t="inlineStr">
@@ -6368,7 +6404,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I85" s="13" t="inlineStr"/>
+      <c r="I85" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: tokay handling guide now offers the gargoyle gecko for a hand-tolerant gecko and calls the mourning gecko one to watch rather than hold.</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="31" t="inlineStr">
@@ -6444,9 +6484,9 @@
           <t>content/guides/tokay-gecko-cost-guide.mdx</t>
         </is>
       </c>
-      <c r="D88" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D88" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E88" s="13" t="inlineStr">
@@ -6469,7 +6509,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I88" s="13" t="inlineStr"/>
+      <c r="I88" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: cost guide now says juveniles dusted every feeding, adults at least twice a week, plain calcium under UVB, matching the feeding guide.</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="32" t="inlineStr">
@@ -6982,9 +7026,9 @@
           <t>content/guides/hamster-skink-whitestreefrog-pacmanfrog-overview.mdx</t>
         </is>
       </c>
-      <c r="D106" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D106" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E106" s="13" t="inlineStr">
@@ -7007,7 +7051,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I106" s="13" t="inlineStr"/>
+      <c r="I106" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: overview now says adults reach about 17 to 24 inches, matching the encyclopedia and hub.</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="35" t="inlineStr">
@@ -7328,7 +7376,11 @@
           <t>Copy the cost guide's figure into the hub line, exactly as the cost guide prints it.</t>
         </is>
       </c>
-      <c r="I117" s="13" t="inlineStr"/>
+      <c r="I117" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: prices are never changed (owner). Note only: hub route line says $390 to $470; the cost guide and hub Budget row say $350 to $520.</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="12" t="inlineStr">
@@ -7373,9 +7425,9 @@
           <t>content/guides/green-anole-enrichment-guide.mdx</t>
         </is>
       </c>
-      <c r="D119" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D119" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E119" s="13" t="inlineStr">
@@ -7398,7 +7450,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I119" s="13" t="inlineStr"/>
+      <c r="I119" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: priority list item 6 now reads One anole per enclosure, matching the same page and the setup guide.</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="12" t="inlineStr">
@@ -7634,7 +7690,11 @@
           <t>Copy the cost guide's figure into the hub line, exactly as the cost guide prints it.</t>
         </is>
       </c>
-      <c r="I127" s="13" t="inlineStr"/>
+      <c r="I127" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: prices are never changed (owner). Note only: hub route line and FAQ say about $1,041 to $1,105; the cost guide and hub Budget row say $1,032 to $1,101.</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="17" t="inlineStr">
@@ -7900,9 +7960,9 @@
           <t>content/guides/iguana-fireskink-quaker-overview.mdx</t>
         </is>
       </c>
-      <c r="D136" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D136" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E136" s="13" t="inlineStr">
@@ -7925,7 +7985,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I136" s="13" t="inlineStr"/>
+      <c r="I136" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: overview now gives air of about 75 to 88F with a cool end near 80F and a basking surface of 100 to 120F, matching the setup guide.</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="17" t="inlineStr">
@@ -8026,7 +8090,11 @@
           <t>Copy the cost guide's figure into the hub line, exactly as the cost guide prints it.</t>
         </is>
       </c>
-      <c r="I139" s="13" t="inlineStr"/>
+      <c r="I139" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: prices are never changed (owner). Note only: hub route line says $400 to $525; the cost guide and hub Budget row say $345 to $475.</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="19" t="inlineStr">
@@ -8649,7 +8717,11 @@
           <t>Copy the cost guide's figure into the hub line, exactly as the cost guide prints it.</t>
         </is>
       </c>
-      <c r="I160" s="13" t="inlineStr"/>
+      <c r="I160" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: prices are never changed (owner). Note only: hub route line says $800 to $1,500; the cost guide says $850 to $2,150 or more.</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="23" t="inlineStr">
@@ -8692,7 +8764,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I161" s="13" t="inlineStr"/>
+      <c r="I161" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: affiliate product, never sourced by Claude (owner rule). Note only: the cost guide links a 48x24x48 PVC unit as the ackie enclosure, under the setup guide minimum of 5 x 2.5 x 4 ft. Needs an owner pick.</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="23" t="inlineStr">
@@ -8940,7 +9016,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I169" s="13" t="inlineStr"/>
+      <c r="I169" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: prices are never changed (owner). Note only: overview says an $800 to $1,500 setup; the cost guide says $850 to $2,150 or more.</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="25" t="inlineStr">
@@ -9248,9 +9328,9 @@
           <t>content/guides/savannah-russiantortoise-cockatoo-stickinsect-overview.mdx</t>
         </is>
       </c>
-      <c r="D180" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D180" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E180" s="13" t="inlineStr">
@@ -9273,7 +9353,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I180" s="13" t="inlineStr"/>
+      <c r="I180" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: overview now says an adult enclosure of at least 8 by 4 by 4 feet, matching the setup guide.</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="26" t="inlineStr">
@@ -9430,9 +9514,9 @@
           <t>content/guides/argentine-tegu-feeding-guide.mdx</t>
         </is>
       </c>
-      <c r="D186" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D186" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E186" s="13" t="inlineStr">
@@ -9455,7 +9539,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I186" s="13" t="inlineStr"/>
+      <c r="I186" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: feeding guide now says brumation usually lasts about 2 to 4 months, matching the setup and handling guides and hub.</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="30" t="inlineStr">
@@ -9543,9 +9631,9 @@
           <t>content/guides/argentine-tegu-health-issues-guide.mdx</t>
         </is>
       </c>
-      <c r="D189" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D189" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E189" s="13" t="inlineStr">
@@ -9568,7 +9656,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I189" s="13" t="inlineStr"/>
+      <c r="I189" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: health FAQ and body now name the mistake as a juvenile's feeding pace carried into adulthood with fatty extras, not a rodent-heavy juvenile diet, matching the feeding guide.</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="30" t="inlineStr">
@@ -9770,7 +9862,11 @@
           <t>Copy the cost guide's figure into the hub line, exactly as the cost guide prints it.</t>
         </is>
       </c>
-      <c r="I195" s="13" t="inlineStr"/>
+      <c r="I195" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: prices are never changed (owner). Note only: hub route line says $500 to $900; the cost guide says $515 to $1,210.</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="32" t="inlineStr">
@@ -9831,9 +9927,9 @@
           <t>content/guides/uromastyx-cost-guide.mdx</t>
         </is>
       </c>
-      <c r="D197" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D197" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E197" s="13" t="inlineStr">
@@ -9856,7 +9952,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I197" s="13" t="inlineStr"/>
+      <c r="I197" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: cost guide no longer calls pollen half the diet; the topper adds floral variety on a mostly leafy greens and flowers diet, matching the feeding guide.</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="32" t="inlineStr">
@@ -9982,9 +10082,9 @@
           <t>content/guides/uromastyx-tank-setup-guide.mdx</t>
         </is>
       </c>
-      <c r="D202" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D202" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E202" s="13" t="inlineStr">
@@ -10007,7 +10107,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I202" s="13" t="inlineStr"/>
+      <c r="I202" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: setup guide now puts uromastyx in Zone 4 alongside ackie monitors only, matching the UVB guide (tegus are Zone 3).</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="32" t="inlineStr">
@@ -10205,7 +10309,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I208" s="13" t="inlineStr"/>
+      <c r="I208" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: prices are never changed (owner). Note only: line 128 says snake, setup and exam total $560 to $1,450; line 69 says $560 to $1,395 for setup and exam alone; with the snake it would be about $600 to $1,495.</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" s="34" t="inlineStr">
@@ -10454,9 +10562,9 @@
           <t>content/guides/boa-constrictor-cost-guide.mdx</t>
         </is>
       </c>
-      <c r="D218" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D218" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E218" s="13" t="inlineStr">
@@ -10479,7 +10587,11 @@
           <t>Re-read the legal guide table and its cited statutes, then make this line match the table.</t>
         </is>
       </c>
-      <c r="I218" s="13" t="inlineStr"/>
+      <c r="I218" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: cost guide now says Hawaii, New York City and a few permit states are worth checking; the New Jersey subspecies rule is gone, matching the legal guide.</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" s="36" t="inlineStr">
@@ -10686,9 +10798,9 @@
           <t>content/guides/ball-python-vs-boa-constrictor-guide.mdx</t>
         </is>
       </c>
-      <c r="D226" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D226" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E226" s="13" t="inlineStr">
@@ -10711,7 +10823,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I226" s="13" t="inlineStr"/>
+      <c r="I226" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: comparison table now gives boa humidity 60 to 70 percent, higher when shedding, matching the setup guide.</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" s="11" t="inlineStr">
@@ -10744,9 +10860,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D228" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D228" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E228" s="13" t="inlineStr">
@@ -10769,7 +10885,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I228" s="13" t="inlineStr"/>
+      <c r="I228" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: hub ban row and legal route line now add West Virginia's native ban and New Jersey's permit, matching the legal guide.</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="12" t="inlineStr">
@@ -11109,9 +11229,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D239" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D239" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E239" s="13" t="inlineStr">
@@ -11134,7 +11254,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I239" s="13" t="inlineStr"/>
+      <c r="I239" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: hub legal route line now names Georgia, West Virginia and Hawaii bans and New Jersey's nine named morphs, matching the legal guide.</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" s="17" t="inlineStr">
@@ -11177,7 +11301,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I240" s="13" t="inlineStr"/>
+      <c r="I240" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: left open. Fixing the count (adults eat every 14 to 21 days, so one or two mice a month) changes the $2 to $4 monthly mouse bill in the same sentence, a price. Needs owner OK.</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" s="17" t="inlineStr">
@@ -11281,9 +11409,9 @@
           <t>content/guides/corn-snake-feeding-guide.mdx</t>
         </is>
       </c>
-      <c r="D243" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D243" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E243" s="13" t="inlineStr">
@@ -11306,7 +11434,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I243" s="13" t="inlineStr"/>
+      <c r="I243" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: feeding FAQ now says the specialist consensus is the less frequent schedule, matching its own body.</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" s="17" t="inlineStr">
@@ -11564,9 +11696,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D252" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D252" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E252" s="13" t="inlineStr">
@@ -11589,7 +11721,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I252" s="13" t="inlineStr"/>
+      <c r="I252" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: hub Legal row now says New York has no permit path, even for a pet-store snake, matching the legal guide.</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" s="19" t="inlineStr">
@@ -11762,9 +11898,9 @@
           <t>content/guides/garter-snake-legal-guide.mdx</t>
         </is>
       </c>
-      <c r="D258" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D258" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E258" s="13" t="inlineStr">
@@ -11787,7 +11923,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I258" s="13" t="inlineStr"/>
+      <c r="I258" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: legal guide excerpt and intro now say there is no permit to get in New York, matching its own FAQ and table.</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" s="19" t="inlineStr">
@@ -11879,9 +12019,9 @@
           <t>content/guides/snake-sexing-growth-body-condition-guide.mdx</t>
         </is>
       </c>
-      <c r="D261" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D261" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E261" s="13" t="inlineStr">
@@ -11904,7 +12044,11 @@
           <t>Fix it in the shared cross-species guide; one edit there clears the same conflict for every animal it covers. Source check the figure first.</t>
         </is>
       </c>
-      <c r="I261" s="13" t="inlineStr"/>
+      <c r="I261" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: sexing and growth guide now says garter snakes usually stay around 18 to 26 inches, matching the encyclopedia and hub.</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" s="20" t="inlineStr">
@@ -12088,9 +12232,9 @@
           <t>content/guides/hognose-snake-health-issues-guide.mdx</t>
         </is>
       </c>
-      <c r="D268" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D268" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E268" s="13" t="inlineStr">
@@ -12113,7 +12257,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I268" s="13" t="inlineStr"/>
+      <c r="I268" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: health guide now quarantines a new arrival for 3 to 6 months, matching the hub and the reptile quarantine guide.</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" s="21" t="inlineStr">
@@ -13312,9 +13460,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D308" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D308" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E308" s="13" t="inlineStr">
@@ -13337,7 +13485,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I308" s="13" t="inlineStr"/>
+      <c r="I308" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: hub Legal row and route line now name four permit states, West Virginia included, matching the legal guide.</t>
+        </is>
+      </c>
     </row>
     <row r="309">
       <c r="A309" s="32" t="inlineStr">
@@ -13355,9 +13507,9 @@
           <t>content/guides/red-footed-tortoise-cost-guide.mdx</t>
         </is>
       </c>
-      <c r="D309" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D309" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E309" s="13" t="inlineStr">
@@ -13380,7 +13532,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I309" s="13" t="inlineStr"/>
+      <c r="I309" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: cost guide FAQ and body now call animal protein a small but regular share, matching the feeding guide.</t>
+        </is>
+      </c>
     </row>
     <row r="310">
       <c r="A310" s="32" t="inlineStr">
@@ -14094,7 +14250,11 @@
           <t>Copy the cost guide's figure into the hub line, exactly as the cost guide prints it.</t>
         </is>
       </c>
-      <c r="I331" s="13" t="inlineStr"/>
+      <c r="I331" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: prices are never changed (owner). Note only: hub route line says $345 to $453; the cost guide and hub Budget row say $325 to $489.</t>
+        </is>
+      </c>
     </row>
     <row r="332">
       <c r="A332" s="36" t="inlineStr">
@@ -14628,9 +14788,9 @@
           <t>content/guides/red-eared-slider-health-issues-guide.mdx</t>
         </is>
       </c>
-      <c r="D348" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D348" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E348" s="13" t="inlineStr">
@@ -14653,7 +14813,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I348" s="13" t="inlineStr"/>
+      <c r="I348" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: health FAQ and body now set the food refusal point at 2 to 3 weeks outside brumation, matching the feeding guide and hub emergency card.</t>
+        </is>
+      </c>
     </row>
     <row r="349">
       <c r="A349" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Sweep: corrections from the Fable check
Cockatoo encyclopedia card, cat kidney study wording and HCM schedule,
guinea pig vitamin C, ghost shrimp, scorpion molts, ferret wording and
legal guide dashes, tegu brumation, slider and garter wording, lines
too close to sources rewritten, chinchilla hairs back to 60 site-wide,
leftover lines on the dog toy, golden, dachshund, French bulldog,
chinchilla, sugar glider, leaf-tail, gargoyle and rat pages. Sources
combined or added on four pages so each backs its changed line.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CONSISTENCY_CHECK.xlsx
+++ b/CONSISTENCY_CHECK.xlsx
@@ -5796,7 +5796,7 @@
       </c>
       <c r="I67" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: hub Temperature row and FAQ now set heat by species (about 75 to 82F by day, satanic leaf-tail no basking spot, Henkel's warm end near 92F), matching the setup guide table.</t>
+          <t>2026-10-05: hub Temperature row and FAQ now set heat by species (about 75 to 82F by day, satanic leaf-tail no basking spot, Henkel's warm end near 92F), matching the setup guide table. Fable follow-up: setup guide description, FAQ, heading and body plus two hub descriptions now set heat by species.</t>
         </is>
       </c>
     </row>
@@ -6406,7 +6406,7 @@
       </c>
       <c r="I85" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: tokay handling guide now offers the gargoyle gecko for a hand-tolerant gecko and calls the mourning gecko one to watch rather than hold.</t>
+          <t>2026-10-05: tokay handling guide now offers the gargoyle gecko for a hand-tolerant gecko and calls the mourning gecko one to watch rather than hold. Fable follow-up: gargoyle handling guide line 91 no longer calls the mourning gecko easygoing for handling.</t>
         </is>
       </c>
     </row>
@@ -7053,7 +7053,7 @@
       </c>
       <c r="I106" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: overview now says adults reach about 17 to 24 inches, matching the encyclopedia and hub.</t>
+          <t>2026-10-05: overview now says adults reach about 17 to 24 inches, matching the encyclopedia and hub. Fable follow-up: overview now 17 to 22 in to match its added Smithsonian source (combined with the White's tree frog page).</t>
         </is>
       </c>
     </row>
@@ -7987,7 +7987,7 @@
       </c>
       <c r="I136" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: overview now gives air of about 75 to 88F with a cool end near 80F and a basking surface of 100 to 120F, matching the setup guide.</t>
+          <t>2026-10-05: overview now gives air of about 75 to 88F with a cool end near 80F and a basking surface of 100 to 120F, matching the setup guide. Fable follow-up: ReptiFiles green iguana care sheet added to the overview, combined with its fire skink entry.</t>
         </is>
       </c>
     </row>
@@ -9541,7 +9541,7 @@
       </c>
       <c r="I186" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: feeding guide now says brumation usually lasts about 2 to 4 months, matching the setup and handling guides and hub.</t>
+          <t>2026-10-05: feeding guide now says brumation usually lasts about 2 to 4 months, matching the setup and handling guides and hub. Fable follow-up: now about 2 to 4 months indoors, though some sleep 6 or 7, since the page's own ReptiFiles source says 6 to 7.</t>
         </is>
       </c>
     </row>
@@ -10825,7 +10825,7 @@
       </c>
       <c r="I226" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: comparison table now gives boa humidity 60 to 70 percent, higher when shedding, matching the setup guide.</t>
+          <t>2026-10-05: comparison table now gives boa humidity 60 to 70 percent, higher when shedding, matching the setup guide. Fable follow-up: PetMD entries combined and ReptiFiles boa humidity added to the comparison sources.</t>
         </is>
       </c>
     </row>
@@ -11436,7 +11436,7 @@
       </c>
       <c r="I243" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: feeding FAQ now says the specialist consensus is the less frequent schedule, matching its own body.</t>
+          <t>2026-10-05: feeding FAQ now says the specialist consensus is the less frequent schedule, matching its own body. Fable follow-up: wording tidied.</t>
         </is>
       </c>
     </row>
@@ -11925,7 +11925,7 @@
       </c>
       <c r="I258" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: legal guide excerpt and intro now say there is no permit to get in New York, matching its own FAQ and table.</t>
+          <t>2026-10-05: legal guide excerpt and intro now say there is no permit to get in New York, matching its own FAQ and table. Fable follow-up: excerpt reworded to one clause.</t>
         </is>
       </c>
     </row>
@@ -14815,7 +14815,7 @@
       </c>
       <c r="I348" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: health FAQ and body now set the food refusal point at 2 to 3 weeks outside brumation, matching the feeding guide and hub emergency card.</t>
+          <t>2026-10-05: health FAQ and body now set the food refusal point at 2 to 3 weeks outside brumation, matching the feeding guide and hub emergency card. Fable follow-up: FAQ and body now list the 2 to 3 week refusal as a prompt vet visit, not an emergency.</t>
         </is>
       </c>
     </row>
@@ -22083,7 +22083,7 @@
       </c>
       <c r="I24" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: hub Adult size row and the encyclopedia entry (same page, toggle) now say 12 to 27 inches and roughly 300 to 900 g across species, Goffin's and galahs light, Moluccans heavy. VCA Cockatoos General Information: 300 to 900 g, 12 to 27 in. Package figures (about 350 to 880 g) sit inside it.</t>
+          <t>2026-10-05: hub Adult size row and the encyclopedia entry (same page, toggle) now say 12 to 27 inches and roughly 300 to 900 g across species, Goffin's and galahs light, Moluccans heavy. VCA Cockatoos General Information: 300 to 900 g, 12 to 27 in. Package figures (about 350 to 880 g) sit inside it. Fable follow-up: encyclopedia card is the umbrella cockatoo only, so it now gives 18 in and 400 to 800 g for the umbrella, then the family range.</t>
         </is>
       </c>
     </row>
@@ -24627,7 +24627,7 @@
       </c>
       <c r="I5" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: enrichment guide excerpt, description, FAQ and body now say wild cavies, the guinea pig's closest relatives; no wild Cavia porcellus exists (legal guide).</t>
+          <t>2026-10-05: enrichment guide excerpt, description, FAQ and body now say wild cavies, the guinea pig's closest relatives; no wild Cavia porcellus exists (legal guide). Fable follow-up: body and FAQ reworded; they tracked the RSPCA wording too closely.</t>
         </is>
       </c>
     </row>
@@ -24674,7 +24674,7 @@
       </c>
       <c r="I6" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: feeding guide now says about one and a half times an adult's vitamin C, 30 to 40 mg a day against 20 to 25, matching the scurvy guide.</t>
+          <t>2026-10-05: feeding guide now says about one and a half times an adult's vitamin C, 30 to 40 mg a day against 20 to 25, matching the scurvy guide. Fable follow-up: one and a half times dropped; the guide now says more, with the 30 to 40 vs 20 to 25 mg figures.</t>
         </is>
       </c>
     </row>
@@ -25267,7 +25267,7 @@
       </c>
       <c r="I25" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: comparison FAQ and table now say a hamster needs a sand bath, not dust, matching the hamster setup guide.</t>
+          <t>2026-10-05: comparison FAQ and table now say a hamster needs a sand bath, not dust, matching the hamster setup guide. Fable follow-up: description now says dust bathing versus sand bathing.</t>
         </is>
       </c>
     </row>
@@ -26237,7 +26237,7 @@
       </c>
       <c r="I55" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: overview now says up to 80 hairs per follicle and a bath of up to 15 minutes two or three times a week, matching the encyclopedia and setup guide.</t>
+          <t>2026-10-05: overview now says up to 80 hairs per follicle and a bath of up to 15 minutes two or three times a week, matching the encyclopedia and setup guide. Fable follow-up: hairs per follicle back to up to 60 (Merck, ADW; the 80 figure is breeder lore), also fixed on the encyclopedia, hub fun fact and chinchilla vs guinea pig guide. Merck chinchilla pages combined into one source entry that covers the dust bath schedule.</t>
         </is>
       </c>
     </row>
@@ -26947,7 +26947,7 @@
       </c>
       <c r="I77" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: FAQ and body now present the figures as population-dependent (about 0.55 percent in Dutch studies, about a quarter of US ferrets, a repeated 70 percent estimate for 2003) instead of a range the 70 percent falls outside.</t>
+          <t>2026-10-05: FAQ and body now present the figures as population-dependent (about 0.55 percent in Dutch studies, about a quarter of US ferrets, a repeated 70 percent estimate for 2003) instead of a range the 70 percent falls outside. Fable follow-up: one Dutch study, not studies.</t>
         </is>
       </c>
     </row>
@@ -26994,7 +26994,7 @@
       </c>
       <c r="I78" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: FAQ and body now name neutering itself as the leading suspect and say age at neutering is no longer thought to matter much, matching the adrenal guide.</t>
+          <t>2026-10-05: FAQ and body now name neutering itself as the leading suspect and say age at neutering is no longer thought to matter much, matching the adrenal guide. Fable follow-up: punctuation fixed (glands. Early).</t>
         </is>
       </c>
     </row>
@@ -27041,7 +27041,7 @@
       </c>
       <c r="I79" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: lines 46 and 88 now name New Jersey and Rhode Island as the permit states, matching the table. A spaced hyphen used as a dash on line 46 removed too.</t>
+          <t>2026-10-05: lines 46 and 88 now name New Jersey and Rhode Island as the permit states, matching the table. A spaced hyphen used as a dash on line 46 removed too. Fable follow-up: spaced hyphens used as dashes removed across the legal guide.</t>
         </is>
       </c>
     </row>
@@ -28688,7 +28688,7 @@
       </c>
       <c r="I132" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: lines 94 and 66 now make labored breathing, head tilt and sudden lethargy a prompt or same-day visit, with lingering sneezing within the week, matching the FAQ and hub emergency card.</t>
+          <t>2026-10-05: lines 94 and 66 now make labored breathing, head tilt and sudden lethargy a prompt or same-day visit, with lingering sneezing within the week, matching the FAQ and hub emergency card. Fable follow-up: rat guide now treats sneezing that does not clear up as prompt, matching the hub emergency card and PDSA.</t>
         </is>
       </c>
     </row>
@@ -28898,7 +28898,7 @@
       </c>
       <c r="I138" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: cost guide FAQ now says Pennsylvania bars possession with no pet permit path, matching the legal guide.</t>
+          <t>2026-10-05: cost guide FAQ now says Pennsylvania bars possession with no pet permit path, matching the legal guide. Fable follow-up: sugar glider cost guide line 62 and hub legal row also drop effectively illegal.</t>
         </is>
       </c>
     </row>
@@ -30231,7 +30231,7 @@
       </c>
       <c r="I34" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: fun fact now says a young scorpion molts around five times and never again once mature, matching the health guide.</t>
+          <t>2026-10-05: fun fact now says a young scorpion molts around five times and never again once mature, matching the health guide. Fable follow-up: molt count now roughly five to seven, since keeper sources put this species at 6 to 7.</t>
         </is>
       </c>
     </row>
@@ -30689,7 +30689,7 @@
       </c>
       <c r="I48" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: overview now says at least 10 gallons per small or medium crab, so a pair starts at 20, matching the setup guide.</t>
+          <t>2026-10-05: overview now says at least 10 gallons per small or medium crab, so a pair starts at 20, matching the setup guide. Fable follow-up: owner chose 10 gallons per crab; Crab Street Journal added to the overview sources.</t>
         </is>
       </c>
     </row>
@@ -31024,7 +31024,7 @@
       </c>
       <c r="I57" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: fun fact now says they are not escape-proof: foot pads and hooks climb smooth glass (ADW), so a tight lid and a petroleum jelly band, matching the setup guide.</t>
+          <t>2026-10-05: fun fact now says they are not escape-proof: foot pads and hooks climb smooth glass (ADW), so a tight lid and a petroleum jelly band, matching the setup guide. Fable follow-up: climbing line reworded; it tracked ADW too closely.</t>
         </is>
       </c>
     </row>
@@ -31549,7 +31549,7 @@
       </c>
       <c r="I72" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: hub ootheca row now says nymphs come all at once or in waves over several weeks, matching the ootheca guide.</t>
+          <t>2026-10-05: hub ootheca row now says nymphs come all at once or in waves over several weeks, matching the ootheca guide. Fable follow-up: hub line reworded; it tracked the amentsoc caresheet. Ootheca guide line 83 reworded for the same reason.</t>
         </is>
       </c>
     </row>
@@ -32735,7 +32735,7 @@
       </c>
       <c r="I110" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: setup guide now says adult ghost shrimp prey on cherry shrimp and their young, so keep them in separate tanks, matching the cost and stocking guides.</t>
+          <t>2026-10-05: setup guide now says adult ghost shrimp prey on cherry shrimp and their young, so keep them in separate tanks, matching the cost and stocking guides. Fable follow-up: softened to a breeding colony keeps them apart, since a listed source allows the pairing.</t>
         </is>
       </c>
     </row>
@@ -33219,7 +33219,7 @@
       </c>
       <c r="I3" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: general cat hub diet line and FAQ now say wet food raises water intake and helps urinary health, but wet versus dry did not change who developed kidney disease, matching the kidney guide. Maine Coon diet line also drops "and kidney health".</t>
+          <t>2026-10-05: general cat hub diet line and FAQ now say wet food raises water intake and helps urinary health, but wet versus dry did not change who developed kidney disease, matching the kidney guide. Maine Coon diet line also drops "and kidney health". Fable follow-up: kidney guide line 281 called the study longitudinal; it was case-control (Greene 2014 and others), now "the studies that tested it". Ragdoll checklist now says hydration only.</t>
         </is>
       </c>
     </row>
@@ -33800,7 +33800,7 @@
       </c>
       <c r="I22" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: cardiomyopathy guide now says echo screening is standard for the four breeds, and for the Maine Coon starts at age 1, yearly until past 3, then at 5, matching the Maine Coon hub.</t>
+          <t>2026-10-05: cardiomyopathy guide now says echo screening is standard for the four breeds, and for the Maine Coon starts at age 1, yearly until past 3, then at 5, matching the Maine Coon hub. Fable follow-up: schedule credited to the Maine Coon breeding program, not called standard practice.</t>
         </is>
       </c>
     </row>
@@ -34789,7 +34789,7 @@
       </c>
       <c r="I6" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: toy guide chew row now says heavy-duty rubber that dents under a thumbnail and to skip hard nylon, matching the periodontal guide (Tufts thumbnail test).</t>
+          <t>2026-10-05: toy guide chew row now says heavy-duty rubber that dents under a thumbnail and to skip hard nylon, matching the periodontal guide (Tufts thumbnail test). Fable follow-up: toy guide line 77 also drops heavy-duty nylon.</t>
         </is>
       </c>
     </row>
@@ -35567,7 +35567,7 @@
       </c>
       <c r="I32" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: Dachshund hub housing line and IVDD FAQ rewritten to the IVDD guide: furniture and stair bans show no protective effect, more than an hour of exercise a day had lower odds, delay neutering, tested parents; ramps kept for a sore dog. Checklist and cost rows for ramps and gates left as is.</t>
+          <t>2026-10-05: Dachshund hub housing line and IVDD FAQ rewritten to the IVDD guide: furniture and stair bans show no protective effect, more than an hour of exercise a day had lower odds, delay neutering, tested parents; ramps kept for a sore dog. Checklist and cost rows for ramps and gates left as is. Fable follow-up: dachshund enrichment guide FAQ and do-not list reworded to match; hub checklist ramps and gates now framed for a sore or recovering dog; French bulldog checklist IVDD line reworded.</t>
         </is>
       </c>
     </row>
@@ -36192,7 +36192,7 @@
       </c>
       <c r="I51" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: comparison FAQ and table now say goldens shed year-round with seasonal blowouts on top, matching the golden hub.</t>
+          <t>2026-10-05: comparison FAQ and table now say goldens shed year-round with seasonal blowouts on top, matching the golden hub. Fable follow-up: comparison body line 78 now says both shed all year with seasonal blowouts.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mourning gecko humidity and corn snake mouse count
Mourning gecko: 60 to 70% ambient, peaks after misting, dry back to 50
to 60%, on the setup guide and hub. Corn snake cost guide: one to two
mice a month, about $1 to $2 at the unchanged $0.99 unit price.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CONSISTENCY_CHECK.xlsx
+++ b/CONSISTENCY_CHECK.xlsx
@@ -1280,7 +1280,7 @@
         <v>0.625</v>
       </c>
       <c r="G26" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27">
@@ -3625,13 +3625,13 @@
         <v>0.7525510204081632</v>
       </c>
       <c r="G113" s="7" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="9" t="inlineStr">
         <is>
-          <t>Every number on this tab is a value counted from the category tabs, recounted on each update (no formulas, so it reads the same in any viewer). Conflicts overall: 324 found, 110 fixed, 214 open (34% fixed). Last recount 2026-10-05.</t>
+          <t>Every number on this tab is a value counted from the category tabs, recounted on each update (no formulas, so it reads the same in any viewer). Conflicts overall: 324 found, 111 fixed, 213 open (34% fixed). Last recount 2026-10-05.</t>
         </is>
       </c>
     </row>
@@ -6285,7 +6285,7 @@
       </c>
       <c r="I82" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: misting line now dries back toward 60 percent, the bottom of the 60 to 80 percent range on the same page.</t>
+          <t>2026-10-05: misting line now dries back toward 60 percent, the bottom of the 60 to 80 percent range on the same page. Owner and Fable follow-up: FAQ, line 71, line 95 and the hub humidity row now say 60 to 70% ambient, peaks to 80 to 90% after misting, dry back to 50 to 60% (ReptiFiles, Reptiles Magazine).</t>
         </is>
       </c>
     </row>
@@ -11276,9 +11276,9 @@
           <t>content/guides/corn-snake-cost-guide.mdx</t>
         </is>
       </c>
-      <c r="D240" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D240" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E240" s="13" t="inlineStr">
@@ -11303,7 +11303,7 @@
       </c>
       <c r="I240" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: left open. Fixing the count (adults eat every 14 to 21 days, so one or two mice a month) changes the $2 to $4 monthly mouse bill in the same sentence, a price. Needs owner OK.</t>
+          <t>2026-10-05: owner OK. Cost guide now says every two to three weeks, one to two mice a month, about $1 to $2 a month at the unchanged $0.99 unit price; table label 1 to 2 mice, $10 to $20 kept. Note: RodentPro list price is $1.09; $0.99 was a sale price.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Consistency sweep: bird and amphibian minor rows
Grey powder down, conure and zebra finch lifespans, Quaker lifespan
and outage figure, zebra finch pellet dish, axolotl bottle cooling and
legal description, White's tree frog rich feeders, tiger salamander
dusting and wild-caught stock. Prices and the D3 product line noted;
cockatoo maturity noted in FIX_PACKAGES.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CONSISTENCY_CHECK.xlsx
+++ b/CONSISTENCY_CHECK.xlsx
@@ -1541,16 +1541,16 @@
         <v>10</v>
       </c>
       <c r="D36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="F36" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G36" s="5" t="n">
         <v>3</v>
-      </c>
-      <c r="E36" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="F36" s="6" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="G36" s="5" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -1568,16 +1568,16 @@
         <v>8</v>
       </c>
       <c r="D37" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F37" s="6" t="n">
-        <v>0.625</v>
+        <v>0.75</v>
       </c>
       <c r="G37" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38">
@@ -1649,16 +1649,16 @@
         <v>10</v>
       </c>
       <c r="D40" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F40" s="6" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="G40" s="5" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="41">
@@ -2135,16 +2135,16 @@
         <v>11</v>
       </c>
       <c r="D58" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E58" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F58" s="6" t="n">
-        <v>0.8181818181818182</v>
+        <v>0.9090909090909091</v>
       </c>
       <c r="G58" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="59">
@@ -2189,16 +2189,16 @@
         <v>9</v>
       </c>
       <c r="D60" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E60" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="F60" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="E60" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="F60" s="6" t="n">
-        <v>0.8888888888888888</v>
-      </c>
       <c r="G60" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="61">
@@ -2243,16 +2243,16 @@
         <v>8</v>
       </c>
       <c r="D62" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E62" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="F62" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="E62" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="F62" s="6" t="n">
-        <v>0.875</v>
-      </c>
       <c r="G62" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63">
@@ -2297,16 +2297,16 @@
         <v>8</v>
       </c>
       <c r="D64" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E64" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="F64" s="6" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G64" s="5" t="n">
         <v>2</v>
-      </c>
-      <c r="E64" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="F64" s="6" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G64" s="5" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="65">
@@ -2324,16 +2324,16 @@
         <v>8</v>
       </c>
       <c r="D65" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E65" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F65" s="6" t="n">
-        <v>0.625</v>
+        <v>0.875</v>
       </c>
       <c r="G65" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="66">
@@ -3616,22 +3616,22 @@
         <v>784</v>
       </c>
       <c r="D113" s="7" t="n">
-        <v>194</v>
+        <v>182</v>
       </c>
       <c r="E113" s="7" t="n">
-        <v>590</v>
+        <v>602</v>
       </c>
       <c r="F113" s="8" t="n">
-        <v>0.7525510204081632</v>
+        <v>0.7678571428571429</v>
       </c>
       <c r="G113" s="7" t="n">
-        <v>111</v>
+        <v>124</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="9" t="inlineStr">
         <is>
-          <t>Every number on this tab is a value counted from the category tabs, recounted on each update (no formulas, so it reads the same in any viewer). Conflicts overall: 324 found, 111 fixed, 213 open (34% fixed). Last recount 2026-10-05.</t>
+          <t>Every number on this tab is a value counted from the category tabs, recounted on each update (no formulas, so it reads the same in any viewer). Conflicts overall: 324 found, 124 fixed, 200 open (38% fixed). Last recount 2026-10-05.</t>
         </is>
       </c>
     </row>
@@ -15047,9 +15047,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D3" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D3" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E3" s="13" t="inlineStr">
@@ -15072,7 +15072,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I3" s="13" t="inlineStr"/>
+      <c r="I3" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: hub heat-wave row now says to watch a thermometer, since even a bottle can cool faster than about 1F an hour (cooling guide, Merck).</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
@@ -15225,9 +15229,9 @@
           <t>content/guides/axolotl-legal-guide.mdx</t>
         </is>
       </c>
-      <c r="D9" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E9" s="13" t="inlineStr">
@@ -15250,7 +15254,11 @@
           <t>Re-read the legal guide table and its cited statutes, then make this line match the table.</t>
         </is>
       </c>
-      <c r="I9" s="13" t="inlineStr"/>
+      <c r="I9" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: legal guide description now lists all seven, matching its FAQ and the hub.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="12" t="inlineStr">
@@ -15322,9 +15330,9 @@
           <t>content/guides/aquarium-power-outage-and-transport-guide.mdx</t>
         </is>
       </c>
-      <c r="D12" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E12" s="13" t="inlineStr">
@@ -15347,7 +15355,11 @@
           <t>Fix it in the shared cross-species guide; one edit there clears the same conflict for every animal it covers. Source check the figure first.</t>
         </is>
       </c>
-      <c r="I12" s="13" t="inlineStr"/>
+      <c r="I12" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: outage guide no longer calls a frozen bottle gradual and predictable; it says gentler than ice but able to exceed about 1F an hour, so watch a thermometer, matching the cooling guide.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="16" t="inlineStr">
@@ -15405,7 +15417,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I14" s="13" t="inlineStr"/>
+      <c r="I14" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: affiliate product wording, left as a note. The buy list line is a catalog covers match for Repashy Calcium Plus (contains D3); the feeding guide says D3 depends on UVB. Needs an owner product call.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="17" t="inlineStr">
@@ -15450,7 +15466,7 @@
       </c>
       <c r="I15" s="13" t="inlineStr">
         <is>
-          <t>Tied to the FIX_PACKAGES Repashy gear note.</t>
+          <t>2026-10-05: affiliate product wording, left as a note, same as the hub buy list row: the linked Repashy Calcium Plus contains D3.</t>
         </is>
       </c>
     </row>
@@ -15497,9 +15513,9 @@
           <t>content/guides/whites-tree-frog-feeding-guide.mdx</t>
         </is>
       </c>
-      <c r="D17" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D17" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E17" s="13" t="inlineStr">
@@ -15522,7 +15538,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I17" s="13" t="inlineStr"/>
+      <c r="I17" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: FAQ and line 56 now put the earthworm and pinkie at once a month at most, matching line 66.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="17" t="inlineStr">
@@ -15966,7 +15986,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I33" s="13" t="inlineStr"/>
+      <c r="I33" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: prices are never changed (owner). Note only: lines 64 and 81 say $100 to $225; the six table rows sum to $113 to $210.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="21" t="inlineStr">
@@ -16282,9 +16306,9 @@
           <t>content/guides/tiger-salamander-feeding-guide.mdx</t>
         </is>
       </c>
-      <c r="D44" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D44" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E44" s="13" t="inlineStr">
@@ -16307,7 +16331,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I44" s="13" t="inlineStr"/>
+      <c r="I44" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: tiger salamander feeding guide no longer says the pacman guide runs the same schedule; it shares the idea on its own schedule.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="23" t="inlineStr">
@@ -16507,9 +16535,9 @@
           <t>content/guides/tiger-salamander-vs-axolotl-guide.mdx</t>
         </is>
       </c>
-      <c r="D51" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D51" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E51" s="13" t="inlineStr">
@@ -16532,7 +16560,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I51" s="13" t="inlineStr"/>
+      <c r="I51" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: comparison now says axolotls are captive-bred while many tiger salamanders are still wild-caught, matching the health guide and hub.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:I51"/>
@@ -22184,9 +22216,9 @@
           <t>content/guides/cockatoo-handling-guide.mdx</t>
         </is>
       </c>
-      <c r="D28" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D28" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E28" s="13" t="inlineStr">
@@ -22211,7 +22243,7 @@
       </c>
       <c r="I28" s="13" t="inlineStr">
         <is>
-          <t>Source check needed to decide which is right.</t>
+          <t>2026-10-05: no site change needed. The handling guide matches its listed PetMD source (about 5 to 7 years); the package is the outlier and is noted in FIX_PACKAGES.md.</t>
         </is>
       </c>
     </row>
@@ -22366,7 +22398,7 @@
       </c>
       <c r="I33" s="13" t="inlineStr">
         <is>
-          <t>Logged in FIX_PACKAGES.md. Source check needed.</t>
+          <t>2026-10-05: care package, never edited from the sweep. Noted in FIX_PACKAGES.md under Cockatoo: match the site and PetMD, about 5 to 7 years.</t>
         </is>
       </c>
     </row>
@@ -22922,9 +22954,9 @@
           <t>content/guides/african-grey-parrot-vs-cockatoo-guide.mdx</t>
         </is>
       </c>
-      <c r="D54" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D54" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E54" s="13" t="inlineStr">
@@ -22947,7 +22979,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I54" s="13" t="inlineStr"/>
+      <c r="I54" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: comparison table and body now say greys shed heavy powder down too, matching the grey setup guide.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="25" t="inlineStr">
@@ -23521,9 +23557,9 @@
           <t>content/guides/choosing-a-pet-bird-guide.mdx</t>
         </is>
       </c>
-      <c r="D75" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D75" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E75" s="13" t="inlineStr">
@@ -23546,7 +23582,11 @@
           <t>Fix it in the shared cross-species guide; one edit there clears the same conflict for every animal it covers. Source check the figure first.</t>
         </is>
       </c>
-      <c r="I75" s="13" t="inlineStr"/>
+      <c r="I75" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: choosing guide now says 20 to 25 years or more, matching the conure cost guide.</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="31" t="inlineStr">
@@ -23862,7 +23902,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I87" s="13" t="inlineStr"/>
+      <c r="I87" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: prices are never changed (owner). Note only: body says an annual exam runs $85 and up; the table and hub say $78 to $115.</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="34" t="inlineStr">
@@ -23880,9 +23924,9 @@
           <t>content/guides/quaker-parakeet-cost-guide.mdx</t>
         </is>
       </c>
-      <c r="D88" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D88" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E88" s="13" t="inlineStr">
@@ -23905,7 +23949,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I88" s="13" t="inlineStr"/>
+      <c r="I88" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: cost guide FAQ and body now say longer than most small birds but short of the largest parrots.</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="34" t="inlineStr">
@@ -23977,9 +24025,9 @@
           <t>content/guides/quaker-parakeet-handling-guide.mdx</t>
         </is>
       </c>
-      <c r="D91" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D91" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E91" s="13" t="inlineStr">
@@ -24002,7 +24050,11 @@
           <t>Re-read the legal guide table and its cited statutes, then make this line match the table.</t>
         </is>
       </c>
-      <c r="I91" s="13" t="inlineStr"/>
+      <c r="I91" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: handling guide now gives the recorded figure, 498 outages in five months of 2001, projecting to about 1,000 a year, matching the legal guide.</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="34" t="inlineStr">
@@ -24217,9 +24269,9 @@
           <t>content/guides/zebra-finch-enrichment-guide.mdx</t>
         </is>
       </c>
-      <c r="D99" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D99" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E99" s="13" t="inlineStr">
@@ -24242,7 +24294,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I99" s="13" t="inlineStr"/>
+      <c r="I99" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: enrichment priority list now keeps a pellet dish that never runs empty under the scattered food, matching the feeding guide.</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="36" t="inlineStr">
@@ -24395,9 +24451,9 @@
           <t>content/guides/choosing-a-pet-bird-guide.mdx</t>
         </is>
       </c>
-      <c r="D105" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D105" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E105" s="13" t="inlineStr">
@@ -24420,7 +24476,11 @@
           <t>Fix it in the shared cross-species guide; one edit there clears the same conflict for every animal it covers. Source check the figure first.</t>
         </is>
       </c>
-      <c r="I105" s="13" t="inlineStr"/>
+      <c r="I105" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: choosing guide now says 5 to 7 years, matching the zebra finch cost guide.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:I105"/>

</xml_diff>

<commit_message>
Consistency sweep: cat and dog minor rows
Cat dental figures, Bengal folklore, second cat and state law lines,
Maine Coon companionship and OFA wording, Persian PKD and PRA figures,
Ragdoll combing and kidney lines, Scottish Fold PKD; dog neutering
timing, small breed lifespans, gram scale portions, medium breed list,
Border Collie exercise, Bulldog bowl, dachshund and French Bulldog back
advice, BOAS study, GSD bloat, Golden brushing and uveitis, Husky heat
and exercise table.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CONSISTENCY_CHECK.xlsx
+++ b/CONSISTENCY_CHECK.xlsx
@@ -2972,16 +2972,16 @@
         <v>1</v>
       </c>
       <c r="D89" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E89" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E89" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="F89" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G89" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="90">
@@ -3026,16 +3026,16 @@
         <v>4</v>
       </c>
       <c r="D91" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E91" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F91" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G91" s="5" t="n">
         <v>3</v>
-      </c>
-      <c r="E91" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F91" s="6" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="G91" s="5" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="92">
@@ -3080,16 +3080,16 @@
         <v>4</v>
       </c>
       <c r="D93" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E93" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F93" s="6" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="G93" s="5" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="94">
@@ -3107,16 +3107,16 @@
         <v>2</v>
       </c>
       <c r="D94" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E94" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F94" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="E94" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F94" s="6" t="n">
-        <v>0.5</v>
-      </c>
       <c r="G94" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="95">
@@ -3134,16 +3134,16 @@
         <v>1</v>
       </c>
       <c r="D95" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E95" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E95" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="F95" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G95" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="96">
@@ -3161,16 +3161,16 @@
         <v>1</v>
       </c>
       <c r="D96" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E96" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E96" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="F96" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G96" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="97">
@@ -3242,16 +3242,16 @@
         <v>2</v>
       </c>
       <c r="D99" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E99" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F99" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="E99" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F99" s="6" t="n">
-        <v>0.5</v>
-      </c>
       <c r="G99" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="100">
@@ -3269,16 +3269,16 @@
         <v>1</v>
       </c>
       <c r="D100" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E100" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E100" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="F100" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G100" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="101">
@@ -3296,16 +3296,16 @@
         <v>1</v>
       </c>
       <c r="D101" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E101" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E101" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="F101" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G101" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="102">
@@ -3377,16 +3377,16 @@
         <v>2</v>
       </c>
       <c r="D104" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E104" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F104" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="E104" s="4" t="n">
+      <c r="G104" s="5" t="n">
         <v>1</v>
-      </c>
-      <c r="F104" s="6" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G104" s="5" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="105">
@@ -3404,16 +3404,16 @@
         <v>2</v>
       </c>
       <c r="D105" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E105" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F105" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="E105" s="4" t="n">
+      <c r="G105" s="5" t="n">
         <v>1</v>
-      </c>
-      <c r="F105" s="6" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G105" s="5" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="106">
@@ -3431,16 +3431,16 @@
         <v>2</v>
       </c>
       <c r="D106" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E106" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F106" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="E106" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F106" s="6" t="n">
-        <v>0.5</v>
-      </c>
       <c r="G106" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="107">
@@ -3458,16 +3458,16 @@
         <v>4</v>
       </c>
       <c r="D107" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E107" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F107" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G107" s="5" t="n">
         <v>3</v>
-      </c>
-      <c r="E107" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F107" s="6" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="G107" s="5" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="108">
@@ -3485,16 +3485,16 @@
         <v>2</v>
       </c>
       <c r="D108" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E108" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F108" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="E108" s="4" t="n">
+      <c r="G108" s="5" t="n">
         <v>1</v>
-      </c>
-      <c r="F108" s="6" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G108" s="5" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="109">
@@ -3512,16 +3512,16 @@
         <v>3</v>
       </c>
       <c r="D109" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E109" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F109" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="E109" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="F109" s="6" t="n">
-        <v>0.6666666666666666</v>
-      </c>
       <c r="G109" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="110">
@@ -3593,16 +3593,16 @@
         <v>3</v>
       </c>
       <c r="D112" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E112" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F112" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G112" s="5" t="n">
         <v>2</v>
-      </c>
-      <c r="E112" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F112" s="6" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="G112" s="5" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="113">
@@ -3616,22 +3616,22 @@
         <v>784</v>
       </c>
       <c r="D113" s="7" t="n">
-        <v>182</v>
+        <v>160</v>
       </c>
       <c r="E113" s="7" t="n">
-        <v>602</v>
+        <v>624</v>
       </c>
       <c r="F113" s="8" t="n">
-        <v>0.7678571428571429</v>
+        <v>0.7959183673469388</v>
       </c>
       <c r="G113" s="7" t="n">
-        <v>124</v>
+        <v>152</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="9" t="inlineStr">
         <is>
-          <t>Every number on this tab is a value counted from the category tabs, recounted on each update (no formulas, so it reads the same in any viewer). Conflicts overall: 324 found, 124 fixed, 200 open (38% fixed). Last recount 2026-10-05.</t>
+          <t>Every number on this tab is a value counted from the category tabs, recounted on each update (no formulas, so it reads the same in any viewer). Conflicts overall: 324 found, 152 fixed, 172 open (47% fixed). Last recount 2026-10-05.</t>
         </is>
       </c>
     </row>
@@ -33299,9 +33299,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D4" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">
@@ -33324,7 +33324,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I4" s="13" t="inlineStr"/>
+      <c r="I4" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: cat hub now says up to 70% by age 2 and about 85% past age 6, matching the periodontal guide (Merck, Cornell).</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
@@ -33453,9 +33457,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D10" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E10" s="13" t="inlineStr">
@@ -33478,7 +33482,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I10" s="13" t="inlineStr"/>
+      <c r="I10" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: Bengal FAQ drops the faucet and door-handle claims the hub itself calls folklore.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="19" t="inlineStr">
@@ -33496,9 +33504,9 @@
           <t>content/guides/bengal-cat-enrichment-guide.mdx</t>
         </is>
       </c>
-      <c r="D11" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D11" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E11" s="13" t="inlineStr">
@@ -33521,7 +33529,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I11" s="13" t="inlineStr"/>
+      <c r="I11" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: enrichment guide now says a second cat can help a great deal but is not an automatic fix, matching the hub.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="19" t="inlineStr">
@@ -33593,9 +33605,9 @@
           <t>content/guides/why-cats-need-mental-enrichment-and-how-boredom-can-break-them.mdx</t>
         </is>
       </c>
-      <c r="D14" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E14" s="13" t="inlineStr">
@@ -33618,7 +33630,11 @@
           <t>Fix it in the shared cross-species guide; one edit there clears the same conflict for every animal it covers. Source check the figure first.</t>
         </is>
       </c>
-      <c r="I14" s="13" t="inlineStr"/>
+      <c r="I14" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: boredom guide now calls the Bengal the breed most often named in state law, alongside the Savannah and Chausie, matching the legal guide.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="20" t="inlineStr">
@@ -33720,9 +33736,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D19" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D19" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E19" s="13" t="inlineStr">
@@ -33745,7 +33761,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I19" s="13" t="inlineStr"/>
+      <c r="I19" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: already fixed with Cats row 3 (diet line now says supports hydration only).</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="23" t="inlineStr">
@@ -33763,9 +33783,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D20" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D20" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E20" s="13" t="inlineStr">
@@ -33788,7 +33808,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I20" s="13" t="inlineStr"/>
+      <c r="I20" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: checklist now reads daily interaction, fairly independent, matching the CFA quote on the same hub.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="23" t="inlineStr">
@@ -33927,9 +33951,9 @@
           <t>content/guides/hip-and-elbow-dysplasia-guide.mdx</t>
         </is>
       </c>
-      <c r="D24" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D24" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E24" s="13" t="inlineStr">
@@ -33952,7 +33976,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I24" s="13" t="inlineStr"/>
+      <c r="I24" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: no number was wrong. The study holds 2,708 Maine Coons, 2,548 with hip results (24.9 percent of 2,548); the line now says with hip results.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="25" t="inlineStr">
@@ -34032,9 +34060,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D27" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D27" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E27" s="13" t="inlineStr">
@@ -34057,7 +34085,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I27" s="13" t="inlineStr"/>
+      <c r="I27" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: health line now says 29 percent of UK test submissions in 2005 to 10 percent by 2009, then 0.7 percent of 3,235 under care, matching the funFact, FAQ and kidney guide. The unsourced 2 percent in 2016 is gone.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="26" t="inlineStr">
@@ -34075,9 +34107,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D28" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D28" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E28" s="13" t="inlineStr">
@@ -34100,7 +34132,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I28" s="13" t="inlineStr"/>
+      <c r="I28" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: health line now says blind by about 16 to 17 weeks, often soon after going home, matching the eye disease guide.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="26" t="inlineStr">
@@ -34254,9 +34290,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D33" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D33" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E33" s="13" t="inlineStr">
@@ -34279,7 +34315,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I33" s="13" t="inlineStr"/>
+      <c r="I33" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: housing line now says combing once or twice a week, matching the checklist, FAQ and CFA.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="30" t="inlineStr">
@@ -34297,9 +34337,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D34" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D34" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E34" s="13" t="inlineStr">
@@ -34322,7 +34362,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I34" s="13" t="inlineStr"/>
+      <c r="I34" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: diet line now says wet food has not been shown to prevent kidney disease; checklist fixed earlier.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="30" t="inlineStr">
@@ -34382,9 +34426,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D37" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D37" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E37" s="13" t="inlineStr">
@@ -34407,7 +34451,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I37" s="13" t="inlineStr"/>
+      <c r="I37" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: diet line now says wet food cannot prevent PKD, since cysts are inherited and present from birth, matching the kidney guide.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="32" t="inlineStr">
@@ -34752,9 +34800,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D4" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">
@@ -34777,7 +34825,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I4" s="13" t="inlineStr"/>
+      <c r="I4" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: general hub now says spay or neuter prevents some cancers and litters, but timing matters in some large and long-backed breeds, matching the Rottweiler hub and IVDD guide. Owner allows dog changes.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
@@ -34884,9 +34936,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D8" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E8" s="13" t="inlineStr">
@@ -34909,7 +34961,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I8" s="13" t="inlineStr"/>
+      <c r="I8" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: funFact now says Chihuahuas 14 to 16 and Dachshunds 12 to 16, matching the encyclopedia.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="17" t="inlineStr">
@@ -35016,9 +35072,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D12" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E12" s="13" t="inlineStr">
@@ -35041,7 +35097,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I12" s="13" t="inlineStr"/>
+      <c r="I12" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: medium hub diet, checklist and FAQ now say weigh meals on a kitchen scale, matching the obesity guide.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="19" t="inlineStr">
@@ -35059,9 +35119,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D13" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E13" s="13" t="inlineStr">
@@ -35084,7 +35144,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I13" s="13" t="inlineStr"/>
+      <c r="I13" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: medium hub health line and FAQ now keep Border Collies and note Labs and Goldens are large breeds.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="19" t="inlineStr">
@@ -35403,9 +35467,9 @@
           <t>content/guides/border-collie-enrichment-guide.mdx</t>
         </is>
       </c>
-      <c r="D25" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D25" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E25" s="13" t="inlineStr">
@@ -35428,7 +35492,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I25" s="13" t="inlineStr"/>
+      <c r="I25" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: enrichment guide now says exercise is needed in quantity, more than two hours a day per the hub, and the puzzle line sits on top of it.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="26" t="inlineStr">
@@ -35488,9 +35556,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D28" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D28" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E28" s="13" t="inlineStr">
@@ -35513,7 +35581,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I28" s="13" t="inlineStr"/>
+      <c r="I28" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: Bulldog hub cost row, diet and checklist now say slow-feed bowl without elevated, price kept (owner allows dog changes), matching the bloat guide.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="30" t="inlineStr">
@@ -35647,9 +35719,9 @@
           <t>content/guides/dachshund-enrichment-guide.mdx</t>
         </is>
       </c>
-      <c r="D33" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D33" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E33" s="13" t="inlineStr">
@@ -35672,7 +35744,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I33" s="13" t="inlineStr"/>
+      <c r="I33" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: dachshund enrichment line 97 drops stair gating; lines 49 and 137 fixed earlier.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="32" t="inlineStr">
@@ -35690,9 +35766,9 @@
           <t>content/guides/dachshund-enrichment-guide.mdx</t>
         </is>
       </c>
-      <c r="D34" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D34" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E34" s="13" t="inlineStr">
@@ -35715,7 +35791,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I34" s="13" t="inlineStr"/>
+      <c r="I34" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: enrichment line 113 now says more than an hour of walking a day for a fit dog, matching the IVDD guide.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="32" t="inlineStr">
@@ -35775,9 +35855,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D37" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D37" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E37" s="13" t="inlineStr">
@@ -35800,7 +35880,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I37" s="13" t="inlineStr"/>
+      <c r="I37" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: French Bulldog hub FAQ now says stair and furniture restriction has not been shown to prevent disc disease; checklist fixed earlier.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="34" t="inlineStr">
@@ -35818,9 +35902,9 @@
           <t>content/guides/french-bulldog-enrichment-guide.mdx</t>
         </is>
       </c>
-      <c r="D38" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D38" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E38" s="13" t="inlineStr">
@@ -35843,7 +35927,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I38" s="13" t="inlineStr"/>
+      <c r="I38" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: French Bulldog enrichment guide lines 51 and 109 drop stair discouragement as prevention.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="34" t="inlineStr">
@@ -35915,9 +36003,9 @@
           <t>content/guides/brachycephalic-airway-syndrome-boas-guide.mdx</t>
         </is>
       </c>
-      <c r="D41" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D41" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E41" s="13" t="inlineStr">
@@ -35940,7 +36028,11 @@
           <t>Fix it in the shared cross-species guide; one edit there clears the same conflict for every animal it covers. Source check the figure first.</t>
         </is>
       </c>
-      <c r="I41" s="13" t="inlineStr"/>
+      <c r="I41" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: BOAS guide now names the VetCompass comparison of 2,781 French Bulldogs with 21,850 other dogs drawn from 905,544, matching the hub.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="35" t="inlineStr">
@@ -35973,9 +36065,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D43" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D43" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E43" s="13" t="inlineStr">
@@ -35998,7 +36090,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I43" s="13" t="inlineStr"/>
+      <c r="I43" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: German Shepherd checklist now says a high-risk bloat breed, matching the bloat guide.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="36" t="inlineStr">
@@ -36085,9 +36181,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D47" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D47" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E47" s="13" t="inlineStr">
@@ -36110,7 +36206,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I47" s="13" t="inlineStr"/>
+      <c r="I47" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: Golden checklist now says brushing three to four times a week, matching the hub.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="12" t="inlineStr">
@@ -36128,9 +36228,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D48" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D48" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E48" s="13" t="inlineStr">
@@ -36153,7 +36253,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I48" s="13" t="inlineStr"/>
+      <c r="I48" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: Golden hub health line and FAQ now say about one in ten to nearly one in four, matching the eye disease guide.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="12" t="inlineStr">
@@ -36526,9 +36630,9 @@
           <t>content/guides/siberian-husky-enrichment-guide.mdx</t>
         </is>
       </c>
-      <c r="D62" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D62" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E62" s="13" t="inlineStr">
@@ -36551,7 +36655,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I62" s="13" t="inlineStr"/>
+      <c r="I62" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: Husky enrichment FAQ and body now say heat needs planning but UK data did not find higher odds than Labradors, matching the hub.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="21" t="inlineStr">
@@ -36596,9 +36704,9 @@
           <t>content/guides/why-your-dog-needs-daily-exercise.mdx</t>
         </is>
       </c>
-      <c r="D64" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D64" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E64" s="13" t="inlineStr">
@@ -36621,7 +36729,11 @@
           <t>Fix it in the shared cross-species guide; one edit there clears the same conflict for every animal it covers. Source check the figure first.</t>
         </is>
       </c>
-      <c r="I64" s="13" t="inlineStr"/>
+      <c r="I64" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: exercise table now says 1 to 2+ hours for working breeds, covering the Husky hub 60 to 120 minutes and the Border Collie hub.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:I64"/>

</xml_diff>

<commit_message>
Consistency sweep: fish minor rows
Zebra danio group size, angelfish temperature and guppy line, ich table
angelfish ceiling and guppy salt, bristlenose overview, cardinal tetra
school and tank, guppy broods, koi lifespan claims, oscar growth,
livebearer stocking and lifespans, swordtail acclimation and lid gaps.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CONSISTENCY_CHECK.xlsx
+++ b/CONSISTENCY_CHECK.xlsx
@@ -17258,7 +17258,11 @@
           <t>Copy the cost guide's figure into the hub line, exactly as the cost guide prints it.</t>
         </is>
       </c>
-      <c r="I24" s="13" t="inlineStr"/>
+      <c r="I24" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: prices are never changed (owner). Note only: hub route line says $130 to $260; the cost guide and hub Budget row say $135 to $280.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="19" t="inlineStr">
@@ -17554,9 +17558,9 @@
           <t>content/guides/zebra-danio-enrichment-guide.mdx</t>
         </is>
       </c>
-      <c r="D35" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D35" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E35" s="13" t="inlineStr">
@@ -17579,7 +17583,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I35" s="13" t="inlineStr"/>
+      <c r="I35" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: enrichment guide now says at least six, eight to ten better, matching the handling guide.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="21" t="inlineStr">
@@ -17597,9 +17605,9 @@
           <t>content/guides/zebra-danio-feeding-guide.mdx</t>
         </is>
       </c>
-      <c r="D36" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D36" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E36" s="13" t="inlineStr">
@@ -17622,7 +17630,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I36" s="13" t="inlineStr"/>
+      <c r="I36" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: no change needed: lines 44 and 74 are about avoiding spawning (no fine-leaved plants if you do not want fry), line 80 and the setup guide are about general planting. Read in context they do not clash.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="21" t="inlineStr">
@@ -18026,9 +18038,9 @@
           <t>content/guides/ackie-milksnake-mhc-angelfish-overview.mdx</t>
         </is>
       </c>
-      <c r="D51" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D51" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E51" s="13" t="inlineStr">
@@ -18051,7 +18063,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I51" s="13" t="inlineStr"/>
+      <c r="I51" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: overview now says comfortable at 78 to 82F, matching the setup guide.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="23" t="inlineStr">
@@ -18069,9 +18085,9 @@
           <t>content/guides/ackie-milksnake-mhc-angelfish-overview.mdx</t>
         </is>
       </c>
-      <c r="D52" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D52" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E52" s="13" t="inlineStr">
@@ -18094,7 +18110,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I52" s="13" t="inlineStr"/>
+      <c r="I52" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: overview now says a guppy becomes prey once the angel passes about 3 inches, matching the handling guide.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="23" t="inlineStr">
@@ -18112,9 +18132,9 @@
           <t>content/guides/aquarium-ich-treatment-guide.mdx</t>
         </is>
       </c>
-      <c r="D53" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D53" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E53" s="13" t="inlineStr">
@@ -18137,7 +18157,11 @@
           <t>Fix it in the shared cross-species guide; one edit there clears the same conflict for every animal it covers. Source check the figure first.</t>
         </is>
       </c>
-      <c r="I53" s="13" t="inlineStr"/>
+      <c r="I53" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: ich table angelfish ceiling now says comfortable to 82F, tolerates to 86F, so the Yes matches the page rule and the setup guide.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="25" t="inlineStr">
@@ -18453,9 +18477,9 @@
           <t>content/guides/zebra-danio-bristlenose-pleco-discus-cardinal-tetra-overview.mdx</t>
         </is>
       </c>
-      <c r="D64" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D64" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E64" s="13" t="inlineStr">
@@ -18478,7 +18502,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I64" s="13" t="inlineStr"/>
+      <c r="I64" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: overview excerpt and body no longer call the bristlenose a low-maintenance algae eater, matching the feeding guide.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="29" t="inlineStr">
@@ -18538,9 +18566,9 @@
           <t>content/guides/cardinal-tetra-cost-guide.mdx</t>
         </is>
       </c>
-      <c r="D67" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D67" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E67" s="13" t="inlineStr">
@@ -18563,7 +18591,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I67" s="13" t="inlineStr"/>
+      <c r="I67" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: cost guide now says a 20-gallon long for the school of 10. Prices unchanged.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="30" t="inlineStr">
@@ -18635,9 +18667,9 @@
           <t>content/guides/cardinal-tetra-handling-guide.mdx</t>
         </is>
       </c>
-      <c r="D70" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D70" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E70" s="13" t="inlineStr">
@@ -18660,7 +18692,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I70" s="13" t="inlineStr"/>
+      <c r="I70" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: handling guide now says ten is where natural schooling settles in, matching its own minimum of 10.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="30" t="inlineStr">
@@ -18705,9 +18741,9 @@
           <t>content/guides/cardinal-tetra-tank-setup-guide.mdx</t>
         </is>
       </c>
-      <c r="D72" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D72" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E72" s="13" t="inlineStr">
@@ -18730,7 +18766,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I72" s="13" t="inlineStr"/>
+      <c r="I72" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: setup guide FAQ and body now plan on a 20-gallon long for a school of 10; the 10-gallon link stays, now described as too small.</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="30" t="inlineStr">
@@ -19696,9 +19736,9 @@
           <t>content/guides/aquarium-ich-treatment-guide.mdx</t>
         </is>
       </c>
-      <c r="D105" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D105" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E105" s="13" t="inlineStr">
@@ -19721,7 +19761,11 @@
           <t>Fix it in the shared cross-species guide; one edit there clears the same conflict for every animal it covers. Source check the figure first.</t>
         </is>
       </c>
-      <c r="I105" s="13" t="inlineStr"/>
+      <c r="I105" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: ich guide salt line now names mollies and platies and sends guppies to medication, matching the guppy health guide.</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="36" t="inlineStr">
@@ -19739,9 +19783,9 @@
           <t>content/guides/sulcata-hedgehog-lovebird-guppy-overview.mdx</t>
         </is>
       </c>
-      <c r="D106" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D106" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E106" s="13" t="inlineStr">
@@ -19764,7 +19808,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I106" s="13" t="inlineStr"/>
+      <c r="I106" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: overview keeps the study figure and adds that well-fed females in warm water average about 25 and reach 50, matching the handling guide.</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="11" t="inlineStr">
@@ -19844,9 +19892,9 @@
           <t>content/guides/koi-cost-guide.mdx</t>
         </is>
       </c>
-      <c r="D109" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D109" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E109" s="13" t="inlineStr">
@@ -19869,7 +19917,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I109" s="13" t="inlineStr"/>
+      <c r="I109" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: already fixed earlier (koi cost guide pump line).</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="12" t="inlineStr">
@@ -20069,9 +20121,9 @@
           <t>content/guides/koi-vs-goldfish-guide.mdx</t>
         </is>
       </c>
-      <c r="D116" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D116" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E116" s="13" t="inlineStr">
@@ -20094,7 +20146,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I116" s="13" t="inlineStr"/>
+      <c r="I116" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: comparison FAQ and table now call 100-year koi claims unverified, matching the cost guide.</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="16" t="inlineStr">
@@ -20390,9 +20446,9 @@
           <t>encyclopedia (src/lib/data/encyclopedia/fish.js)</t>
         </is>
       </c>
-      <c r="D127" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D127" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E127" s="13" t="inlineStr">
@@ -20415,7 +20471,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I127" s="13" t="inlineStr"/>
+      <c r="I127" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: no change needed: the encyclopedia field is wild lifespan (hobby sources give about 8 years in the wild), the cost guide figures are captive. Not a conflict.</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="18" t="inlineStr">
@@ -20630,9 +20690,9 @@
           <t>content/guides/oscar-fish-tank-setup-guide.mdx</t>
         </is>
       </c>
-      <c r="D135" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D135" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E135" s="13" t="inlineStr">
@@ -20655,7 +20715,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I135" s="13" t="inlineStr"/>
+      <c r="I135" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: setup guide body and FAQ, cost guide and hub now say about two-thirds of adult size in the first year, matching the feeding and handling guides.</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="19" t="inlineStr">
@@ -20931,9 +20995,9 @@
           <t>content/guides/aquarium-stocking-and-tankmates-guide.mdx</t>
         </is>
       </c>
-      <c r="D146" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D146" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E146" s="13" t="inlineStr">
@@ -20956,7 +21020,11 @@
           <t>Fix it in the shared cross-species guide; one edit there clears the same conflict for every animal it covers. Source check the figure first.</t>
         </is>
       </c>
-      <c r="I146" s="13" t="inlineStr"/>
+      <c r="I146" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: stocking table now gives 10 gallons for about five platies, 20 for mollies or a swordtail trio, 29 or more for a swordtail group.</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="21" t="inlineStr">
@@ -20974,9 +21042,9 @@
           <t>content/guides/platy-swordtail-molly-overview.mdx</t>
         </is>
       </c>
-      <c r="D147" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D147" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E147" s="13" t="inlineStr">
@@ -20999,7 +21067,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I147" s="13" t="inlineStr"/>
+      <c r="I147" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: overview now gives platies 2 to 4 years and mollies and swordtails 3 to 5, matching the cost guides.</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="22" t="inlineStr">
@@ -21140,9 +21212,9 @@
           <t>content/guides/swordtail-handling-guide.mdx</t>
         </is>
       </c>
-      <c r="D153" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D153" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E153" s="13" t="inlineStr">
@@ -21165,7 +21237,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I153" s="13" t="inlineStr"/>
+      <c r="I153" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: handling FAQ and hub now drip only for soft or acidic water, matching line 58.</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="23" t="inlineStr">
@@ -21257,9 +21333,9 @@
           <t>content/guides/swordtail-tank-setup-guide.mdx</t>
         </is>
       </c>
-      <c r="D156" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D156" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E156" s="13" t="inlineStr">
@@ -21282,7 +21358,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I156" s="13" t="inlineStr"/>
+      <c r="I156" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: FAQ now says gaps of well under an inch, matching the FunFact and hub.</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="23" t="inlineStr">
@@ -21374,9 +21454,9 @@
           <t>content/guides/aquarium-stocking-and-tankmates-guide.mdx</t>
         </is>
       </c>
-      <c r="D159" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D159" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E159" s="13" t="inlineStr">
@@ -21399,7 +21479,11 @@
           <t>Fix it in the shared cross-species guide; one edit there clears the same conflict for every animal it covers. Source check the figure first.</t>
         </is>
       </c>
-      <c r="I159" s="13" t="inlineStr"/>
+      <c r="I159" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: same stocking table fix as row 146.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:I159"/>

</xml_diff>

<commit_message>
Consistency sweep: small mammal minor rows
Guinea pig alfalfa, hamster bedding conversion, grip and bedding lines,
rabbit vet timing, chinchilla size, handling, companionship and heat,
degu legal count, ferret tumor and NYC dates, flying squirrel pairs,
gerbil size, pellets and humidity, hedgehog lifespan, mouse temperature,
rat mammary tissue, sugar glider room temperature. Prices and one buy
list covers line noted.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CONSISTENCY_CHECK.xlsx
+++ b/CONSISTENCY_CHECK.xlsx
@@ -24838,9 +24838,9 @@
           <t>content/guides/guinea-pig-feeding-guide.mdx</t>
         </is>
       </c>
-      <c r="D7" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E7" s="13" t="inlineStr">
@@ -24863,7 +24863,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I7" s="13" t="inlineStr"/>
+      <c r="I7" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: feeding FAQ and line 62 now keep alfalfa for growing, pregnant and nursing animals, an ill adult only on vet advice, matching the setup and health guides.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
@@ -25267,9 +25271,9 @@
           <t>content/guides/hamster-tank-setup-guide.mdx</t>
         </is>
       </c>
-      <c r="D22" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D22" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E22" s="13" t="inlineStr">
@@ -25292,7 +25296,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I22" s="13" t="inlineStr"/>
+      <c r="I22" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: conversion now reads about 16 to 31 inches (40 to 80 cm).</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="17" t="inlineStr">
@@ -25431,9 +25439,9 @@
           <t>content/guides/chinchilla-vs-hamster-guide.mdx</t>
         </is>
       </c>
-      <c r="D26" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D26" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E26" s="13" t="inlineStr">
@@ -25456,7 +25464,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I26" s="13" t="inlineStr"/>
+      <c r="I26" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: comparison table and body now say scooped up in two cupped hands, matching the hamster handling guide.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="17" t="inlineStr">
@@ -25474,9 +25486,9 @@
           <t>content/guides/gerbil-vs-hamster-guide.mdx</t>
         </is>
       </c>
-      <c r="D27" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D27" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E27" s="13" t="inlineStr">
@@ -25499,7 +25511,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I27" s="13" t="inlineStr"/>
+      <c r="I27" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: comparison now says deep bedding is a welfare requirement for hamsters too, matching the setup guide.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="18" t="inlineStr">
@@ -25802,9 +25818,9 @@
           <t>content/guides/rabbit-budgie-overview.mdx</t>
         </is>
       </c>
-      <c r="D39" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D39" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E39" s="13" t="inlineStr">
@@ -25827,7 +25843,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I39" s="13" t="inlineStr"/>
+      <c r="I39" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: overview now says call the vet at 8 hours and treat 12 hours as an emergency, matching the health guide.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="20" t="inlineStr">
@@ -25885,7 +25905,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I41" s="13" t="inlineStr"/>
+      <c r="I41" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: affiliate covers text, left as a note. The buy list line "24x24x36 inch multi-level metal cage" is a catalog covers match for the Critter Nation link; the setup guide calls 24x24x36 the smallest accepted. Needs an owner call on the buy list wording.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="21" t="inlineStr">
@@ -25903,9 +25927,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D42" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D42" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E42" s="13" t="inlineStr">
@@ -25928,7 +25952,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I42" s="13" t="inlineStr"/>
+      <c r="I42" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: hub and encyclopedia adult size now say about 0.9 to 1.5 lbs (400 to 700 g), matching the health guide.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="21" t="inlineStr">
@@ -25971,7 +25999,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I43" s="13" t="inlineStr"/>
+      <c r="I43" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: prices are never changed (owner). Note only: line 76 says $455 to $1,225; the table sums to about $345 to $420 low and $1,420 high.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="21" t="inlineStr">
@@ -26178,9 +26210,9 @@
           <t>content/guides/chinchilla-vs-guinea-pig-guide.mdx</t>
         </is>
       </c>
-      <c r="D51" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D51" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E51" s="13" t="inlineStr">
@@ -26203,7 +26235,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I51" s="13" t="inlineStr"/>
+      <c r="I51" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: comparison FAQ, table and body now say chinchillas tame with daily handling, matching the handling guide.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="21" t="inlineStr">
@@ -26221,9 +26257,9 @@
           <t>content/guides/chinchilla-vs-guinea-pig-guide.mdx</t>
         </is>
       </c>
-      <c r="D52" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D52" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E52" s="13" t="inlineStr">
@@ -26246,7 +26282,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I52" s="13" t="inlineStr"/>
+      <c r="I52" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: comparison FAQ, table and body now say chinchillas usually do better with a same-sex companion, a single one workable with daily attention, matching the enrichment and handling guides.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="21" t="inlineStr">
@@ -26264,9 +26304,9 @@
           <t>content/guides/chinchilla-vs-guinea-pig-guide.mdx</t>
         </is>
       </c>
-      <c r="D53" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D53" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E53" s="13" t="inlineStr">
@@ -26289,7 +26329,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I53" s="13" t="inlineStr"/>
+      <c r="I53" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: comparison FAQ and table now say comfortable to about 68F and at risk from about 80F, matching the setup guide; a spaced hyphen in the table removed too.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="21" t="inlineStr">
@@ -26488,7 +26532,11 @@
           <t>Copy the cost guide's figure into the hub line, exactly as the cost guide prints it.</t>
         </is>
       </c>
-      <c r="I58" s="13" t="inlineStr"/>
+      <c r="I58" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: prices are never changed (owner). Note only: hub route line says $375 to $520; the cost guide and Budget row say $395 to $525.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="23" t="inlineStr">
@@ -26506,9 +26554,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D59" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D59" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E59" s="13" t="inlineStr">
@@ -26531,7 +26579,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I59" s="13" t="inlineStr"/>
+      <c r="I59" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: hub legal row and route now say restricted or unsettled in eighteen, banned in eight, matching the legal guide.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="23" t="inlineStr">
@@ -26854,9 +26906,9 @@
           <t>content/guides/ferret-adrenal-disease-guide.mdx</t>
         </is>
       </c>
-      <c r="D71" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D71" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E71" s="13" t="inlineStr">
@@ -26879,7 +26931,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I71" s="13" t="inlineStr"/>
+      <c r="I71" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: adrenal guide now says one of the two most common ferret tumors, alongside insulinoma, matching the health guide.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="26" t="inlineStr">
@@ -26922,7 +26978,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I72" s="13" t="inlineStr"/>
+      <c r="I72" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: prices are never changed (owner). Note only: headline and FAQ say the ferret costs $75 to $400 while rescue adoption is priced at $50 to $150.</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="26" t="inlineStr">
@@ -26965,7 +27025,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I73" s="13" t="inlineStr"/>
+      <c r="I73" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: prices are never changed (owner). Note only: the annual items total $350 to $630, about $29 to $53 a month, while the headline says $50 to $60 a month.</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="26" t="inlineStr">
@@ -27205,9 +27269,9 @@
           <t>content/guides/ferret-legal-guide.mdx</t>
         </is>
       </c>
-      <c r="D80" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D80" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E80" s="13" t="inlineStr">
@@ -27230,7 +27294,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I80" s="13" t="inlineStr"/>
+      <c r="I80" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: legal table now says restricted since 1959, banned under the current rule since 1999, matching line 78.</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="26" t="inlineStr">
@@ -27445,9 +27513,9 @@
           <t>content/guides/flying-squirrel-handling-guide.mdx</t>
         </is>
       </c>
-      <c r="D88" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D88" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E88" s="13" t="inlineStr">
@@ -27470,7 +27538,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I88" s="13" t="inlineStr"/>
+      <c r="I88" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: handling guide now pairs same-sex squirrels and notes neutering is not routine, matching the cost guide and hub.</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="30" t="inlineStr">
@@ -27636,7 +27708,11 @@
           <t>Copy the cost guide's figure into the hub line, exactly as the cost guide prints it.</t>
         </is>
       </c>
-      <c r="I94" s="13" t="inlineStr"/>
+      <c r="I94" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: prices are never changed (owner). Note only: hub route line says $150 to $350; the cost guide and Budget row say $145 to $385.</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="32" t="inlineStr">
@@ -27654,9 +27730,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D95" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D95" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E95" s="13" t="inlineStr">
@@ -27679,7 +27755,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I95" s="13" t="inlineStr"/>
+      <c r="I95" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: hub adult size now about 2.5 to 4.6 oz (70 to 130 g), matching the cost guide.</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="32" t="inlineStr">
@@ -27722,7 +27802,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I96" s="13" t="inlineStr"/>
+      <c r="I96" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: prices are never changed (owner). Note only: FAQ prices a gerbil at $10 to $20 against the table's $5 to $50, and the setup total against the table sum; the "Hamster pellets" budget line is a cost item, left for the owner with the prices.</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="32" t="inlineStr">
@@ -27949,9 +28033,9 @@
           <t>content/guides/gerbil-vs-guinea-pig-guide.mdx</t>
         </is>
       </c>
-      <c r="D104" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D104" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E104" s="13" t="inlineStr">
@@ -27974,7 +28058,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I104" s="13" t="inlineStr"/>
+      <c r="I104" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: comparison FAQ, table and body now ask for a gerbil pellet at 18 to 20% protein, matching the gerbil feeding guide.</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="32" t="inlineStr">
@@ -27992,9 +28080,9 @@
           <t>content/guides/small-mammal-temperature-heat-stress-guide.mdx</t>
         </is>
       </c>
-      <c r="D105" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D105" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E105" s="13" t="inlineStr">
@@ -28017,7 +28105,11 @@
           <t>Fix it in the shared cross-species guide; one edit there clears the same conflict for every animal it covers. Source check the figure first.</t>
         </is>
       </c>
-      <c r="I105" s="13" t="inlineStr"/>
+      <c r="I105" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: heat stress guide body and table now say humidity below about 40%, a sore nose from about 50%, matching the gerbil setup guide.</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="33" t="inlineStr">
@@ -28293,9 +28385,9 @@
           <t>content/guides/sulcata-hedgehog-lovebird-guppy-overview.mdx</t>
         </is>
       </c>
-      <c r="D116" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D116" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E116" s="13" t="inlineStr">
@@ -28318,7 +28410,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I116" s="13" t="inlineStr"/>
+      <c r="I116" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: overview now says typically 3 to 6 years, some 8 or more, matching the hedgehog cost guide.</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="35" t="inlineStr">
@@ -28376,7 +28472,11 @@
           <t>Copy the cost guide's figure into the hub line, exactly as the cost guide prints it.</t>
         </is>
       </c>
-      <c r="I118" s="13" t="inlineStr"/>
+      <c r="I118" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: prices are never changed (owner). Note only: hub route line says $100 to $210; the cost guide and Budget row say $100 to $225.</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="36" t="inlineStr">
@@ -28569,9 +28669,9 @@
           <t>content/guides/mouse-tank-setup-guide.mdx</t>
         </is>
       </c>
-      <c r="D124" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D124" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E124" s="13" t="inlineStr">
@@ -28594,7 +28694,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I124" s="13" t="inlineStr"/>
+      <c r="I124" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: setup guide now calls 64 to 79F the usual room range and says mice prefer about 79 to 84F, so deep nesting material matters, matching the enrichment guide.</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="36" t="inlineStr">
@@ -28681,9 +28785,9 @@
           <t>content/guides/rat-cost-guide.mdx</t>
         </is>
       </c>
-      <c r="D128" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D128" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E128" s="13" t="inlineStr">
@@ -28706,7 +28810,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I128" s="13" t="inlineStr"/>
+      <c r="I128" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: mammary line now says chin to the base of the tail, matching the health guide. The "around $200" cage line is a price, left as is.</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="12" t="inlineStr">
@@ -29116,9 +29224,9 @@
           <t>content/guides/sugar-glider-handling-guide.mdx</t>
         </is>
       </c>
-      <c r="D141" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D141" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E141" s="13" t="inlineStr">
@@ -29141,7 +29249,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I141" s="13" t="inlineStr"/>
+      <c r="I141" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: handling guide and hub bonding row now say about 75F or warmer, matching the setup guide.</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="17" t="inlineStr">

</xml_diff>

<commit_message>
Consistency sweep: invertebrate minor rows
Tarantula prey rule, jumping spider prey size, scorpion grouping,
portions, outage heat and lifespan, hissing cockroach dishes, hiss,
food refusal and handling lines, millipede imports and tankmates,
mantis prey and lifespan, stick insect water, humidity and substrate,
shrimp group sizes, heater, kinship, feeding, drip rate, ghost shrimp
wild diet and an unsourced hub row replaced.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CONSISTENCY_CHECK.xlsx
+++ b/CONSISTENCY_CHECK.xlsx
@@ -1757,16 +1757,16 @@
         <v>7</v>
       </c>
       <c r="D44" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="F44" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G44" s="5" t="n">
         <v>2</v>
-      </c>
-      <c r="E44" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="F44" s="6" t="n">
-        <v>0.7142857142857143</v>
-      </c>
-      <c r="G44" s="5" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="45">
@@ -1784,16 +1784,16 @@
         <v>9</v>
       </c>
       <c r="D45" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E45" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F45" s="6" t="n">
-        <v>0.7777777777777778</v>
+        <v>1</v>
       </c>
       <c r="G45" s="5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="46">
@@ -1811,16 +1811,16 @@
         <v>9</v>
       </c>
       <c r="D46" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E46" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="F46" s="6" t="n">
+        <v>0.8888888888888888</v>
+      </c>
+      <c r="G46" s="5" t="n">
         <v>2</v>
-      </c>
-      <c r="E46" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="F46" s="6" t="n">
-        <v>0.7777777777777778</v>
-      </c>
-      <c r="G46" s="5" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="47">
@@ -1838,16 +1838,16 @@
         <v>7</v>
       </c>
       <c r="D47" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="F47" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G47" s="5" t="n">
         <v>3</v>
-      </c>
-      <c r="E47" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="F47" s="6" t="n">
-        <v>0.5714285714285714</v>
-      </c>
-      <c r="G47" s="5" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="48">
@@ -1919,16 +1919,16 @@
         <v>9</v>
       </c>
       <c r="D50" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>0.7777777777777778</v>
+        <v>1</v>
       </c>
       <c r="G50" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="51">
@@ -1946,16 +1946,16 @@
         <v>8</v>
       </c>
       <c r="D51" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F51" s="6" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="G51" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="52">
@@ -1973,16 +1973,16 @@
         <v>9</v>
       </c>
       <c r="D52" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E52" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="F52" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="E52" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="F52" s="6" t="n">
-        <v>0.8888888888888888</v>
-      </c>
       <c r="G52" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53">
@@ -2000,16 +2000,16 @@
         <v>7</v>
       </c>
       <c r="D53" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E53" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F53" s="6" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.8571428571428571</v>
       </c>
       <c r="G53" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54">
@@ -2027,16 +2027,16 @@
         <v>9</v>
       </c>
       <c r="D54" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E54" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="F54" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G54" s="5" t="n">
         <v>2</v>
-      </c>
-      <c r="E54" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="F54" s="6" t="n">
-        <v>0.7777777777777778</v>
-      </c>
-      <c r="G54" s="5" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="55">
@@ -2054,16 +2054,16 @@
         <v>9</v>
       </c>
       <c r="D55" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E55" s="4" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F55" s="6" t="n">
-        <v>0.6666666666666666</v>
+        <v>1</v>
       </c>
       <c r="G55" s="5" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="56">
@@ -2351,16 +2351,16 @@
         <v>10</v>
       </c>
       <c r="D66" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E66" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F66" s="6" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="G66" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="67">
@@ -2378,16 +2378,16 @@
         <v>11</v>
       </c>
       <c r="D67" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E67" s="4" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F67" s="6" t="n">
-        <v>0.7272727272727273</v>
+        <v>1</v>
       </c>
       <c r="G67" s="5" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="68">
@@ -2405,16 +2405,16 @@
         <v>11</v>
       </c>
       <c r="D68" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E68" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="F68" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="E68" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="F68" s="6" t="n">
-        <v>0.9090909090909091</v>
-      </c>
       <c r="G68" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="69">
@@ -2432,16 +2432,16 @@
         <v>12</v>
       </c>
       <c r="D69" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E69" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F69" s="6" t="n">
-        <v>0.75</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="G69" s="5" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="70">
@@ -2468,7 +2468,7 @@
         <v>0.8888888888888888</v>
       </c>
       <c r="G70" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="71">
@@ -2486,16 +2486,16 @@
         <v>9</v>
       </c>
       <c r="D71" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E71" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F71" s="6" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.8888888888888888</v>
       </c>
       <c r="G71" s="5" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="72">
@@ -2513,16 +2513,16 @@
         <v>8</v>
       </c>
       <c r="D72" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E72" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="F72" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="E72" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="F72" s="6" t="n">
-        <v>0.875</v>
-      </c>
       <c r="G72" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="73">
@@ -2540,16 +2540,16 @@
         <v>10</v>
       </c>
       <c r="D73" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E73" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="F73" s="6" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G73" s="5" t="n">
         <v>4</v>
-      </c>
-      <c r="E73" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="F73" s="6" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="G73" s="5" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="74">
@@ -2567,16 +2567,16 @@
         <v>9</v>
       </c>
       <c r="D74" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E74" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="F74" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="E74" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="F74" s="6" t="n">
-        <v>0.8888888888888888</v>
-      </c>
       <c r="G74" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="75">
@@ -2594,16 +2594,16 @@
         <v>7</v>
       </c>
       <c r="D75" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E75" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F75" s="6" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.8571428571428571</v>
       </c>
       <c r="G75" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="76">
@@ -2621,16 +2621,16 @@
         <v>7</v>
       </c>
       <c r="D76" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E76" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="F76" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="E76" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="F76" s="6" t="n">
-        <v>0.8571428571428571</v>
-      </c>
       <c r="G76" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="77">
@@ -2648,16 +2648,16 @@
         <v>8</v>
       </c>
       <c r="D77" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E77" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F77" s="6" t="n">
-        <v>0.75</v>
+        <v>0.875</v>
       </c>
       <c r="G77" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="78">
@@ -2675,16 +2675,16 @@
         <v>9</v>
       </c>
       <c r="D78" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E78" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F78" s="6" t="n">
-        <v>0.7777777777777778</v>
+        <v>0.8888888888888888</v>
       </c>
       <c r="G78" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="79">
@@ -2702,16 +2702,16 @@
         <v>8</v>
       </c>
       <c r="D79" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E79" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F79" s="6" t="n">
-        <v>0.75</v>
+        <v>0.875</v>
       </c>
       <c r="G79" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="80">
@@ -2729,16 +2729,16 @@
         <v>12</v>
       </c>
       <c r="D80" s="5" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E80" s="4" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F80" s="6" t="n">
-        <v>0.6666666666666666</v>
+        <v>1</v>
       </c>
       <c r="G80" s="5" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="81">
@@ -2783,16 +2783,16 @@
         <v>6</v>
       </c>
       <c r="D82" s="5" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E82" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F82" s="6" t="n">
-        <v>0.3333333333333333</v>
+        <v>1</v>
       </c>
       <c r="G82" s="5" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="83">
@@ -2810,16 +2810,16 @@
         <v>9</v>
       </c>
       <c r="D83" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E83" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F83" s="6" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.8888888888888888</v>
       </c>
       <c r="G83" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="84">
@@ -2837,16 +2837,16 @@
         <v>9</v>
       </c>
       <c r="D84" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E84" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="F84" s="6" t="n">
+        <v>0.8888888888888888</v>
+      </c>
+      <c r="G84" s="5" t="n">
         <v>3</v>
-      </c>
-      <c r="E84" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="F84" s="6" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="G84" s="5" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="85">
@@ -2864,16 +2864,16 @@
         <v>8</v>
       </c>
       <c r="D85" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E85" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="F85" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G85" s="5" t="n">
         <v>3</v>
-      </c>
-      <c r="E85" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="F85" s="6" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="G85" s="5" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="86">
@@ -2891,16 +2891,16 @@
         <v>8</v>
       </c>
       <c r="D86" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E86" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F86" s="6" t="n">
-        <v>0.75</v>
+        <v>0.875</v>
       </c>
       <c r="G86" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="87">
@@ -2918,16 +2918,16 @@
         <v>7</v>
       </c>
       <c r="D87" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E87" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F87" s="6" t="n">
-        <v>0.5714285714285714</v>
+        <v>1</v>
       </c>
       <c r="G87" s="5" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="88">
@@ -2945,16 +2945,16 @@
         <v>8</v>
       </c>
       <c r="D88" s="5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E88" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F88" s="6" t="n">
-        <v>0.5</v>
+        <v>0.875</v>
       </c>
       <c r="G88" s="5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="89">
@@ -3616,22 +3616,22 @@
         <v>784</v>
       </c>
       <c r="D113" s="7" t="n">
-        <v>160</v>
+        <v>102</v>
       </c>
       <c r="E113" s="7" t="n">
-        <v>624</v>
+        <v>682</v>
       </c>
       <c r="F113" s="8" t="n">
-        <v>0.7959183673469388</v>
+        <v>0.8698979591836735</v>
       </c>
       <c r="G113" s="7" t="n">
-        <v>152</v>
+        <v>218</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="9" t="inlineStr">
         <is>
-          <t>Every number on this tab is a value counted from the category tabs, recounted on each update (no formulas, so it reads the same in any viewer). Conflicts overall: 324 found, 152 fixed, 172 open (47% fixed). Last recount 2026-10-05.</t>
+          <t>Every number on this tab is a value counted from the category tabs, recounted on each update (no formulas, so it reads the same in any viewer). Conflicts overall: 324 found, 218 fixed, 106 open (67% fixed). Last recount 2026-10-05.</t>
         </is>
       </c>
     </row>
@@ -29676,9 +29676,9 @@
           <t>content/guides/tarantula-tank-setup-guide.mdx</t>
         </is>
       </c>
-      <c r="D10" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E10" s="13" t="inlineStr">
@@ -29701,7 +29701,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I10" s="13" t="inlineStr"/>
+      <c r="I10" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: line 110 now reads as the sling tightening of the 24-hour rule, so the two lines agree.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -29746,7 +29750,7 @@
       </c>
       <c r="I11" s="13" t="inlineStr">
         <is>
-          <t>Logged in FIX_PACKAGES.md.</t>
+          <t>2026-10-05: care package, never edited from the sweep. The site now frames overnight as the sling rule inside the 24-hour rule; the package can copy that framing on its next edit.</t>
         </is>
       </c>
     </row>
@@ -29900,7 +29904,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I15" s="13" t="inlineStr"/>
+      <c r="I15" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: affiliate covers text, left as a note. The buy list line is a catalog covers match for the enclosure link; the setup guide says about 8 inches tall for an adult. Needs an owner call on the wording.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="17" t="inlineStr">
@@ -29945,9 +29953,9 @@
           <t>content/guides/jumping-spider-enrichment-guide.mdx</t>
         </is>
       </c>
-      <c r="D17" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D17" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E17" s="13" t="inlineStr">
@@ -29970,7 +29978,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I17" s="13" t="inlineStr"/>
+      <c r="I17" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: enrichment guide now says no more than about three quarters of body length, matching the feeding guide and its Bugs in Cyberspace source (the abdomen rule was retired earlier).</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="17" t="inlineStr">
@@ -30239,9 +30251,9 @@
           <t>content/guides/emperor-scorpion-enrichment-guide.mdx</t>
         </is>
       </c>
-      <c r="D27" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D27" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E27" s="13" t="inlineStr">
@@ -30264,7 +30276,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I27" s="13" t="inlineStr"/>
+      <c r="I27" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: do-not list now says start with a single scorpion and graduate to a group, matching line 95.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="19" t="inlineStr">
@@ -30282,9 +30298,9 @@
           <t>content/guides/emperor-scorpion-feeding-guide.mdx</t>
         </is>
       </c>
-      <c r="D28" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D28" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E28" s="13" t="inlineStr">
@@ -30307,7 +30323,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I28" s="13" t="inlineStr"/>
+      <c r="I28" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: feeding guide now gives an adult portion of 2 to 3 insects, matching its own schedule, FAQ, hub and cost guide.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="19" t="inlineStr">
@@ -30507,9 +30527,9 @@
           <t>content/guides/invertebrate-emergency-travel-shipping-guide.mdx</t>
         </is>
       </c>
-      <c r="D35" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D35" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E35" s="13" t="inlineStr">
@@ -30532,7 +30552,11 @@
           <t>Fix it in the shared cross-species guide; one edit there clears the same conflict for every animal it covers. Source check the figure first.</t>
         </is>
       </c>
-      <c r="I35" s="13" t="inlineStr"/>
+      <c r="I35" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: travel guide body and table now treat emperor scorpions as warm-kept, 75 to 85F with a side heat mat, so an outage matters, matching the setup guide.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="19" t="inlineStr">
@@ -30597,9 +30621,9 @@
           <t>content/guides/koi-conure-slider-scorpion-overview.mdx</t>
         </is>
       </c>
-      <c r="D37" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D37" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E37" s="13" t="inlineStr">
@@ -30622,7 +30646,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I37" s="13" t="inlineStr"/>
+      <c r="I37" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: overview now says about 5 to 8 years, matching the cost guide.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="20" t="inlineStr">
@@ -31034,9 +31062,9 @@
           <t>content/guides/hissing-cockroach-enrichment-guide.mdx</t>
         </is>
       </c>
-      <c r="D52" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D52" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E52" s="13" t="inlineStr">
@@ -31059,7 +31087,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I52" s="13" t="inlineStr"/>
+      <c r="I52" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: enrichment guide now scatters some food on top of the usual dishes, matching the feeding guide.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="23" t="inlineStr">
@@ -31077,9 +31109,9 @@
           <t>content/guides/hissing-cockroach-feeding-guide.mdx</t>
         </is>
       </c>
-      <c r="D53" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D53" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E53" s="13" t="inlineStr">
@@ -31102,7 +31134,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I53" s="13" t="inlineStr"/>
+      <c r="I53" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: feeding FAQ and concern list drop failure to hiss, matching the handling guide (the hiss habituates).</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="23" t="inlineStr">
@@ -31120,9 +31156,9 @@
           <t>content/guides/hissing-cockroach-handling-guide.mdx</t>
         </is>
       </c>
-      <c r="D54" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D54" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E54" s="13" t="inlineStr">
@@ -31145,7 +31181,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I54" s="13" t="inlineStr"/>
+      <c r="I54" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: handling line now allows that a new arrival may skip meals while settling, matching the feeding guide.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="23" t="inlineStr">
@@ -31163,9 +31203,9 @@
           <t>content/guides/hissing-cockroach-handling-guide.mdx</t>
         </is>
       </c>
-      <c r="D55" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D55" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E55" s="13" t="inlineStr">
@@ -31188,7 +31228,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I55" s="13" t="inlineStr"/>
+      <c r="I55" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: handling line 94 now says a display pet first that takes gentle handling well, matching line 50.</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="23" t="inlineStr">
@@ -31300,9 +31344,9 @@
           <t>content/guides/ackie-milksnake-mhc-angelfish-overview.mdx</t>
         </is>
       </c>
-      <c r="D58" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D58" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E58" s="13" t="inlineStr">
@@ -31325,7 +31369,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I58" s="13" t="inlineStr"/>
+      <c r="I58" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: overview FAQ now says the hiss is an alarm and, between males, a territorial warning, matching its own line 73 and the handling guide.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="25" t="inlineStr">
@@ -31383,7 +31431,11 @@
           <t>Copy the cost guide's figure into the hub line, exactly as the cost guide prints it.</t>
         </is>
       </c>
-      <c r="I60" s="13" t="inlineStr"/>
+      <c r="I60" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: prices are never changed (owner). Note only: hub Budget row and route say setup $75 to $150; the cost guide says $75 to $190.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="26" t="inlineStr">
@@ -31401,9 +31453,9 @@
           <t>content/guides/giant-millipede-cost-guide.mdx</t>
         </is>
       </c>
-      <c r="D61" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D61" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E61" s="13" t="inlineStr">
@@ -31426,7 +31478,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I61" s="13" t="inlineStr"/>
+      <c r="I61" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: cost guide now says imports have all but dried up, not that the route is closed, matching its own FAQ and the legal guide.</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="26" t="inlineStr">
@@ -31444,9 +31500,9 @@
           <t>content/guides/giant-millipede-enrichment-guide.mdx</t>
         </is>
       </c>
-      <c r="D62" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D62" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E62" s="13" t="inlineStr">
@@ -31469,7 +31525,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I62" s="13" t="inlineStr"/>
+      <c r="I62" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: enrichment FAQ and body now discourage mixing millipede species but welcome isopods and springtails, matching the setup guide.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="26" t="inlineStr">
@@ -31852,9 +31912,9 @@
           <t>content/guides/praying-mantis-enrichment-guide.mdx</t>
         </is>
       </c>
-      <c r="D74" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D74" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E74" s="13" t="inlineStr">
@@ -31877,7 +31937,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I74" s="13" t="inlineStr"/>
+      <c r="I74" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: enrichment line now releases some prey but warns that released prey can hide and a mantis go hungry, matching the feeding guide.</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="30" t="inlineStr">
@@ -32057,9 +32121,9 @@
           <t>content/guides/10-surprising-praying-mantis-facts.mdx</t>
         </is>
       </c>
-      <c r="D81" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D81" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E81" s="13" t="inlineStr">
@@ -32082,7 +32146,11 @@
           <t>Correct the fun fact to match the deep dive; never renumber or remove a fact id.</t>
         </is>
       </c>
-      <c r="I81" s="13" t="inlineStr"/>
+      <c r="I81" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: fun fact now says about 6 to 12 months, a year and a half at the outside, matching the cost guide.</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="31" t="inlineStr">
@@ -32115,9 +32183,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D83" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D83" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E83" s="13" t="inlineStr">
@@ -32140,7 +32208,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I83" s="13" t="inlineStr"/>
+      <c r="I83" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: stick insect hub water row now names Haaniella as wanting an open water bowl, matching the feeding guide.</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="32" t="inlineStr">
@@ -32266,9 +32338,9 @@
           <t>content/guides/stick-insect-health-issues-guide.mdx</t>
         </is>
       </c>
-      <c r="D88" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D88" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E88" s="13" t="inlineStr">
@@ -32291,7 +32363,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I88" s="13" t="inlineStr"/>
+      <c r="I88" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: health guide now holds tropical humidity with misting and partial cover, not a sealed cage, matching the enrichment and setup guides.</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="32" t="inlineStr">
@@ -32363,9 +32439,9 @@
           <t>content/guides/invertebrate-quarantine-cleaning-and-escapes-guide.mdx</t>
         </is>
       </c>
-      <c r="D91" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D91" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E91" s="13" t="inlineStr">
@@ -32388,7 +32464,11 @@
           <t>Fix it in the shared cross-species guide; one edit there clears the same conflict for every animal it covers. Source check the figure first.</t>
         </is>
       </c>
-      <c r="I91" s="13" t="inlineStr"/>
+      <c r="I91" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: quarantine guide body and table now make stick insects the weekly exception, matching the stick insect health guide and hub.</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="33" t="inlineStr">
@@ -32446,7 +32526,11 @@
           <t>Copy the cost guide's figure into the hub line, exactly as the cost guide prints it.</t>
         </is>
       </c>
-      <c r="I93" s="13" t="inlineStr"/>
+      <c r="I93" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: prices are never changed (owner). Note only: hub route line says $60 to $150; the cost guide and Budget row say $45 to $170.</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="34" t="inlineStr">
@@ -32653,9 +32737,9 @@
           <t>content/guides/aquarium-stocking-and-tankmates-guide.mdx</t>
         </is>
       </c>
-      <c r="D101" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D101" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E101" s="13" t="inlineStr">
@@ -32678,7 +32762,11 @@
           <t>Fix it in the shared cross-species guide; one edit there clears the same conflict for every animal it covers. Source check the figure first.</t>
         </is>
       </c>
-      <c r="I101" s="13" t="inlineStr"/>
+      <c r="I101" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: stocking table now says alone or in groups for amano shrimp, matching the setup guide.</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="35" t="inlineStr">
@@ -32738,9 +32826,9 @@
           <t>content/guides/cherry-shrimp-cost-guide.mdx</t>
         </is>
       </c>
-      <c r="D104" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D104" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E104" s="13" t="inlineStr">
@@ -32763,7 +32851,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I104" s="13" t="inlineStr"/>
+      <c r="I104" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: cost guide now says above the high 50s, matching its FAQ and the setup guide.</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="36" t="inlineStr">
@@ -32781,9 +32873,9 @@
           <t>content/guides/cherry-shrimp-cost-guide.mdx</t>
         </is>
       </c>
-      <c r="D105" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D105" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E105" s="13" t="inlineStr">
@@ -32806,7 +32898,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I105" s="13" t="inlineStr"/>
+      <c r="I105" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: cost guide now calls ghost shrimp unrelated, matching the ghost shrimp pages and encyclopedia.</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="36" t="inlineStr">
@@ -32851,9 +32947,9 @@
           <t>content/guides/cherry-shrimp-feeding-guide.mdx</t>
         </is>
       </c>
-      <c r="D107" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D107" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E107" s="13" t="inlineStr">
@@ -32876,7 +32972,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I107" s="13" t="inlineStr"/>
+      <c r="I107" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: feeding FAQ now says a couple of times a week on top of grazing, matching line 61 and the hub.</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="36" t="inlineStr">
@@ -32894,9 +32994,9 @@
           <t>content/guides/cherry-shrimp-handling-guide.mdx</t>
         </is>
       </c>
-      <c r="D108" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D108" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E108" s="13" t="inlineStr">
@@ -32919,7 +33019,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I108" s="13" t="inlineStr"/>
+      <c r="I108" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: handling FAQ now says one drop every one to two seconds, matching line 60 and the hub.</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="36" t="inlineStr">
@@ -33053,9 +33157,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D113" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D113" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E113" s="13" t="inlineStr">
@@ -33078,7 +33182,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I113" s="13" t="inlineStr"/>
+      <c r="I113" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: the hub Recovery first row had no source anywhere on the site; replaced with a Buy carefully row backed by the cost guide (feeder stock, whisker shrimp mislabeling). Route line now describes what the enrichment guide covers.</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="12" t="inlineStr">
@@ -33121,7 +33229,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I114" s="13" t="inlineStr"/>
+      <c r="I114" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: prices are never changed (owner). Note only: line 96 says $40 to $180; the heading, FAQ and hub say $50 to $180.</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="12" t="inlineStr">
@@ -33139,9 +33251,9 @@
           <t>content/guides/ghost-shrimp-enrichment-guide.mdx</t>
         </is>
       </c>
-      <c r="D115" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D115" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E115" s="13" t="inlineStr">
@@ -33164,7 +33276,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I115" s="13" t="inlineStr"/>
+      <c r="I115" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: resolved the other way. ADW (listed on both pages) says the wild diet is dominated by algae, so the enrichment guide stands; the feeding guide FAQ and body now say wild shrimp eat algae but are a detritus crew in a tank, matching the hub.</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="12" t="inlineStr">
@@ -33317,9 +33433,9 @@
           <t>content/guides/aquarium-stocking-and-tankmates-guide.mdx</t>
         </is>
       </c>
-      <c r="D121" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D121" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E121" s="13" t="inlineStr">
@@ -33342,7 +33458,11 @@
           <t>Fix it in the shared cross-species guide; one edit there clears the same conflict for every animal it covers. Source check the figure first.</t>
         </is>
       </c>
-      <c r="I121" s="13" t="inlineStr"/>
+      <c r="I121" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: stocking table now says solitary, no group needed for ghost shrimp, matching the enrichment guide.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:I121"/>

</xml_diff>

<commit_message>
Consistency sweep: reptile minor rows
Bearded dragon and leopard gecko feeding, crested gecko space, insects
and cool area, fat-tail dusting and gut-loading, tokay diet, nights and
dusting, blue-tongue brumation, fire skink humidity, anole bulb, iguana
housing, size and greens, chameleon diet, water and UVB, savannah size
and calcium, tegu weighing and calcium, uromastyx weight, seeds and
lifespan, snake outage lows, kingsnake feeding, snake sizes, corn snake
heat and enclosure, hognose size, rosy boa legal and size, tortoise
sizes, pyramiding study, red-foot lifespan, sulcata weight and pen,
box turtle space, diet and brumation threshold, slider size. Prices,
products and two package lines noted.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CONSISTENCY_CHECK.xlsx
+++ b/CONSISTENCY_CHECK.xlsx
@@ -704,16 +704,16 @@
         <v>16</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.8125</v>
+        <v>1</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -731,16 +731,16 @@
         <v>11</v>
       </c>
       <c r="D6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="F6" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="F6" s="6" t="n">
-        <v>0.9090909090909091</v>
-      </c>
       <c r="G6" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -758,16 +758,16 @@
         <v>10</v>
       </c>
       <c r="D7" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G7" s="5" t="n">
         <v>4</v>
-      </c>
-      <c r="E7" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="F7" s="6" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="G7" s="5" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -785,16 +785,16 @@
         <v>8</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0.75</v>
+        <v>0.875</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
@@ -839,16 +839,16 @@
         <v>7</v>
       </c>
       <c r="D10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="F10" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="E10" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="F10" s="6" t="n">
-        <v>0.8571428571428571</v>
-      </c>
       <c r="G10" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
@@ -893,16 +893,16 @@
         <v>8</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>0.625</v>
+        <v>1</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
@@ -920,16 +920,16 @@
         <v>9</v>
       </c>
       <c r="D13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="F13" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="E13" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="F13" s="6" t="n">
-        <v>0.8888888888888888</v>
-      </c>
       <c r="G13" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
@@ -947,16 +947,16 @@
         <v>7</v>
       </c>
       <c r="D14" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.8571428571428571</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -974,16 +974,16 @@
         <v>8</v>
       </c>
       <c r="D15" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G15" s="5" t="n">
         <v>2</v>
-      </c>
-      <c r="E15" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="F15" s="6" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G15" s="5" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -1001,16 +1001,16 @@
         <v>9</v>
       </c>
       <c r="D16" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="F16" s="6" t="n">
+        <v>0.8888888888888888</v>
+      </c>
+      <c r="G16" s="5" t="n">
         <v>4</v>
-      </c>
-      <c r="E16" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="F16" s="6" t="n">
-        <v>0.5555555555555556</v>
-      </c>
-      <c r="G16" s="5" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -1028,16 +1028,16 @@
         <v>9</v>
       </c>
       <c r="D17" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.8888888888888888</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
@@ -1055,16 +1055,16 @@
         <v>8</v>
       </c>
       <c r="D18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="F18" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="5" t="n">
         <v>2</v>
-      </c>
-      <c r="E18" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="F18" s="6" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G18" s="5" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -1109,16 +1109,16 @@
         <v>9</v>
       </c>
       <c r="D20" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="F20" s="6" t="n">
+        <v>0.8888888888888888</v>
+      </c>
+      <c r="G20" s="5" t="n">
         <v>3</v>
-      </c>
-      <c r="E20" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="F20" s="6" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="G20" s="5" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -1136,16 +1136,16 @@
         <v>8</v>
       </c>
       <c r="D21" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="22">
@@ -1163,16 +1163,16 @@
         <v>8</v>
       </c>
       <c r="D22" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E22" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="F22" s="6" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G22" s="5" t="n">
         <v>5</v>
-      </c>
-      <c r="F22" s="6" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="G22" s="5" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="23">
@@ -1244,16 +1244,16 @@
         <v>8</v>
       </c>
       <c r="D25" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="F25" s="6" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G25" s="5" t="n">
         <v>4</v>
-      </c>
-      <c r="E25" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="F25" s="6" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G25" s="5" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -1271,16 +1271,16 @@
         <v>8</v>
       </c>
       <c r="D26" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E26" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="F26" s="6" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G26" s="5" t="n">
         <v>5</v>
-      </c>
-      <c r="F26" s="6" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="G26" s="5" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="27">
@@ -1325,16 +1325,16 @@
         <v>11</v>
       </c>
       <c r="D28" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F28" s="6" t="n">
-        <v>0.7272727272727273</v>
+        <v>1</v>
       </c>
       <c r="G28" s="5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="29">
@@ -1352,16 +1352,16 @@
         <v>9</v>
       </c>
       <c r="D29" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F29" s="6" t="n">
-        <v>0.7777777777777778</v>
+        <v>0.8888888888888888</v>
       </c>
       <c r="G29" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30">
@@ -1379,16 +1379,16 @@
         <v>9</v>
       </c>
       <c r="D30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="F30" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" s="5" t="n">
         <v>3</v>
-      </c>
-      <c r="E30" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="F30" s="6" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="G30" s="5" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -1406,16 +1406,16 @@
         <v>10</v>
       </c>
       <c r="D31" s="5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F31" s="6" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="G31" s="5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32">
@@ -1433,16 +1433,16 @@
         <v>9</v>
       </c>
       <c r="D32" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E32" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="F32" s="6" t="n">
+        <v>0.7777777777777778</v>
+      </c>
+      <c r="G32" s="5" t="n">
         <v>5</v>
-      </c>
-      <c r="E32" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="F32" s="6" t="n">
-        <v>0.4444444444444444</v>
-      </c>
-      <c r="G32" s="5" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="33">
@@ -1460,16 +1460,16 @@
         <v>9</v>
       </c>
       <c r="D33" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F33" s="6" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.8888888888888888</v>
       </c>
       <c r="G33" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34">
@@ -1487,16 +1487,16 @@
         <v>10</v>
       </c>
       <c r="D34" s="5" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F34" s="6" t="n">
-        <v>0.4</v>
+        <v>0.9</v>
       </c>
       <c r="G34" s="5" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="35">
@@ -1514,16 +1514,16 @@
         <v>9</v>
       </c>
       <c r="D35" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="F35" s="6" t="n">
+        <v>0.8888888888888888</v>
+      </c>
+      <c r="G35" s="5" t="n">
         <v>2</v>
-      </c>
-      <c r="E35" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="F35" s="6" t="n">
-        <v>0.7777777777777778</v>
-      </c>
-      <c r="G35" s="5" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="36">
@@ -3616,22 +3616,22 @@
         <v>784</v>
       </c>
       <c r="D113" s="7" t="n">
-        <v>102</v>
+        <v>48</v>
       </c>
       <c r="E113" s="7" t="n">
-        <v>682</v>
+        <v>736</v>
       </c>
       <c r="F113" s="8" t="n">
-        <v>0.8698979591836735</v>
+        <v>0.9387755102040817</v>
       </c>
       <c r="G113" s="7" t="n">
-        <v>218</v>
+        <v>274</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="9" t="inlineStr">
         <is>
-          <t>Every number on this tab is a value counted from the category tabs, recounted on each update (no formulas, so it reads the same in any viewer). Conflicts overall: 324 found, 218 fixed, 106 open (67% fixed). Last recount 2026-10-05.</t>
+          <t>Every number on this tab is a value counted from the category tabs, recounted on each update (no formulas, so it reads the same in any viewer). Conflicts overall: 324 found, 274 fixed, 50 open (85% fixed). Last recount 2026-10-05.</t>
         </is>
       </c>
     </row>
@@ -3970,9 +3970,9 @@
           <t>content/guides/bearded-dragon-feeding-guide.mdx</t>
         </is>
       </c>
-      <c r="D10" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E10" s="13" t="inlineStr">
@@ -3995,7 +3995,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I10" s="13" t="inlineStr"/>
+      <c r="I10" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: feeding guide now says mealworms and superworms are an occasional adult food only, matching the safe foods guide.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -4249,9 +4253,9 @@
           <t>content/guides/bearded-dragon-vs-leopard-gecko-guide.mdx</t>
         </is>
       </c>
-      <c r="D19" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D19" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E19" s="13" t="inlineStr">
@@ -4274,7 +4278,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I19" s="13" t="inlineStr"/>
+      <c r="I19" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: comparison FAQ and table now say adult dragons get greens daily or every other day and insects a few times a week, matching the feeding guide.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
@@ -4292,9 +4300,9 @@
           <t>content/guides/uromastyx-vs-bearded-dragon-guide.mdx</t>
         </is>
       </c>
-      <c r="D20" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D20" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E20" s="13" t="inlineStr">
@@ -4317,7 +4325,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I20" s="13" t="inlineStr"/>
+      <c r="I20" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: comparison now says about 80% insects for juveniles and humidity about 30 to 40%, matching the setup guide.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="16" t="inlineStr">
@@ -4640,9 +4652,9 @@
           <t>content/guides/bearded-dragon-vs-leopard-gecko-guide.mdx</t>
         </is>
       </c>
-      <c r="D32" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D32" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E32" s="13" t="inlineStr">
@@ -4665,7 +4677,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I32" s="13" t="inlineStr"/>
+      <c r="I32" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: comparison FAQ and table now say adult leopard geckos eat every 2 to 4 days, matching the feeding guide.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="18" t="inlineStr">
@@ -4725,9 +4741,9 @@
           <t>content/guides/crested-gecko-cost-guide.mdx</t>
         </is>
       </c>
-      <c r="D35" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D35" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E35" s="13" t="inlineStr">
@@ -4750,7 +4766,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I35" s="13" t="inlineStr"/>
+      <c r="I35" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: cost guide now doubles the 18x18x24 single-adult minimum, about 15,500 cubic inches.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="19" t="inlineStr">
@@ -4768,9 +4788,9 @@
           <t>content/guides/crested-gecko-enrichment-guide.mdx</t>
         </is>
       </c>
-      <c r="D36" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D36" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E36" s="13" t="inlineStr">
@@ -4793,7 +4813,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I36" s="13" t="inlineStr"/>
+      <c r="I36" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: enrichment guide now says about once a week at most, matching the feeding guide.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="19" t="inlineStr">
@@ -4946,9 +4970,9 @@
           <t>content/guides/crested-gecko-tank-setup-guide.mdx</t>
         </is>
       </c>
-      <c r="D42" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D42" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E42" s="13" t="inlineStr">
@@ -4971,7 +4995,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I42" s="13" t="inlineStr"/>
+      <c r="I42" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: setup table cool area now 72 to 75F, matching its own line 81.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="19" t="inlineStr">
@@ -5063,7 +5091,7 @@
       </c>
       <c r="I44" s="13" t="inlineStr">
         <is>
-          <t>Logged in FIX_PACKAGES.md.</t>
+          <t>2026-10-05: care package, never edited from the sweep. Noted in FIX_PACKAGES.md under Crested gecko.</t>
         </is>
       </c>
     </row>
@@ -5150,7 +5178,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I47" s="13" t="inlineStr"/>
+      <c r="I47" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: prices are never changed (owner). Note only: heading says $100 to $200 for Normals; line 59, the hub and package say around $100.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="21" t="inlineStr">
@@ -5242,9 +5274,9 @@
           <t>content/guides/african-fat-tail-feeding-guide.mdx</t>
         </is>
       </c>
-      <c r="D50" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D50" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E50" s="13" t="inlineStr">
@@ -5267,7 +5299,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I50" s="13" t="inlineStr"/>
+      <c r="I50" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: feeding guide dusting now adds a reptile multivitamin about once a week, matching the cost guide, hub and package.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="21" t="inlineStr">
@@ -5285,9 +5321,9 @@
           <t>content/guides/african-fat-tail-feeding-guide.mdx</t>
         </is>
       </c>
-      <c r="D51" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D51" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E51" s="13" t="inlineStr">
@@ -5310,7 +5346,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I51" s="13" t="inlineStr"/>
+      <c r="I51" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: feeding guide now says 24 to 72 hours, matching its own line 97 and the gut-loading guide.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="21" t="inlineStr">
@@ -5991,9 +6031,9 @@
           <t>content/guides/leaf-tailed-gecko-tank-setup-guide.mdx</t>
         </is>
       </c>
-      <c r="D73" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D73" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E73" s="13" t="inlineStr">
@@ -6016,7 +6056,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I73" s="13" t="inlineStr"/>
+      <c r="I73" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: already fixed in the Fable correction pass (setup FAQ now sets heat by species).</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="26" t="inlineStr">
@@ -6441,9 +6485,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D87" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D87" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E87" s="13" t="inlineStr">
@@ -6466,7 +6510,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I87" s="13" t="inlineStr"/>
+      <c r="I87" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: hub Diet row now treats a powdered diet as an occasional treat and dusts plain calcium under UVB, matching the feeding guide.</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="32" t="inlineStr">
@@ -6612,9 +6660,9 @@
           <t>content/guides/tokay-gecko-health-issues-guide.mdx</t>
         </is>
       </c>
-      <c r="D92" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D92" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E92" s="13" t="inlineStr">
@@ -6637,7 +6685,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I92" s="13" t="inlineStr"/>
+      <c r="I92" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: health guide now says nights 75 to 80F, never below about 70F, matching the setup guide.</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="32" t="inlineStr">
@@ -6682,9 +6734,9 @@
           <t>content/guides/tokay-gecko-tank-setup-guide.mdx</t>
         </is>
       </c>
-      <c r="D94" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D94" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E94" s="13" t="inlineStr">
@@ -6707,7 +6759,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I94" s="13" t="inlineStr"/>
+      <c r="I94" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: setup FAQ and body now dust plain calcium under UVB and D3 only without it, matching the feeding guide.</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="32" t="inlineStr">
@@ -6848,9 +6904,9 @@
           <t>content/guides/blue-tongue-skink-feeding-guide.mdx</t>
         </is>
       </c>
-      <c r="D100" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D100" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E100" s="13" t="inlineStr">
@@ -6873,7 +6929,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I100" s="13" t="inlineStr"/>
+      <c r="I100" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: feeding guide now says about 1 to 4 months, Australian species only, and the FAQ and line 93 say up to about 4 months, matching the health guide.</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="34" t="inlineStr">
@@ -7140,7 +7200,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I109" s="13" t="inlineStr"/>
+      <c r="I109" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: prices are never changed (owner). Note only: monthly cost says $40 to $65; its own items add to about $32 to $60.</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="36" t="inlineStr">
@@ -7239,9 +7303,9 @@
           <t>content/guides/fire-skink-health-issues-guide.mdx</t>
         </is>
       </c>
-      <c r="D113" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D113" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E113" s="13" t="inlineStr">
@@ -7264,7 +7328,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I113" s="13" t="inlineStr"/>
+      <c r="I113" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: health FAQ and hub now say 60 to 70% ambient humidity with damp substrate, matching the setup guide.</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="36" t="inlineStr">
@@ -7580,9 +7648,9 @@
           <t>content/guides/green-anole-tank-setup-guide.mdx</t>
         </is>
       </c>
-      <c r="D124" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D124" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E124" s="13" t="inlineStr">
@@ -7605,7 +7673,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I124" s="13" t="inlineStr"/>
+      <c r="I124" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: setup text now says 75-watt, matching the linked product and the cost guide.</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="12" t="inlineStr">
@@ -7793,9 +7865,9 @@
           <t>content/guides/green-iguana-handling-guide.mdx</t>
         </is>
       </c>
-      <c r="D131" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D131" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E131" s="13" t="inlineStr">
@@ -7818,7 +7890,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I131" s="13" t="inlineStr"/>
+      <c r="I131" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: handling mistake now says two adults, males above all, and adults live alone, matching the enrichment guide and hub.</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="17" t="inlineStr">
@@ -7863,9 +7939,9 @@
           <t>content/guides/green-iguana-legal-guide.mdx</t>
         </is>
       </c>
-      <c r="D133" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D133" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E133" s="13" t="inlineStr">
@@ -7888,7 +7964,11 @@
           <t>Re-read the legal guide table and its cited statutes, then make this line match the table.</t>
         </is>
       </c>
-      <c r="I133" s="13" t="inlineStr"/>
+      <c r="I133" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: legal guide now says six to seven feet, matching the handling guide and encyclopedia.</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="17" t="inlineStr">
@@ -8007,9 +8087,9 @@
           <t>content/guides/iguana-fireskink-quaker-overview.mdx</t>
         </is>
       </c>
-      <c r="D137" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D137" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E137" s="13" t="inlineStr">
@@ -8032,7 +8112,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I137" s="13" t="inlineStr"/>
+      <c r="I137" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: overview now names collards, mustard and turnip greens, with kale rotated in, matching the feeding guide.</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="18" t="inlineStr">
@@ -8274,9 +8358,9 @@
           <t>content/guides/jacksons-chameleon-tank-setup-guide.mdx</t>
         </is>
       </c>
-      <c r="D146" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D146" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E146" s="13" t="inlineStr">
@@ -8299,7 +8383,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I146" s="13" t="inlineStr"/>
+      <c r="I146" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: setup guide now puts crickets, roaches, silkworms and grasshoppers as the core and the worms as occasional extras, matching the feeding guide.</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="19" t="inlineStr">
@@ -8344,9 +8432,9 @@
           <t>content/guides/chameleon-hydration-drippers-misters-fogging.mdx</t>
         </is>
       </c>
-      <c r="D148" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D148" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E148" s="13" t="inlineStr">
@@ -8369,7 +8457,11 @@
           <t>Fix it in the shared cross-species guide; one edit there clears the same conflict for every animal it covers. Source check the figure first.</t>
         </is>
       </c>
-      <c r="I148" s="13" t="inlineStr"/>
+      <c r="I148" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: hydration FAQ now treats tap water first and runs automatic misters, foggers and drippers on distilled water, matching both setup guides.</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="20" t="inlineStr">
@@ -8402,9 +8494,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D150" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D150" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E150" s="13" t="inlineStr">
@@ -8427,7 +8519,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I150" s="13" t="inlineStr"/>
+      <c r="I150" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: hub Legal check now adds West Virginia importation permit, matching the legal guide.</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="21" t="inlineStr">
@@ -8445,9 +8541,9 @@
           <t>content/guides/veiled-chameleon-cost-guide.mdx</t>
         </is>
       </c>
-      <c r="D151" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D151" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E151" s="13" t="inlineStr">
@@ -8470,7 +8566,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I151" s="13" t="inlineStr"/>
+      <c r="I151" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: cost table now names ReptiSun 5.0 or Arcadia 6%, matching the setup guide. Price unchanged.</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="21" t="inlineStr">
@@ -8811,7 +8911,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I162" s="13" t="inlineStr"/>
+      <c r="I162" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: affiliate product link, left as a note. The enrichment guide links the 48x24x48 PVC enclosure, under the setup minimum of 5 x 2.5 x 4 ft; same product question as Reptiles row 161.</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="23" t="inlineStr">
@@ -9053,9 +9157,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D171" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D171" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E171" s="13" t="inlineStr">
@@ -9078,7 +9182,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I171" s="13" t="inlineStr"/>
+      <c r="I171" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: hub route line now says plain calcium under UVB and D3 only without it, matching the feeding guide.</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="26" t="inlineStr">
@@ -9121,7 +9229,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I172" s="13" t="inlineStr"/>
+      <c r="I172" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: prices are never changed (owner). Note only: FAQ says several hundred to over a thousand dollars; the enclosure row alone is $725 to $1,500.</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="26" t="inlineStr">
@@ -9375,9 +9487,9 @@
           <t>content/guides/savannah-russiantortoise-cockatoo-stickinsect-overview.mdx</t>
         </is>
       </c>
-      <c r="D181" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D181" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E181" s="13" t="inlineStr">
@@ -9400,7 +9512,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I181" s="13" t="inlineStr"/>
+      <c r="I181" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: overview FAQ and body now say most adults reach 3 to 4 feet, matching the handling guide and encyclopedia.</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="29" t="inlineStr">
@@ -9561,9 +9677,9 @@
           <t>content/guides/argentine-tegu-feeding-guide.mdx</t>
         </is>
       </c>
-      <c r="D187" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D187" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E187" s="13" t="inlineStr">
@@ -9586,7 +9702,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I187" s="13" t="inlineStr"/>
+      <c r="I187" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: feeding table now says weigh weekly, matching the health guide.</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="30" t="inlineStr">
@@ -9752,9 +9872,9 @@
           <t>content/guides/argentine-tegu-tank-setup-guide.mdx</t>
         </is>
       </c>
-      <c r="D192" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D192" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E192" s="13" t="inlineStr">
@@ -9777,7 +9897,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I192" s="13" t="inlineStr"/>
+      <c r="I192" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: setup guide, hub and health guide now put calcium on everything except whole prey, matching the feeding guide.</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="30" t="inlineStr">
@@ -9884,9 +10008,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D196" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D196" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E196" s="13" t="inlineStr">
@@ -9909,7 +10033,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I196" s="13" t="inlineStr"/>
+      <c r="I196" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: hub now says more than 10%, matching the feeding guide.</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="32" t="inlineStr">
@@ -10129,9 +10257,9 @@
           <t>content/guides/uromastyx-tank-setup-guide.mdx</t>
         </is>
       </c>
-      <c r="D203" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D203" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E203" s="13" t="inlineStr">
@@ -10154,7 +10282,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I203" s="13" t="inlineStr"/>
+      <c r="I203" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: setup FAQ and body now call uromastyx near-strict herbivores with seeds a limited extra, matching the feeding guide.</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="32" t="inlineStr">
@@ -10199,9 +10331,9 @@
           <t>content/guides/uromastyx-tokay-africangrey-jumpingspider-overview.mdx</t>
         </is>
       </c>
-      <c r="D205" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D205" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E205" s="13" t="inlineStr">
@@ -10224,7 +10356,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I205" s="13" t="inlineStr"/>
+      <c r="I205" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: overview now says 15 to 20 years, past 25 with excellent care, matching the cost guide.</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="33" t="inlineStr">
@@ -10907,9 +11043,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D229" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D229" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E229" s="13" t="inlineStr">
@@ -10932,7 +11068,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I229" s="13" t="inlineStr"/>
+      <c r="I229" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: kingsnake hub power outage row now says 68 to 72F night low, matching the setup and health guides.</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" s="12" t="inlineStr">
@@ -10975,7 +11115,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I230" s="13" t="inlineStr"/>
+      <c r="I230" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: prices are never changed (owner). Note only: lines 45 and 89 say $200 to $500; the setup table sums to about $354 to $506.</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="12" t="inlineStr">
@@ -11020,9 +11164,9 @@
           <t>content/guides/california-kingsnake-feeding-guide.mdx</t>
         </is>
       </c>
-      <c r="D232" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D232" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E232" s="13" t="inlineStr">
@@ -11045,7 +11189,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I232" s="13" t="inlineStr"/>
+      <c r="I232" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: feeding FAQ and line 65 now say every 10 to 14 days maintains an adult, matching line 61.</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="12" t="inlineStr">
@@ -11171,9 +11319,9 @@
           <t>content/guides/snake-sexing-growth-body-condition-guide.mdx</t>
         </is>
       </c>
-      <c r="D237" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D237" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E237" s="13" t="inlineStr">
@@ -11196,7 +11344,11 @@
           <t>Fix it in the shared cross-species guide; one edit there clears the same conflict for every animal it covers. Source check the figure first.</t>
         </is>
       </c>
-      <c r="I237" s="13" t="inlineStr"/>
+      <c r="I237" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: sexing guide now says corn snakes 3.5 to 5 feet and kingsnakes 3 to 4, matching the encyclopedia and setup guides.</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" s="16" t="inlineStr">
@@ -11348,7 +11500,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I241" s="13" t="inlineStr"/>
+      <c r="I241" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: prices are never changed (owner). Note only: lines 45 and 91 say $200 to $500 a year; the tables sum to about $260 to $660.</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" s="17" t="inlineStr">
@@ -11366,9 +11522,9 @@
           <t>content/guides/corn-snake-enrichment-guide.mdx</t>
         </is>
       </c>
-      <c r="D242" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D242" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E242" s="13" t="inlineStr">
@@ -11391,7 +11547,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I242" s="13" t="inlineStr"/>
+      <c r="I242" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: enrichment guide now says a 4x2x2 suits most adults, a 5-foot snake is happier in something longer.</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" s="17" t="inlineStr">
@@ -11456,9 +11616,9 @@
           <t>content/guides/corn-snake-feeding-guide.mdx</t>
         </is>
       </c>
-      <c r="D244" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D244" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E244" s="13" t="inlineStr">
@@ -11481,7 +11641,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I244" s="13" t="inlineStr"/>
+      <c r="I244" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: feeding guide now says 85 to 90F warm side, matching the setup guide.</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" s="17" t="inlineStr">
@@ -12081,9 +12245,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D263" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D263" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E263" s="13" t="inlineStr">
@@ -12106,7 +12270,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I263" s="13" t="inlineStr"/>
+      <c r="I263" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: hub and encyclopedia now give 14 to 46 inches across species, western hognoses 14 to 37, matching both comparison pages.</t>
+        </is>
+      </c>
     </row>
     <row r="264">
       <c r="A264" s="21" t="inlineStr">
@@ -12360,9 +12528,9 @@
           <t>content/guides/corn-snake-vs-hognose-snake-guide.mdx</t>
         </is>
       </c>
-      <c r="D272" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D272" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E272" s="13" t="inlineStr">
@@ -12385,7 +12553,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I272" s="13" t="inlineStr"/>
+      <c r="I272" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: cleared by row 263 (hub and encyclopedia now carry the western 14 to 37 inch figure).</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" s="21" t="inlineStr">
@@ -12403,9 +12575,9 @@
           <t>content/guides/veiled-chameleon-ferret-hognose-overview.mdx</t>
         </is>
       </c>
-      <c r="D273" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D273" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E273" s="13" t="inlineStr">
@@ -12428,7 +12600,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I273" s="13" t="inlineStr"/>
+      <c r="I273" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: cleared by row 263 (hub and encyclopedia now carry the 14 to 46 inch species range).</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" s="22" t="inlineStr">
@@ -12461,9 +12637,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D275" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D275" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E275" s="13" t="inlineStr">
@@ -12486,7 +12662,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I275" s="13" t="inlineStr"/>
+      <c r="I275" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: milk snake hub power outage row now says 70 to 75F night low, heat below 70F, matching the setup guide.</t>
+        </is>
+      </c>
     </row>
     <row r="276">
       <c r="A276" s="23" t="inlineStr">
@@ -12745,7 +12925,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I284" s="13" t="inlineStr"/>
+      <c r="I284" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: affiliate product link, left as a note. The comparison links a 36x18x18 enclosure while the text gives the milk snake adult minimum of 48x24x24. Needs an owner product call.</t>
+        </is>
+      </c>
     </row>
     <row r="285">
       <c r="A285" s="25" t="inlineStr">
@@ -12778,9 +12962,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D286" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D286" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E286" s="13" t="inlineStr">
@@ -12803,7 +12987,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I286" s="13" t="inlineStr"/>
+      <c r="I286" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: hub Legal check now adds Delaware permit and West Virginia import permit, matching the legal guide.</t>
+        </is>
+      </c>
     </row>
     <row r="287">
       <c r="A287" s="26" t="inlineStr">
@@ -12956,9 +13144,9 @@
           <t>content/guides/rosy-boa-legal-guide.mdx</t>
         </is>
       </c>
-      <c r="D292" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D292" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E292" s="13" t="inlineStr">
@@ -12981,7 +13169,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I292" s="13" t="inlineStr"/>
+      <c r="I292" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: legal FAQ drops the West Virginia six-foot threshold, matching its own table and the boa legal guide.</t>
+        </is>
+      </c>
     </row>
     <row r="293">
       <c r="A293" s="26" t="inlineStr">
@@ -13053,9 +13245,9 @@
           <t>content/guides/red-footed-tortoise-garter-snake-rosy-boa-overview.mdx</t>
         </is>
       </c>
-      <c r="D295" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D295" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E295" s="13" t="inlineStr">
@@ -13078,7 +13270,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I295" s="13" t="inlineStr"/>
+      <c r="I295" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: overview now says 24 to 36 inches, rarely over 4 feet, matching the setup guide and encyclopedia.</t>
+        </is>
+      </c>
     </row>
     <row r="296">
       <c r="A296" s="29" t="inlineStr">
@@ -13111,9 +13307,9 @@
           <t>src/lib/data/guides (hub entry)</t>
         </is>
       </c>
-      <c r="D297" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D297" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E297" s="13" t="inlineStr">
@@ -13136,7 +13332,11 @@
           <t>Update the hub row to match the owner deep dive; the hub routes, the deep dive owns the number.</t>
         </is>
       </c>
-      <c r="I297" s="13" t="inlineStr"/>
+      <c r="I297" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: hub and encyclopedia now say 5 to 9 inches, matching the handling guide.</t>
+        </is>
+      </c>
     </row>
     <row r="298">
       <c r="A298" s="30" t="inlineStr">
@@ -13154,9 +13354,9 @@
           <t>content/guides/russian-tortoise-cost-guide.mdx</t>
         </is>
       </c>
-      <c r="D298" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D298" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E298" s="13" t="inlineStr">
@@ -13179,7 +13379,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I298" s="13" t="inlineStr"/>
+      <c r="I298" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: cost guide now says 5 to 9 inches in all three places.</t>
+        </is>
+      </c>
     </row>
     <row r="299">
       <c r="A299" s="30" t="inlineStr">
@@ -13384,7 +13588,11 @@
           <t>Book fix: logged in FIX_PACKAGES.md; make the change in the package source at the next edition, after the site side is settled.</t>
         </is>
       </c>
-      <c r="I305" s="13" t="inlineStr"/>
+      <c r="I305" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: care package, never edited from the sweep. Noted in FIX_PACKAGES.md under Russian tortoise.</t>
+        </is>
+      </c>
     </row>
     <row r="306">
       <c r="A306" s="30" t="inlineStr">
@@ -13402,9 +13610,9 @@
           <t>content/guides/sulcata-tortoise-vs-russian-tortoise-guide.mdx</t>
         </is>
       </c>
-      <c r="D306" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D306" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E306" s="13" t="inlineStr">
@@ -13427,7 +13635,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I306" s="13" t="inlineStr"/>
+      <c r="I306" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: comparison now says 5 to 9 inches in both places.</t>
+        </is>
+      </c>
     </row>
     <row r="307">
       <c r="A307" s="31" t="inlineStr">
@@ -13579,7 +13791,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I310" s="13" t="inlineStr"/>
+      <c r="I310" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: prices are never changed (owner). Note only: line 69 says $500 to $950; its own rows top $990 before the bulb and emitter.</t>
+        </is>
+      </c>
     </row>
     <row r="311">
       <c r="A311" s="32" t="inlineStr">
@@ -13678,9 +13894,9 @@
           <t>content/guides/red-footed-tortoise-health-issues-guide.mdx</t>
         </is>
       </c>
-      <c r="D314" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D314" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E314" s="13" t="inlineStr">
@@ -13703,7 +13919,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I314" s="13" t="inlineStr"/>
+      <c r="I314" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: health FAQ now credits the hatchling study with starch vs fiber and other tortoise research with humidity, matching line 78.</t>
+        </is>
+      </c>
     </row>
     <row r="315">
       <c r="A315" s="32" t="inlineStr">
@@ -13721,9 +13941,9 @@
           <t>content/guides/red-footed-tortoise-legal-guide.mdx</t>
         </is>
       </c>
-      <c r="D315" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D315" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E315" s="13" t="inlineStr">
@@ -13746,7 +13966,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I315" s="13" t="inlineStr"/>
+      <c r="I315" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: no change needed: the table has 9 restricted rows, not 10, so 43 plus 9 is 52, matching line 38.</t>
+        </is>
+      </c>
     </row>
     <row r="316">
       <c r="A316" s="32" t="inlineStr">
@@ -13789,7 +14013,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I316" s="13" t="inlineStr"/>
+      <c r="I316" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: prices are never changed (owner). Note only: setup guide says a basic fogger or misting system is $35 to $60; the cost guide says $50 to $180.</t>
+        </is>
+      </c>
     </row>
     <row r="317">
       <c r="A317" s="32" t="inlineStr">
@@ -13834,9 +14062,9 @@
           <t>content/guides/red-footed-tortoise-garter-snake-rosy-boa-overview.mdx</t>
         </is>
       </c>
-      <c r="D318" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D318" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E318" s="13" t="inlineStr">
@@ -13859,7 +14087,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I318" s="13" t="inlineStr"/>
+      <c r="I318" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: overview now says captive individuals commonly live 50 years or more, some reported past 90, matching the cost guide and encyclopedia.</t>
+        </is>
+      </c>
     </row>
     <row r="319">
       <c r="A319" s="33" t="inlineStr">
@@ -13944,7 +14176,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I321" s="13" t="inlineStr"/>
+      <c r="I321" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: prices are never changed (owner). Note only: line 87 prices heated-shelter electricity at $150 to $350 a year; lines 101 and 107 work out to about $60 to $120 a season.</t>
+        </is>
+      </c>
     </row>
     <row r="322">
       <c r="A322" s="34" t="inlineStr">
@@ -14070,9 +14306,9 @@
           <t>content/guides/sulcata-tortoise-legal-guide.mdx</t>
         </is>
       </c>
-      <c r="D326" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D326" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E326" s="13" t="inlineStr">
@@ -14095,7 +14331,11 @@
           <t>Re-read the legal guide table and its cited statutes, then make this line match the table.</t>
         </is>
       </c>
-      <c r="I326" s="13" t="inlineStr"/>
+      <c r="I326" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: excerpt now says 80 to 110 pounds, big males to 200, and the description drops the 200 lb wording, matching the handling guide and encyclopedia.</t>
+        </is>
+      </c>
     </row>
     <row r="327">
       <c r="A327" s="34" t="inlineStr">
@@ -14167,9 +14407,9 @@
           <t>content/guides/sulcata-tortoise-vs-russian-tortoise-guide.mdx</t>
         </is>
       </c>
-      <c r="D329" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D329" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E329" s="13" t="inlineStr">
@@ -14192,7 +14432,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I329" s="13" t="inlineStr"/>
+      <c r="I329" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: comparison table now says 80 to 100+ sq ft per tortoise, matching the setup guide.</t>
+        </is>
+      </c>
     </row>
     <row r="330">
       <c r="A330" s="35" t="inlineStr">
@@ -14272,9 +14516,9 @@
           <t>content/guides/box-turtle-cost-guide.mdx</t>
         </is>
       </c>
-      <c r="D332" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D332" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E332" s="13" t="inlineStr">
@@ -14297,7 +14541,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I332" s="13" t="inlineStr"/>
+      <c r="I332" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: cost guide now scales from the 5.5 by 3 foot eastern box turtle size, matching the setup guide. Prices unchanged.</t>
+        </is>
+      </c>
     </row>
     <row r="333">
       <c r="A333" s="36" t="inlineStr">
@@ -14342,9 +14590,9 @@
           <t>content/guides/box-turtle-feeding-guide.mdx</t>
         </is>
       </c>
-      <c r="D334" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D334" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E334" s="13" t="inlineStr">
@@ -14367,7 +14615,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I334" s="13" t="inlineStr"/>
+      <c r="I334" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: feeding FAQ now says 60 or 70% plant matter overall, matching line 54.</t>
+        </is>
+      </c>
     </row>
     <row r="335">
       <c r="A335" s="36" t="inlineStr">
@@ -14466,9 +14718,9 @@
           <t>content/guides/box-turtle-tank-setup-guide.mdx</t>
         </is>
       </c>
-      <c r="D338" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D338" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E338" s="13" t="inlineStr">
@@ -14491,7 +14743,11 @@
           <t>Source check the owner page's figure, then rewrite this line to match it.</t>
         </is>
       </c>
-      <c r="I338" s="13" t="inlineStr"/>
+      <c r="I338" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: setup guide now says most tortoises are herbivores, the red-footed the omnivorous exception, matching the red-footed feeding guide.</t>
+        </is>
+      </c>
     </row>
     <row r="339">
       <c r="A339" s="36" t="inlineStr">
@@ -14536,9 +14792,9 @@
           <t>content/guides/leaftailedgecko-kingsnake-boxturtle-oscar-overview.mdx</t>
         </is>
       </c>
-      <c r="D340" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D340" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E340" s="13" t="inlineStr">
@@ -14561,7 +14817,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I340" s="13" t="inlineStr"/>
+      <c r="I340" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: overview FAQ and body now say most tortoises are herbivores.</t>
+        </is>
+      </c>
     </row>
     <row r="341">
       <c r="A341" s="36" t="inlineStr">
@@ -14579,9 +14839,9 @@
           <t>content/guides/tortoise-brumation-guide.mdx</t>
         </is>
       </c>
-      <c r="D341" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D341" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E341" s="13" t="inlineStr">
@@ -14604,7 +14864,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I341" s="13" t="inlineStr"/>
+      <c r="I341" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: brumation FAQ, hub and health guide now act at about 7 percent, before the 10 percent stop line, matching the guide's own line 122.</t>
+        </is>
+      </c>
     </row>
     <row r="342">
       <c r="A342" s="11" t="inlineStr">
@@ -14689,7 +14953,11 @@
           <t>Source check which of the page's own two statements is right, then make every line on this page say it.</t>
         </is>
       </c>
-      <c r="I344" s="13" t="inlineStr"/>
+      <c r="I344" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: prices are never changed (owner). Note only: line 99 says food $10 to $30 and electricity $10 to $25 a month; the table works out to $100 to $180 a year for each.</t>
+        </is>
+      </c>
     </row>
     <row r="345">
       <c r="A345" s="12" t="inlineStr">
@@ -14916,9 +15184,9 @@
           <t>content/guides/koi-conure-slider-scorpion-overview.mdx</t>
         </is>
       </c>
-      <c r="D352" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D352" s="14" t="inlineStr">
+        <is>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E352" s="13" t="inlineStr">
@@ -14941,7 +15209,11 @@
           <t>Change the overview or comparison line to match the owner page named in Conflicts with; it summarizes, the deep dive decides.</t>
         </is>
       </c>
-      <c r="I352" s="13" t="inlineStr"/>
+      <c r="I352" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-05: overview now says females average about 10 inches, males 7, big females 11 or 12, matching the setup guide.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:I352"/>

</xml_diff>

<commit_message>
Minor-row corrections from the Fable check
Guppy salt reversed (guppies tolerate salt; ich guide back to
livebearers, guppy health guide offers a salt course), cardinal tetra
school of 10 everywhere, oscar growth leftovers, hamster bedding hub,
chinchilla weight table and softer heat band, uveitis glossary,
emperor scorpion outage FAQ, cat dental figure corrected to Cornell's,
cherry shrimp drip wording. Two source items added to FIX_PLAN.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CONSISTENCY_CHECK.xlsx
+++ b/CONSISTENCY_CHECK.xlsx
@@ -18865,7 +18865,7 @@
       </c>
       <c r="I67" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: cost guide now says a 20-gallon long for the school of 10. Prices unchanged.</t>
+          <t>2026-10-05: cost guide now says a 20-gallon long for the school of 10. Prices unchanged. Fable follow-up: handling, setup, cost guide and hub leftovers now say a school of 10 too. The hub buy list line keeps its catalog covers text.</t>
         </is>
       </c>
     </row>
@@ -18966,7 +18966,7 @@
       </c>
       <c r="I70" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: handling guide now says ten is where natural schooling settles in, matching its own minimum of 10.</t>
+          <t>2026-10-05: handling guide now says ten is where natural schooling settles in, matching its own minimum of 10. Fable follow-up: description, FAQ and hub FAQ now say ten, with no 8 to 10.</t>
         </is>
       </c>
     </row>
@@ -19040,7 +19040,7 @@
       </c>
       <c r="I72" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: setup guide FAQ and body now plan on a 20-gallon long for a school of 10; the 10-gallon link stays, now described as too small.</t>
+          <t>2026-10-05: setup guide FAQ and body now plan on a 20-gallon long for a school of 10; the 10-gallon link stays, now described as too small. Fable follow-up: setup line 65 tail and hub tank size row now say the school of 10, a standard 10-gallon too small.</t>
         </is>
       </c>
     </row>
@@ -20035,7 +20035,7 @@
       </c>
       <c r="I105" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: ich guide salt line now names mollies and platies and sends guppies to medication, matching the guppy health guide.</t>
+          <t>2026-10-05: ich guide salt line now names mollies and platies and sends guppies to medication, matching the guppy health guide. Fable follow-up: reversed. The guppy health guide was the wrong page: guppies tolerate salt well (Chervinski 1984, Journal of Fish Biology; PetMD, listed). The ich guide is back to livebearers, and the guppy health guide FAQ and body now offer a salt course.</t>
         </is>
       </c>
     </row>
@@ -20989,7 +20989,7 @@
       </c>
       <c r="I135" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: setup guide body and FAQ, cost guide and hub now say about two-thirds of adult size in the first year, matching the feeding and handling guides.</t>
+          <t>2026-10-05: setup guide body and FAQ, cost guide and hub now say about two-thirds of adult size in the first year, matching the feeding and handling guides. Fable follow-up: cost guide FAQ line 51 and hub FAQ were left behind; both now say about two-thirds of adult size.</t>
         </is>
       </c>
     </row>
@@ -25570,7 +25570,7 @@
       </c>
       <c r="I22" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: conversion now reads about 16 to 31 inches (40 to 80 cm).</t>
+          <t>2026-10-05: conversion now reads about 16 to 31 inches (40 to 80 cm). Fable follow-up: hub bedding row also now says roughly 16 to 31 inches.</t>
         </is>
       </c>
     </row>
@@ -26226,7 +26226,7 @@
       </c>
       <c r="I42" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: hub and encyclopedia adult size now say about 0.9 to 1.5 lbs (400 to 700 g), matching the health guide.</t>
+          <t>2026-10-05: hub and encyclopedia adult size now say about 0.9 to 1.5 lbs (400 to 700 g), matching the health guide. Fable follow-up: chinchilla vs hamster table now says about 0.9-1.5 lbs too.</t>
         </is>
       </c>
     </row>
@@ -26603,7 +26603,7 @@
       </c>
       <c r="I53" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: comparison FAQ and table now say comfortable to about 68F and at risk from about 80F, matching the setup guide; a spaced hyphen in the table removed too.</t>
+          <t>2026-10-05: comparison FAQ and table now say comfortable to about 68F and at risk from about 80F, matching the setup guide; a spaced hyphen in the table removed too. Fable follow-up: softened to happiest in the 50s and 60s F; the comparison page's own sources run warmer (Merck 65 to 80F, PetMD 55 to 70F), and all agree on danger from about 80F.</t>
         </is>
       </c>
     </row>
@@ -30826,7 +30826,7 @@
       </c>
       <c r="I35" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: travel guide body and table now treat emperor scorpions as warm-kept, 75 to 85F with a side heat mat, so an outage matters, matching the setup guide.</t>
+          <t>2026-10-05: travel guide body and table now treat emperor scorpions as warm-kept, 75 to 85F with a side heat mat, so an outage matters, matching the setup guide. Fable follow-up: the same guide's FAQ line 41 now names the emperor scorpion among the animals kept on supplemental heat.</t>
         </is>
       </c>
     </row>
@@ -33293,7 +33293,7 @@
       </c>
       <c r="I108" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: handling FAQ now says one drop every one to two seconds, matching line 60 and the hub.</t>
+          <t>2026-10-05: handling FAQ now says one drop every one to two seconds, matching line 60 and the hub. Fable follow-up: doubled hedge removed (roughly one drop).</t>
         </is>
       </c>
     </row>
@@ -33914,7 +33914,7 @@
       </c>
       <c r="I4" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: cat hub now says up to 70% by age 2 and about 85% past age 6, matching the periodontal guide (Merck, Cornell).</t>
+          <t>2026-10-05: cat hub now says up to 70% by age 2 and about 85% past age 6, matching the periodontal guide (Merck, Cornell). Fable follow-up: Cornell actually says 50 to 90% of cats over 4; the 85% over 6 figure had no Cornell page behind it. Hub line and periodontal guide table now use the Cornell figure.</t>
         </is>
       </c>
     </row>
@@ -36843,7 +36843,7 @@
       </c>
       <c r="I48" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: Golden hub health line and FAQ now say about one in ten to nearly one in four, matching the eye disease guide.</t>
+          <t>2026-10-05: Golden hub health line and FAQ now say about one in ten to nearly one in four, matching the eye disease guide. Fable follow-up: site glossary entry also now says about one in ten to nearly one in four.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reptile minor-row corrections from the Fable check
Crested gecko cool area and pair space reverted (no conflict), tokay nights
never below 75F, blue-tongue brumation split by species, anole 75-watt
leftovers, iguana greens base, chameleon UVB label back to its covers match,
emergency plan snake night lows, uromastyx near-strict, Russian 5 to 9 inch
leftovers, red-foot lifespan, box turtle footprint and 7% line.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CONSISTENCY_CHECK.xlsx
+++ b/CONSISTENCY_CHECK.xlsx
@@ -758,16 +758,16 @@
         <v>10</v>
       </c>
       <c r="D7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="F7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="F7" s="6" t="n">
-        <v>0.9</v>
-      </c>
       <c r="G7" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -1055,16 +1055,16 @@
         <v>8</v>
       </c>
       <c r="D18" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F18" s="6" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="G18" s="5" t="n">
         <v>1</v>
-      </c>
-      <c r="G18" s="5" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="19">
@@ -3625,13 +3625,13 @@
         <v>0.9387755102040817</v>
       </c>
       <c r="G113" s="7" t="n">
-        <v>274</v>
+        <v>271</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="9" t="inlineStr">
         <is>
-          <t>Every number on this tab is a value counted from the category tabs, recounted on each update (no formulas, so it reads the same in any viewer). Conflicts overall: 324 found, 274 fixed, 50 open (85% fixed). Last recount 2026-10-05.</t>
+          <t>Every number on this tab is a value counted from the category tabs, recounted on each update (no formulas, so it reads the same in any viewer). Conflicts overall: 321 found, 271 fixed, 50 open (84% fixed). Last recount 2026-10-05.</t>
         </is>
       </c>
     </row>
@@ -4743,7 +4743,7 @@
       </c>
       <c r="D35" s="14" t="inlineStr">
         <is>
-          <t>✓ Fixed</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="E35" s="13" t="inlineStr">
@@ -4768,7 +4768,7 @@
       </c>
       <c r="I35" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: cost guide now doubles the 18x18x24 single-adult minimum, about 15,500 cubic inches.</t>
+          <t>2026-10-05: no conflict, reverted. The 18x18x36 is ReptiFiles' recommended size for one adult, a different baseline from the setup guide's 18x18x24 minimum, so double it (about 23,000 cubic inches) stands.</t>
         </is>
       </c>
     </row>
@@ -4972,7 +4972,7 @@
       </c>
       <c r="D42" s="14" t="inlineStr">
         <is>
-          <t>✓ Fixed</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="E42" s="13" t="inlineStr">
@@ -4997,7 +4997,7 @@
       </c>
       <c r="I42" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: setup table cool area now 72 to 75F, matching its own line 81.</t>
+          <t>2026-10-05: no conflict, reverted to 70 - 75F. ReptiFiles (listed) gives 70 to 75F for the bottom; the 72F warning is about the whole enclosure running cold for long stretches.</t>
         </is>
       </c>
     </row>
@@ -5064,9 +5064,9 @@
           <t>content/CAREPACKAGE Guides/source/crested-gecko-src</t>
         </is>
       </c>
-      <c r="D44" s="15" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D44" s="14" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="E44" s="13" t="inlineStr">
@@ -5091,7 +5091,7 @@
       </c>
       <c r="I44" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: care package, never edited from the sweep. Noted in FIX_PACKAGES.md under Crested gecko.</t>
+          <t>2026-10-05: no conflict. The book matches the cost guide (double an 18x18x36); the FIX_PACKAGES note was removed.</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="I92" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: health guide now says nights 75 to 80F, never below about 70F, matching the setup guide.</t>
+          <t>2026-10-05: health guide now says nights 75 to 80F, never below about 70F, matching the setup guide. Fable follow-up: corrected to never below 75F in the health guide and both setup guide lines; PetMD and ReptiFiles back 75F, nothing backs 70F.</t>
         </is>
       </c>
     </row>
@@ -6931,7 +6931,7 @@
       </c>
       <c r="I100" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: feeding guide now says about 1 to 4 months, Australian species only, and the FAQ and line 93 say up to about 4 months, matching the health guide.</t>
+          <t>2026-10-05: feeding guide now says about 1 to 4 months, Australian species only, and the FAQ and line 93 say up to about 4 months, matching the health guide. Fable follow-up: the Australian-only wording was wrong. The feeding guide now matches health guide line 91: temperate species (eastern, blotched, shingleback) brumate about 4 to 6 months; Northern and Indonesian are never cooled but may slow 1 to 4 months with the heat on.</t>
         </is>
       </c>
     </row>
@@ -7675,7 +7675,7 @@
       </c>
       <c r="I124" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: setup text now says 75-watt, matching the linked product and the cost guide.</t>
+          <t>2026-10-05: setup text now says 75-watt, matching the linked product and the cost guide. Fable follow-up: setup FAQ and hub temperature row also now say 75-watt.</t>
         </is>
       </c>
     </row>
@@ -8114,7 +8114,7 @@
       </c>
       <c r="I137" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: overview now names collards, mustard and turnip greens, with kale rotated in, matching the feeding guide.</t>
+          <t>2026-10-05: overview now names collards, mustard and turnip greens, with kale rotated in, matching the feeding guide. Fable follow-up: mustard greens are goitrogenic per the feeding guide, so the base is now collard and turnip greens with kale and mustard rotated in.</t>
         </is>
       </c>
     </row>
@@ -8543,7 +8543,7 @@
       </c>
       <c r="D151" s="14" t="inlineStr">
         <is>
-          <t>✓ Fixed</t>
+          <t>✗</t>
         </is>
       </c>
       <c r="E151" s="13" t="inlineStr">
@@ -8568,7 +8568,7 @@
       </c>
       <c r="I151" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: cost table now names ReptiSun 5.0 or Arcadia 6%, matching the setup guide. Price unchanged.</t>
+          <t>2026-10-05: affiliate covers text, left as a note. The cost table label is a catalog covers match for the UVB link (a new label broke it), so it stays; the setup guide recommends ReptiSun 5.0 or Arcadia 6%. Needs an owner call on the wording. Price unchanged.</t>
         </is>
       </c>
     </row>
@@ -10284,7 +10284,7 @@
       </c>
       <c r="I203" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: setup FAQ and body now call uromastyx near-strict herbivores with seeds a limited extra, matching the feeding guide.</t>
+          <t>2026-10-05: setup FAQ and body now call uromastyx near-strict herbivores with seeds a limited extra, matching the feeding guide. Fable follow-up: overview and handling guide now also say near-strict, the hub seed line drops its stale parenthetical, and setup line 102 grammar fixed.</t>
         </is>
       </c>
     </row>
@@ -11070,7 +11070,7 @@
       </c>
       <c r="I229" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: kingsnake hub power outage row now says 68 to 72F night low, matching the setup and health guides.</t>
+          <t>2026-10-05: kingsnake hub power outage row now says 68 to 72F night low, matching the setup and health guides. Fable follow-up: reptile emergency plan table now gives the kingsnake its own row, 68 to 72F, act below 68F.</t>
         </is>
       </c>
     </row>
@@ -12664,7 +12664,7 @@
       </c>
       <c r="I275" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: milk snake hub power outage row now says 70 to 75F night low, heat below 70F, matching the setup guide.</t>
+          <t>2026-10-05: milk snake hub power outage row now says 70 to 75F night low, heat below 70F, matching the setup guide. Fable follow-up: reptile emergency plan table now says 70 to 75F, act below 70F.</t>
         </is>
       </c>
     </row>
@@ -13637,7 +13637,7 @@
       </c>
       <c r="I306" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: comparison now says 5 to 9 inches in both places.</t>
+          <t>2026-10-05: comparison now says 5 to 9 inches in both places. Fable follow-up: red-footed tortoise cost guide line 99 also said 5 to 10 inches; now 5 to 9.</t>
         </is>
       </c>
     </row>
@@ -14089,7 +14089,7 @@
       </c>
       <c r="I318" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: overview now says captive individuals commonly live 50 years or more, some reported past 90, matching the cost guide and encyclopedia.</t>
+          <t>2026-10-05: overview now says captive individuals commonly live 50 years or more, some reported past 90, matching the cost guide and encyclopedia. Fable follow-up: reworded to 50 to 70 years or more, some reported near 90, matching the hub FAQ.</t>
         </is>
       </c>
     </row>
@@ -14543,7 +14543,7 @@
       </c>
       <c r="I332" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: cost guide now scales from the 5.5 by 3 foot eastern box turtle size, matching the setup guide. Prices unchanged.</t>
+          <t>2026-10-05: cost guide now scales from the 5.5 by 3 foot eastern box turtle size, matching the setup guide. Prices unchanged. Fable follow-up: 5.5 by 3 ft is about 3.7 times a 36x18 inch floor, so the line now says nearly four times.</t>
         </is>
       </c>
     </row>
@@ -14866,7 +14866,7 @@
       </c>
       <c r="I341" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: brumation FAQ, hub and health guide now act at about 7 percent, before the 10 percent stop line, matching the guide's own line 122.</t>
+          <t>2026-10-05: brumation FAQ, hub and health guide now act at about 7 percent, before the 10 percent stop line, matching the guide's own line 122. Fable follow-up: tortoise brumation guide table row also now acts at about 7 percent, stop by 10.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Price redo: ackie monitor, setup $985 to $2,355 everywhere
Every item priced and linked under the package rules; UVB is the 36 in kit;
the 48x24x48 enclosure is unlinked because it is under the 5x2.5x4 minimum.
Hub, route line and the ackie overview now match the cost guide.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CONSISTENCY_CHECK.xlsx
+++ b/CONSISTENCY_CHECK.xlsx
@@ -8794,7 +8794,7 @@
       </c>
       <c r="D160" s="15" t="inlineStr">
         <is>
-          <t>✗</t>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E160" s="13" t="inlineStr">
@@ -8819,7 +8819,7 @@
       </c>
       <c r="I160" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: prices are never changed (owner). Note only: hub route line says $800 to $1,500; the cost guide says $850 to $2,150 or more.</t>
+          <t>2026-10-05: prices are never changed (owner). Note only: hub route line says $800 to $1,500; the cost guide says $850 to $2,150 or more. 2026-10-06 price redo: hub route line and overview now say $985 to $2,355, the cost guide setup total.</t>
         </is>
       </c>
     </row>
@@ -9097,7 +9097,7 @@
       </c>
       <c r="D169" s="15" t="inlineStr">
         <is>
-          <t>✗</t>
+          <t>✓ Fixed</t>
         </is>
       </c>
       <c r="E169" s="13" t="inlineStr">
@@ -9122,7 +9122,7 @@
       </c>
       <c r="I169" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: prices are never changed (owner). Note only: overview says an $800 to $1,500 setup; the cost guide says $850 to $2,150 or more.</t>
+          <t>2026-10-05: prices are never changed (owner). Note only: overview says an $800 to $1,500 setup; the cost guide says $850 to $2,150 or more. 2026-10-06 price redo: hub route line and overview now say $985 to $2,355, the cost guide setup total.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Price redo: ackie table keeps must-haves only, setup $890 to $2,230
Owner rule: the cost table prices what the animal's wellbeing needs; the
daylight LED, puzzle feeder and clicker stay hub links with no cost row.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CONSISTENCY_CHECK.xlsx
+++ b/CONSISTENCY_CHECK.xlsx
@@ -8819,7 +8819,7 @@
       </c>
       <c r="I160" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: prices are never changed (owner). Note only: hub route line says $800 to $1,500; the cost guide says $850 to $2,150 or more. 2026-10-06 price redo: hub route line and overview now say $985 to $2,355, the cost guide setup total.</t>
+          <t>2026-10-05: prices are never changed (owner). Note only: hub route line says $800 to $1,500; the cost guide says $850 to $2,150 or more. 2026-10-06 price redo: hub route line and overview now say $890 to $2,230, the cost guide setup total.</t>
         </is>
       </c>
     </row>
@@ -9122,7 +9122,7 @@
       </c>
       <c r="I169" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: prices are never changed (owner). Note only: overview says an $800 to $1,500 setup; the cost guide says $850 to $2,150 or more. 2026-10-06 price redo: hub route line and overview now say $985 to $2,355, the cost guide setup total.</t>
+          <t>2026-10-05: prices are never changed (owner). Note only: overview says an $800 to $1,500 setup; the cost guide says $850 to $2,150 or more. 2026-10-06 price redo: hub route line and overview now say $890 to $2,230, the cost guide setup total.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Price redo: ackie fixes from the Fable check, setup $880 to $2,230
Basking and substrate rows unlinked (no catalog match for two 100 W PAR30
floods; the bioactive bag mix is far over the row at 12 to 24 inches),
infrared gun and supplement floors cover the catalog prices, the
below-spec enclosure loses its ackie covers string, catalog prices added
for the LED and slate, "an $880" in the overview.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CONSISTENCY_CHECK.xlsx
+++ b/CONSISTENCY_CHECK.xlsx
@@ -652,6 +652,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3628,6 +3629,7 @@
         <v>271</v>
       </c>
     </row>
+    <row r="114"/>
     <row r="115">
       <c r="A115" s="9" t="inlineStr">
         <is>
@@ -8819,7 +8821,7 @@
       </c>
       <c r="I160" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: prices are never changed (owner). Note only: hub route line says $800 to $1,500; the cost guide says $850 to $2,150 or more. 2026-10-06 price redo: hub route line and overview now say $890 to $2,230, the cost guide setup total.</t>
+          <t>2026-10-05: prices are never changed (owner). Note only: hub route line says $800 to $1,500; the cost guide says $850 to $2,150 or more. 2026-10-06 price redo: hub route line and overview now say $880 to $2,230, the cost guide setup total.</t>
         </is>
       </c>
     </row>
@@ -9122,7 +9124,7 @@
       </c>
       <c r="I169" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: prices are never changed (owner). Note only: overview says an $800 to $1,500 setup; the cost guide says $850 to $2,150 or more. 2026-10-06 price redo: hub route line and overview now say $890 to $2,230, the cost guide setup total.</t>
+          <t>2026-10-05: prices are never changed (owner). Note only: overview says an $800 to $1,500 setup; the cost guide says $850 to $2,150 or more. 2026-10-06 price redo: hub route line and overview now say $880 to $2,230, the cost guide setup total.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ackie: basking bulbs and dome lamps priced as separate rows, setup $900 to $2,245
The owner's 100 W 2 pack at $11.99 (rounded to $10 - $15) and two dome
lamps rated to 150 W ($25 to $40 each). Every total, title, FAQ and hub
line moved with the shared price list.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CONSISTENCY_CHECK.xlsx
+++ b/CONSISTENCY_CHECK.xlsx
@@ -8821,7 +8821,7 @@
       </c>
       <c r="I160" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: prices are never changed (owner). Note only: hub route line says $800 to $1,500; the cost guide says $850 to $2,150 or more. 2026-10-06 price redo: hub route line and overview now say $880 to $2,230, the cost guide setup total.</t>
+          <t>2026-10-05: prices are never changed (owner). Note only: hub route line says $800 to $1,500; the cost guide says $850 to $2,150 or more. 2026-10-06 price redo: hub route line and overview now say $900 to $2,245, the cost guide setup total.</t>
         </is>
       </c>
     </row>
@@ -9124,7 +9124,7 @@
       </c>
       <c r="I169" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: prices are never changed (owner). Note only: overview says an $800 to $1,500 setup; the cost guide says $850 to $2,150 or more. 2026-10-06 price redo: hub route line and overview now say $880 to $2,230, the cost guide setup total.</t>
+          <t>2026-10-05: prices are never changed (owner). Note only: overview says an $800 to $1,500 setup; the cost guide says $850 to $2,150 or more. 2026-10-06 price redo: hub route line and overview now say $900 to $2,245, the cost guide setup total.</t>
         </is>
       </c>
     </row>

</xml_diff>